<commit_message>
Catalogo de venta por categoria con imagenes y precios detal/mayor (PDF)
</commit_message>
<xml_diff>
--- a/generator/Sistema_Gestion_Inventario.xlsx
+++ b/generator/Sistema_Gestion_Inventario.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Inventario" sheetId="7" r:id="rId7"/>
     <sheet name="Clientes" sheetId="8" r:id="rId8"/>
     <sheet name="Factura" sheetId="9" r:id="rId9"/>
-    <sheet name="Config" sheetId="10" r:id="rId10"/>
+    <sheet name="Catálogo Venta" sheetId="10" r:id="rId10"/>
+    <sheet name="Config" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="168" formatCode="+#,##0;\-#,##0;0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color rgb="FF2C3E50"/>
@@ -106,6 +107,24 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF1F3A5F"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F3A5F"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF16A085"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -198,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -314,6 +333,21 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3001,6 +3035,928 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D65"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.00" customWidth="1"/>
+    <col min="2" max="2" width="30.00" customWidth="1"/>
+    <col min="3" max="3" width="30.00" customWidth="1"/>
+    <col min="4" max="4" width="20.00" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="44.00" customHeight="1">
+      <c r="A1" s="43">
+        <f>'Config'!$B$2</f>
+      </c>
+    </row>
+    <row r="2" ht="24.00" customHeight="1">
+      <c r="A2" s="6">
+        <f>"Catálogo de productos · "&amp;$B$3&amp;" · Precio "&amp;$D$3</f>
+      </c>
+    </row>
+    <row r="3" ht="22.00" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Categoría:</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrónica</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipo de precio:</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24.00" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imagen</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Producto</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descripción / Código</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90.00" customHeight="1">
+      <c r="A6" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B6" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C6" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D6" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;1,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="7" ht="90.00" customHeight="1">
+      <c r="A7" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B7" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C7" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D7" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;2,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="8" ht="90.00" customHeight="1">
+      <c r="A8" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B8" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C8" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D8" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;3,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="9" ht="90.00" customHeight="1">
+      <c r="A9" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B9" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C9" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D9" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;4,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="10" ht="90.00" customHeight="1">
+      <c r="A10" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B10" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C10" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D10" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;5,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="11" ht="90.00" customHeight="1">
+      <c r="A11" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B11" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C11" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D11" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;6,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="12" ht="90.00" customHeight="1">
+      <c r="A12" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B12" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C12" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D12" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;7,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="13" ht="90.00" customHeight="1">
+      <c r="A13" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B13" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C13" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D13" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;8,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="14" ht="90.00" customHeight="1">
+      <c r="A14" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B14" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C14" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D14" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;9,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="15" ht="90.00" customHeight="1">
+      <c r="A15" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B15" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C15" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D15" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;10,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="16" ht="90.00" customHeight="1">
+      <c r="A16" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B16" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C16" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D16" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;11,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="17" ht="90.00" customHeight="1">
+      <c r="A17" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B17" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C17" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D17" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;12,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="18" ht="90.00" customHeight="1">
+      <c r="A18" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B18" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C18" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D18" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;13,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="19" ht="90.00" customHeight="1">
+      <c r="A19" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B19" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C19" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D19" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;14,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="20" ht="90.00" customHeight="1">
+      <c r="A20" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B20" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C20" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D20" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;15,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="21" ht="90.00" customHeight="1">
+      <c r="A21" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B21" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C21" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D21" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;16,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="22" ht="90.00" customHeight="1">
+      <c r="A22" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B22" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C22" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D22" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;17,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="23" ht="90.00" customHeight="1">
+      <c r="A23" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B23" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C23" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D23" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;18,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="24" ht="90.00" customHeight="1">
+      <c r="A24" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B24" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C24" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D24" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;19,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="25" ht="90.00" customHeight="1">
+      <c r="A25" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B25" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C25" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D25" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;20,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="26" ht="90.00" customHeight="1">
+      <c r="A26" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B26" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C26" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D26" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;21,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="27" ht="90.00" customHeight="1">
+      <c r="A27" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B27" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C27" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D27" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;22,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="28" ht="90.00" customHeight="1">
+      <c r="A28" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B28" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C28" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D28" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;23,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="29" ht="90.00" customHeight="1">
+      <c r="A29" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B29" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C29" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D29" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;24,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="30" ht="90.00" customHeight="1">
+      <c r="A30" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B30" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C30" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D30" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;25,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="31" ht="90.00" customHeight="1">
+      <c r="A31" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B31" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C31" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D31" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;26,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="32" ht="90.00" customHeight="1">
+      <c r="A32" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B32" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C32" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D32" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;27,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="33" ht="90.00" customHeight="1">
+      <c r="A33" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B33" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C33" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D33" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;28,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="34" ht="90.00" customHeight="1">
+      <c r="A34" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B34" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C34" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D34" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;29,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="35" ht="90.00" customHeight="1">
+      <c r="A35" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B35" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C35" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D35" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;30,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="36" ht="90.00" customHeight="1">
+      <c r="A36" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B36" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C36" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D36" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;31,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="37" ht="90.00" customHeight="1">
+      <c r="A37" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B37" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C37" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D37" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;32,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="38" ht="90.00" customHeight="1">
+      <c r="A38" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B38" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C38" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D38" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;33,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="39" ht="90.00" customHeight="1">
+      <c r="A39" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B39" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C39" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D39" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;34,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="40" ht="90.00" customHeight="1">
+      <c r="A40" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B40" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C40" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D40" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;35,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="41" ht="90.00" customHeight="1">
+      <c r="A41" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B41" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C41" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D41" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;36,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="42" ht="90.00" customHeight="1">
+      <c r="A42" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B42" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C42" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D42" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;37,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="43" ht="90.00" customHeight="1">
+      <c r="A43" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B43" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C43" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D43" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;38,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="44" ht="90.00" customHeight="1">
+      <c r="A44" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B44" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C44" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D44" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;39,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="45" ht="90.00" customHeight="1">
+      <c r="A45" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B45" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C45" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D45" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;40,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="46" ht="90.00" customHeight="1">
+      <c r="A46" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B46" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C46" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D46" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;41,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="47" ht="90.00" customHeight="1">
+      <c r="A47" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B47" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C47" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D47" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;42,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="48" ht="90.00" customHeight="1">
+      <c r="A48" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B48" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C48" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D48" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;43,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="49" ht="90.00" customHeight="1">
+      <c r="A49" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B49" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C49" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D49" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;44,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="50" ht="90.00" customHeight="1">
+      <c r="A50" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B50" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C50" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D50" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;45,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="51" ht="90.00" customHeight="1">
+      <c r="A51" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B51" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C51" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D51" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;46,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="52" ht="90.00" customHeight="1">
+      <c r="A52" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B52" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C52" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D52" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;47,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="53" ht="90.00" customHeight="1">
+      <c r="A53" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B53" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C53" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D53" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;48,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="54" ht="90.00" customHeight="1">
+      <c r="A54" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B54" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C54" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D54" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;49,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="55" ht="90.00" customHeight="1">
+      <c r="A55" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B55" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C55" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D55" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;50,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="56" ht="90.00" customHeight="1">
+      <c r="A56" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B56" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C56" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D56" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;51,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="57" ht="90.00" customHeight="1">
+      <c r="A57" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B57" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C57" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D57" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;52,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="58" ht="90.00" customHeight="1">
+      <c r="A58" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B58" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C58" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D58" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;53,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="59" ht="90.00" customHeight="1">
+      <c r="A59" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B59" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C59" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D59" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;54,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="60" ht="90.00" customHeight="1">
+      <c r="A60" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B60" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C60" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D60" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;55,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="61" ht="90.00" customHeight="1">
+      <c r="A61" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B61" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C61" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D61" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;56,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="62" ht="90.00" customHeight="1">
+      <c r="A62" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B62" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C62" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D62" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;57,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="63" ht="90.00" customHeight="1">
+      <c r="A63" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B63" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C63" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D63" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;58,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="64" ht="90.00" customHeight="1">
+      <c r="A64" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B64" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C64" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D64" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;59,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+    <row r="65" ht="90.00" customHeight="1">
+      <c r="A65" s="39">
+        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0)),1)),"")</f>
+      </c>
+      <c r="B65" s="40">
+        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="C65" s="41">
+        <f>IFERROR("Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0)),"")</f>
+      </c>
+      <c r="D65" s="42">
+        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;60,'Catálogo'!$Q:$Q,0))),"")</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="B3:B3">
+      <formula1>'Config'!$D$2:$D$8</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="D3:D3">
+      <formula1>"Detal,Mayor"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3250,7 +4206,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L201"/>
+  <dimension ref="A1:Q201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.00" customWidth="1"/>
@@ -3265,6 +4221,11 @@
     <col min="10" max="10" width="16.00" customWidth="1"/>
     <col min="11" max="11" width="14.00" customWidth="1"/>
     <col min="12" max="12" width="8.00" customWidth="1"/>
+    <col min="13" max="13" width="36.00" customWidth="1"/>
+    <col min="14" max="14" width="14.00" customWidth="1"/>
+    <col min="15" max="15" width="14.00" customWidth="1"/>
+    <col min="16" max="16" width="8.00" customWidth="1" hidden="1"/>
+    <col min="17" max="17" width="8.00" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3328,6 +4289,31 @@
           <t xml:space="preserve">IVA %</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">URL Imagen</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precio Detal</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precio Mayor</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_rank</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_key</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
@@ -3374,6 +4360,23 @@
       <c r="L2" s="17">
         <f>IF($A2="","",IFERROR(VLOOKUP($C2,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N2" s="22">
+        <v>75000</v>
+      </c>
+      <c r="O2" s="22">
+        <v>60000</v>
+      </c>
+      <c r="P2" s="17">
+        <f>IF(OR($A2="",$D2&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C2,$C2,$D$2:$D2,"Activo"))</f>
+      </c>
+      <c r="Q2" s="19">
+        <f>IF($P2="","",$C2&amp;"|"&amp;$P2)</f>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -3420,6 +4423,23 @@
       <c r="L3" s="17">
         <f>IF($A3="","",IFERROR(VLOOKUP($C3,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N3" s="22">
+        <v>28000</v>
+      </c>
+      <c r="O3" s="22">
+        <v>22000</v>
+      </c>
+      <c r="P3" s="17">
+        <f>IF(OR($A3="",$D3&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C3,$C3,$D$2:$D3,"Activo"))</f>
+      </c>
+      <c r="Q3" s="19">
+        <f>IF($P3="","",$C3&amp;"|"&amp;$P3)</f>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
@@ -3466,6 +4486,23 @@
       <c r="L4" s="17">
         <f>IF($A4="","",IFERROR(VLOOKUP($C4,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N4" s="22">
+        <v>25000</v>
+      </c>
+      <c r="O4" s="22">
+        <v>18000</v>
+      </c>
+      <c r="P4" s="17">
+        <f>IF(OR($A4="",$D4&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C4,$C4,$D$2:$D4,"Activo"))</f>
+      </c>
+      <c r="Q4" s="19">
+        <f>IF($P4="","",$C4&amp;"|"&amp;$P4)</f>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -3512,6 +4549,23 @@
       <c r="L5" s="17">
         <f>IF($A5="","",IFERROR(VLOOKUP($C5,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N5" s="22">
+        <v>45000</v>
+      </c>
+      <c r="O5" s="22">
+        <v>36000</v>
+      </c>
+      <c r="P5" s="17">
+        <f>IF(OR($A5="",$D5&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C5,$C5,$D$2:$D5,"Activo"))</f>
+      </c>
+      <c r="Q5" s="19">
+        <f>IF($P5="","",$C5&amp;"|"&amp;$P5)</f>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -3558,6 +4612,23 @@
       <c r="L6" s="17">
         <f>IF($A6="","",IFERROR(VLOOKUP($C6,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N6" s="22">
+        <v>12000</v>
+      </c>
+      <c r="O6" s="22">
+        <v>8000</v>
+      </c>
+      <c r="P6" s="17">
+        <f>IF(OR($A6="",$D6&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C6,$C6,$D$2:$D6,"Activo"))</f>
+      </c>
+      <c r="Q6" s="19">
+        <f>IF($P6="","",$C6&amp;"|"&amp;$P6)</f>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
@@ -3603,6 +4674,23 @@
       </c>
       <c r="L7" s="17">
         <f>IF($A7="","",IFERROR(VLOOKUP($C7,'Config'!$D$2:$E$8,2,FALSE),0))</f>
+      </c>
+      <c r="M7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N7" s="22">
+        <v>38000</v>
+      </c>
+      <c r="O7" s="22">
+        <v>30000</v>
+      </c>
+      <c r="P7" s="17">
+        <f>IF(OR($A7="",$D7&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C7,$C7,$D$2:$D7,"Activo"))</f>
+      </c>
+      <c r="Q7" s="19">
+        <f>IF($P7="","",$C7&amp;"|"&amp;$P7)</f>
       </c>
     </row>
     <row r="8">
@@ -3632,6 +4720,15 @@
       <c r="L8" s="17">
         <f>IF($A8="","",IFERROR(VLOOKUP($C8,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M8" s="20"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="17">
+        <f>IF(OR($A8="",$D8&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C8,$C8,$D$2:$D8,"Activo"))</f>
+      </c>
+      <c r="Q8" s="19">
+        <f>IF($P8="","",$C8&amp;"|"&amp;$P8)</f>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20"/>
@@ -3660,6 +4757,15 @@
       <c r="L9" s="17">
         <f>IF($A9="","",IFERROR(VLOOKUP($C9,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M9" s="20"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="17">
+        <f>IF(OR($A9="",$D9&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C9,$C9,$D$2:$D9,"Activo"))</f>
+      </c>
+      <c r="Q9" s="19">
+        <f>IF($P9="","",$C9&amp;"|"&amp;$P9)</f>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20"/>
@@ -3688,6 +4794,15 @@
       <c r="L10" s="17">
         <f>IF($A10="","",IFERROR(VLOOKUP($C10,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M10" s="20"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="17">
+        <f>IF(OR($A10="",$D10&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C10,$C10,$D$2:$D10,"Activo"))</f>
+      </c>
+      <c r="Q10" s="19">
+        <f>IF($P10="","",$C10&amp;"|"&amp;$P10)</f>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20"/>
@@ -3716,6 +4831,15 @@
       <c r="L11" s="17">
         <f>IF($A11="","",IFERROR(VLOOKUP($C11,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M11" s="20"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="17">
+        <f>IF(OR($A11="",$D11&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C11,$C11,$D$2:$D11,"Activo"))</f>
+      </c>
+      <c r="Q11" s="19">
+        <f>IF($P11="","",$C11&amp;"|"&amp;$P11)</f>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20"/>
@@ -3744,6 +4868,15 @@
       <c r="L12" s="17">
         <f>IF($A12="","",IFERROR(VLOOKUP($C12,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M12" s="20"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="17">
+        <f>IF(OR($A12="",$D12&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C12,$C12,$D$2:$D12,"Activo"))</f>
+      </c>
+      <c r="Q12" s="19">
+        <f>IF($P12="","",$C12&amp;"|"&amp;$P12)</f>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20"/>
@@ -3772,6 +4905,15 @@
       <c r="L13" s="17">
         <f>IF($A13="","",IFERROR(VLOOKUP($C13,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M13" s="20"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="17">
+        <f>IF(OR($A13="",$D13&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C13,$C13,$D$2:$D13,"Activo"))</f>
+      </c>
+      <c r="Q13" s="19">
+        <f>IF($P13="","",$C13&amp;"|"&amp;$P13)</f>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20"/>
@@ -3800,6 +4942,15 @@
       <c r="L14" s="17">
         <f>IF($A14="","",IFERROR(VLOOKUP($C14,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M14" s="20"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="17">
+        <f>IF(OR($A14="",$D14&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C14,$C14,$D$2:$D14,"Activo"))</f>
+      </c>
+      <c r="Q14" s="19">
+        <f>IF($P14="","",$C14&amp;"|"&amp;$P14)</f>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20"/>
@@ -3828,6 +4979,15 @@
       <c r="L15" s="17">
         <f>IF($A15="","",IFERROR(VLOOKUP($C15,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M15" s="20"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="17">
+        <f>IF(OR($A15="",$D15&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C15,$C15,$D$2:$D15,"Activo"))</f>
+      </c>
+      <c r="Q15" s="19">
+        <f>IF($P15="","",$C15&amp;"|"&amp;$P15)</f>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20"/>
@@ -3856,6 +5016,15 @@
       <c r="L16" s="17">
         <f>IF($A16="","",IFERROR(VLOOKUP($C16,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M16" s="20"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="17">
+        <f>IF(OR($A16="",$D16&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C16,$C16,$D$2:$D16,"Activo"))</f>
+      </c>
+      <c r="Q16" s="19">
+        <f>IF($P16="","",$C16&amp;"|"&amp;$P16)</f>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20"/>
@@ -3884,6 +5053,15 @@
       <c r="L17" s="17">
         <f>IF($A17="","",IFERROR(VLOOKUP($C17,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M17" s="20"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="17">
+        <f>IF(OR($A17="",$D17&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C17,$C17,$D$2:$D17,"Activo"))</f>
+      </c>
+      <c r="Q17" s="19">
+        <f>IF($P17="","",$C17&amp;"|"&amp;$P17)</f>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20"/>
@@ -3912,6 +5090,15 @@
       <c r="L18" s="17">
         <f>IF($A18="","",IFERROR(VLOOKUP($C18,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M18" s="20"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="17">
+        <f>IF(OR($A18="",$D18&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C18,$C18,$D$2:$D18,"Activo"))</f>
+      </c>
+      <c r="Q18" s="19">
+        <f>IF($P18="","",$C18&amp;"|"&amp;$P18)</f>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20"/>
@@ -3940,6 +5127,15 @@
       <c r="L19" s="17">
         <f>IF($A19="","",IFERROR(VLOOKUP($C19,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M19" s="20"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="17">
+        <f>IF(OR($A19="",$D19&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C19,$C19,$D$2:$D19,"Activo"))</f>
+      </c>
+      <c r="Q19" s="19">
+        <f>IF($P19="","",$C19&amp;"|"&amp;$P19)</f>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20"/>
@@ -3968,6 +5164,15 @@
       <c r="L20" s="17">
         <f>IF($A20="","",IFERROR(VLOOKUP($C20,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M20" s="20"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="17">
+        <f>IF(OR($A20="",$D20&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C20,$C20,$D$2:$D20,"Activo"))</f>
+      </c>
+      <c r="Q20" s="19">
+        <f>IF($P20="","",$C20&amp;"|"&amp;$P20)</f>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20"/>
@@ -3996,6 +5201,15 @@
       <c r="L21" s="17">
         <f>IF($A21="","",IFERROR(VLOOKUP($C21,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M21" s="20"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
+      <c r="P21" s="17">
+        <f>IF(OR($A21="",$D21&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C21,$C21,$D$2:$D21,"Activo"))</f>
+      </c>
+      <c r="Q21" s="19">
+        <f>IF($P21="","",$C21&amp;"|"&amp;$P21)</f>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20"/>
@@ -4024,6 +5238,15 @@
       <c r="L22" s="17">
         <f>IF($A22="","",IFERROR(VLOOKUP($C22,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M22" s="20"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="17">
+        <f>IF(OR($A22="",$D22&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C22,$C22,$D$2:$D22,"Activo"))</f>
+      </c>
+      <c r="Q22" s="19">
+        <f>IF($P22="","",$C22&amp;"|"&amp;$P22)</f>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20"/>
@@ -4052,6 +5275,15 @@
       <c r="L23" s="17">
         <f>IF($A23="","",IFERROR(VLOOKUP($C23,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M23" s="20"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="17">
+        <f>IF(OR($A23="",$D23&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C23,$C23,$D$2:$D23,"Activo"))</f>
+      </c>
+      <c r="Q23" s="19">
+        <f>IF($P23="","",$C23&amp;"|"&amp;$P23)</f>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="20"/>
@@ -4080,6 +5312,15 @@
       <c r="L24" s="17">
         <f>IF($A24="","",IFERROR(VLOOKUP($C24,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M24" s="20"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="17">
+        <f>IF(OR($A24="",$D24&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C24,$C24,$D$2:$D24,"Activo"))</f>
+      </c>
+      <c r="Q24" s="19">
+        <f>IF($P24="","",$C24&amp;"|"&amp;$P24)</f>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="20"/>
@@ -4108,6 +5349,15 @@
       <c r="L25" s="17">
         <f>IF($A25="","",IFERROR(VLOOKUP($C25,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M25" s="20"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="17">
+        <f>IF(OR($A25="",$D25&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C25,$C25,$D$2:$D25,"Activo"))</f>
+      </c>
+      <c r="Q25" s="19">
+        <f>IF($P25="","",$C25&amp;"|"&amp;$P25)</f>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="20"/>
@@ -4136,6 +5386,15 @@
       <c r="L26" s="17">
         <f>IF($A26="","",IFERROR(VLOOKUP($C26,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M26" s="20"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="17">
+        <f>IF(OR($A26="",$D26&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C26,$C26,$D$2:$D26,"Activo"))</f>
+      </c>
+      <c r="Q26" s="19">
+        <f>IF($P26="","",$C26&amp;"|"&amp;$P26)</f>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="20"/>
@@ -4164,6 +5423,15 @@
       <c r="L27" s="17">
         <f>IF($A27="","",IFERROR(VLOOKUP($C27,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M27" s="20"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="17">
+        <f>IF(OR($A27="",$D27&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C27,$C27,$D$2:$D27,"Activo"))</f>
+      </c>
+      <c r="Q27" s="19">
+        <f>IF($P27="","",$C27&amp;"|"&amp;$P27)</f>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="20"/>
@@ -4192,6 +5460,15 @@
       <c r="L28" s="17">
         <f>IF($A28="","",IFERROR(VLOOKUP($C28,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M28" s="20"/>
+      <c r="N28" s="22"/>
+      <c r="O28" s="22"/>
+      <c r="P28" s="17">
+        <f>IF(OR($A28="",$D28&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C28,$C28,$D$2:$D28,"Activo"))</f>
+      </c>
+      <c r="Q28" s="19">
+        <f>IF($P28="","",$C28&amp;"|"&amp;$P28)</f>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="20"/>
@@ -4220,6 +5497,15 @@
       <c r="L29" s="17">
         <f>IF($A29="","",IFERROR(VLOOKUP($C29,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M29" s="20"/>
+      <c r="N29" s="22"/>
+      <c r="O29" s="22"/>
+      <c r="P29" s="17">
+        <f>IF(OR($A29="",$D29&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C29,$C29,$D$2:$D29,"Activo"))</f>
+      </c>
+      <c r="Q29" s="19">
+        <f>IF($P29="","",$C29&amp;"|"&amp;$P29)</f>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="20"/>
@@ -4248,6 +5534,15 @@
       <c r="L30" s="17">
         <f>IF($A30="","",IFERROR(VLOOKUP($C30,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M30" s="20"/>
+      <c r="N30" s="22"/>
+      <c r="O30" s="22"/>
+      <c r="P30" s="17">
+        <f>IF(OR($A30="",$D30&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C30,$C30,$D$2:$D30,"Activo"))</f>
+      </c>
+      <c r="Q30" s="19">
+        <f>IF($P30="","",$C30&amp;"|"&amp;$P30)</f>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="20"/>
@@ -4276,6 +5571,15 @@
       <c r="L31" s="17">
         <f>IF($A31="","",IFERROR(VLOOKUP($C31,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M31" s="20"/>
+      <c r="N31" s="22"/>
+      <c r="O31" s="22"/>
+      <c r="P31" s="17">
+        <f>IF(OR($A31="",$D31&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C31,$C31,$D$2:$D31,"Activo"))</f>
+      </c>
+      <c r="Q31" s="19">
+        <f>IF($P31="","",$C31&amp;"|"&amp;$P31)</f>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="20"/>
@@ -4304,6 +5608,15 @@
       <c r="L32" s="17">
         <f>IF($A32="","",IFERROR(VLOOKUP($C32,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M32" s="20"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
+      <c r="P32" s="17">
+        <f>IF(OR($A32="",$D32&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C32,$C32,$D$2:$D32,"Activo"))</f>
+      </c>
+      <c r="Q32" s="19">
+        <f>IF($P32="","",$C32&amp;"|"&amp;$P32)</f>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="20"/>
@@ -4332,6 +5645,15 @@
       <c r="L33" s="17">
         <f>IF($A33="","",IFERROR(VLOOKUP($C33,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M33" s="20"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="22"/>
+      <c r="P33" s="17">
+        <f>IF(OR($A33="",$D33&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C33,$C33,$D$2:$D33,"Activo"))</f>
+      </c>
+      <c r="Q33" s="19">
+        <f>IF($P33="","",$C33&amp;"|"&amp;$P33)</f>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="20"/>
@@ -4360,6 +5682,15 @@
       <c r="L34" s="17">
         <f>IF($A34="","",IFERROR(VLOOKUP($C34,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M34" s="20"/>
+      <c r="N34" s="22"/>
+      <c r="O34" s="22"/>
+      <c r="P34" s="17">
+        <f>IF(OR($A34="",$D34&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C34,$C34,$D$2:$D34,"Activo"))</f>
+      </c>
+      <c r="Q34" s="19">
+        <f>IF($P34="","",$C34&amp;"|"&amp;$P34)</f>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="20"/>
@@ -4388,6 +5719,15 @@
       <c r="L35" s="17">
         <f>IF($A35="","",IFERROR(VLOOKUP($C35,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M35" s="20"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
+      <c r="P35" s="17">
+        <f>IF(OR($A35="",$D35&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C35,$C35,$D$2:$D35,"Activo"))</f>
+      </c>
+      <c r="Q35" s="19">
+        <f>IF($P35="","",$C35&amp;"|"&amp;$P35)</f>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="20"/>
@@ -4416,6 +5756,15 @@
       <c r="L36" s="17">
         <f>IF($A36="","",IFERROR(VLOOKUP($C36,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M36" s="20"/>
+      <c r="N36" s="22"/>
+      <c r="O36" s="22"/>
+      <c r="P36" s="17">
+        <f>IF(OR($A36="",$D36&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C36,$C36,$D$2:$D36,"Activo"))</f>
+      </c>
+      <c r="Q36" s="19">
+        <f>IF($P36="","",$C36&amp;"|"&amp;$P36)</f>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="20"/>
@@ -4444,6 +5793,15 @@
       <c r="L37" s="17">
         <f>IF($A37="","",IFERROR(VLOOKUP($C37,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M37" s="20"/>
+      <c r="N37" s="22"/>
+      <c r="O37" s="22"/>
+      <c r="P37" s="17">
+        <f>IF(OR($A37="",$D37&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C37,$C37,$D$2:$D37,"Activo"))</f>
+      </c>
+      <c r="Q37" s="19">
+        <f>IF($P37="","",$C37&amp;"|"&amp;$P37)</f>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="20"/>
@@ -4472,6 +5830,15 @@
       <c r="L38" s="17">
         <f>IF($A38="","",IFERROR(VLOOKUP($C38,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M38" s="20"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="22"/>
+      <c r="P38" s="17">
+        <f>IF(OR($A38="",$D38&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C38,$C38,$D$2:$D38,"Activo"))</f>
+      </c>
+      <c r="Q38" s="19">
+        <f>IF($P38="","",$C38&amp;"|"&amp;$P38)</f>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="20"/>
@@ -4500,6 +5867,15 @@
       <c r="L39" s="17">
         <f>IF($A39="","",IFERROR(VLOOKUP($C39,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M39" s="20"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="17">
+        <f>IF(OR($A39="",$D39&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C39,$C39,$D$2:$D39,"Activo"))</f>
+      </c>
+      <c r="Q39" s="19">
+        <f>IF($P39="","",$C39&amp;"|"&amp;$P39)</f>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="20"/>
@@ -4528,6 +5904,15 @@
       <c r="L40" s="17">
         <f>IF($A40="","",IFERROR(VLOOKUP($C40,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M40" s="20"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="22"/>
+      <c r="P40" s="17">
+        <f>IF(OR($A40="",$D40&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C40,$C40,$D$2:$D40,"Activo"))</f>
+      </c>
+      <c r="Q40" s="19">
+        <f>IF($P40="","",$C40&amp;"|"&amp;$P40)</f>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="20"/>
@@ -4556,6 +5941,15 @@
       <c r="L41" s="17">
         <f>IF($A41="","",IFERROR(VLOOKUP($C41,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M41" s="20"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
+      <c r="P41" s="17">
+        <f>IF(OR($A41="",$D41&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C41,$C41,$D$2:$D41,"Activo"))</f>
+      </c>
+      <c r="Q41" s="19">
+        <f>IF($P41="","",$C41&amp;"|"&amp;$P41)</f>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="20"/>
@@ -4584,6 +5978,15 @@
       <c r="L42" s="17">
         <f>IF($A42="","",IFERROR(VLOOKUP($C42,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M42" s="20"/>
+      <c r="N42" s="22"/>
+      <c r="O42" s="22"/>
+      <c r="P42" s="17">
+        <f>IF(OR($A42="",$D42&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C42,$C42,$D$2:$D42,"Activo"))</f>
+      </c>
+      <c r="Q42" s="19">
+        <f>IF($P42="","",$C42&amp;"|"&amp;$P42)</f>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="20"/>
@@ -4612,6 +6015,15 @@
       <c r="L43" s="17">
         <f>IF($A43="","",IFERROR(VLOOKUP($C43,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M43" s="20"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
+      <c r="P43" s="17">
+        <f>IF(OR($A43="",$D43&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C43,$C43,$D$2:$D43,"Activo"))</f>
+      </c>
+      <c r="Q43" s="19">
+        <f>IF($P43="","",$C43&amp;"|"&amp;$P43)</f>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="20"/>
@@ -4640,6 +6052,15 @@
       <c r="L44" s="17">
         <f>IF($A44="","",IFERROR(VLOOKUP($C44,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M44" s="20"/>
+      <c r="N44" s="22"/>
+      <c r="O44" s="22"/>
+      <c r="P44" s="17">
+        <f>IF(OR($A44="",$D44&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C44,$C44,$D$2:$D44,"Activo"))</f>
+      </c>
+      <c r="Q44" s="19">
+        <f>IF($P44="","",$C44&amp;"|"&amp;$P44)</f>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="20"/>
@@ -4668,6 +6089,15 @@
       <c r="L45" s="17">
         <f>IF($A45="","",IFERROR(VLOOKUP($C45,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M45" s="20"/>
+      <c r="N45" s="22"/>
+      <c r="O45" s="22"/>
+      <c r="P45" s="17">
+        <f>IF(OR($A45="",$D45&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C45,$C45,$D$2:$D45,"Activo"))</f>
+      </c>
+      <c r="Q45" s="19">
+        <f>IF($P45="","",$C45&amp;"|"&amp;$P45)</f>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="20"/>
@@ -4696,6 +6126,15 @@
       <c r="L46" s="17">
         <f>IF($A46="","",IFERROR(VLOOKUP($C46,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M46" s="20"/>
+      <c r="N46" s="22"/>
+      <c r="O46" s="22"/>
+      <c r="P46" s="17">
+        <f>IF(OR($A46="",$D46&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C46,$C46,$D$2:$D46,"Activo"))</f>
+      </c>
+      <c r="Q46" s="19">
+        <f>IF($P46="","",$C46&amp;"|"&amp;$P46)</f>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="20"/>
@@ -4724,6 +6163,15 @@
       <c r="L47" s="17">
         <f>IF($A47="","",IFERROR(VLOOKUP($C47,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M47" s="20"/>
+      <c r="N47" s="22"/>
+      <c r="O47" s="22"/>
+      <c r="P47" s="17">
+        <f>IF(OR($A47="",$D47&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C47,$C47,$D$2:$D47,"Activo"))</f>
+      </c>
+      <c r="Q47" s="19">
+        <f>IF($P47="","",$C47&amp;"|"&amp;$P47)</f>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="20"/>
@@ -4752,6 +6200,15 @@
       <c r="L48" s="17">
         <f>IF($A48="","",IFERROR(VLOOKUP($C48,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M48" s="20"/>
+      <c r="N48" s="22"/>
+      <c r="O48" s="22"/>
+      <c r="P48" s="17">
+        <f>IF(OR($A48="",$D48&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C48,$C48,$D$2:$D48,"Activo"))</f>
+      </c>
+      <c r="Q48" s="19">
+        <f>IF($P48="","",$C48&amp;"|"&amp;$P48)</f>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="20"/>
@@ -4780,6 +6237,15 @@
       <c r="L49" s="17">
         <f>IF($A49="","",IFERROR(VLOOKUP($C49,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M49" s="20"/>
+      <c r="N49" s="22"/>
+      <c r="O49" s="22"/>
+      <c r="P49" s="17">
+        <f>IF(OR($A49="",$D49&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C49,$C49,$D$2:$D49,"Activo"))</f>
+      </c>
+      <c r="Q49" s="19">
+        <f>IF($P49="","",$C49&amp;"|"&amp;$P49)</f>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="20"/>
@@ -4808,6 +6274,15 @@
       <c r="L50" s="17">
         <f>IF($A50="","",IFERROR(VLOOKUP($C50,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M50" s="20"/>
+      <c r="N50" s="22"/>
+      <c r="O50" s="22"/>
+      <c r="P50" s="17">
+        <f>IF(OR($A50="",$D50&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C50,$C50,$D$2:$D50,"Activo"))</f>
+      </c>
+      <c r="Q50" s="19">
+        <f>IF($P50="","",$C50&amp;"|"&amp;$P50)</f>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="20"/>
@@ -4836,6 +6311,15 @@
       <c r="L51" s="17">
         <f>IF($A51="","",IFERROR(VLOOKUP($C51,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M51" s="20"/>
+      <c r="N51" s="22"/>
+      <c r="O51" s="22"/>
+      <c r="P51" s="17">
+        <f>IF(OR($A51="",$D51&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C51,$C51,$D$2:$D51,"Activo"))</f>
+      </c>
+      <c r="Q51" s="19">
+        <f>IF($P51="","",$C51&amp;"|"&amp;$P51)</f>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="20"/>
@@ -4864,6 +6348,15 @@
       <c r="L52" s="17">
         <f>IF($A52="","",IFERROR(VLOOKUP($C52,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M52" s="20"/>
+      <c r="N52" s="22"/>
+      <c r="O52" s="22"/>
+      <c r="P52" s="17">
+        <f>IF(OR($A52="",$D52&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C52,$C52,$D$2:$D52,"Activo"))</f>
+      </c>
+      <c r="Q52" s="19">
+        <f>IF($P52="","",$C52&amp;"|"&amp;$P52)</f>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="20"/>
@@ -4892,6 +6385,15 @@
       <c r="L53" s="17">
         <f>IF($A53="","",IFERROR(VLOOKUP($C53,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M53" s="20"/>
+      <c r="N53" s="22"/>
+      <c r="O53" s="22"/>
+      <c r="P53" s="17">
+        <f>IF(OR($A53="",$D53&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C53,$C53,$D$2:$D53,"Activo"))</f>
+      </c>
+      <c r="Q53" s="19">
+        <f>IF($P53="","",$C53&amp;"|"&amp;$P53)</f>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="20"/>
@@ -4920,6 +6422,15 @@
       <c r="L54" s="17">
         <f>IF($A54="","",IFERROR(VLOOKUP($C54,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M54" s="20"/>
+      <c r="N54" s="22"/>
+      <c r="O54" s="22"/>
+      <c r="P54" s="17">
+        <f>IF(OR($A54="",$D54&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C54,$C54,$D$2:$D54,"Activo"))</f>
+      </c>
+      <c r="Q54" s="19">
+        <f>IF($P54="","",$C54&amp;"|"&amp;$P54)</f>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="20"/>
@@ -4948,6 +6459,15 @@
       <c r="L55" s="17">
         <f>IF($A55="","",IFERROR(VLOOKUP($C55,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M55" s="20"/>
+      <c r="N55" s="22"/>
+      <c r="O55" s="22"/>
+      <c r="P55" s="17">
+        <f>IF(OR($A55="",$D55&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C55,$C55,$D$2:$D55,"Activo"))</f>
+      </c>
+      <c r="Q55" s="19">
+        <f>IF($P55="","",$C55&amp;"|"&amp;$P55)</f>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="20"/>
@@ -4976,6 +6496,15 @@
       <c r="L56" s="17">
         <f>IF($A56="","",IFERROR(VLOOKUP($C56,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M56" s="20"/>
+      <c r="N56" s="22"/>
+      <c r="O56" s="22"/>
+      <c r="P56" s="17">
+        <f>IF(OR($A56="",$D56&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C56,$C56,$D$2:$D56,"Activo"))</f>
+      </c>
+      <c r="Q56" s="19">
+        <f>IF($P56="","",$C56&amp;"|"&amp;$P56)</f>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="20"/>
@@ -5004,6 +6533,15 @@
       <c r="L57" s="17">
         <f>IF($A57="","",IFERROR(VLOOKUP($C57,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M57" s="20"/>
+      <c r="N57" s="22"/>
+      <c r="O57" s="22"/>
+      <c r="P57" s="17">
+        <f>IF(OR($A57="",$D57&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C57,$C57,$D$2:$D57,"Activo"))</f>
+      </c>
+      <c r="Q57" s="19">
+        <f>IF($P57="","",$C57&amp;"|"&amp;$P57)</f>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="20"/>
@@ -5032,6 +6570,15 @@
       <c r="L58" s="17">
         <f>IF($A58="","",IFERROR(VLOOKUP($C58,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M58" s="20"/>
+      <c r="N58" s="22"/>
+      <c r="O58" s="22"/>
+      <c r="P58" s="17">
+        <f>IF(OR($A58="",$D58&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C58,$C58,$D$2:$D58,"Activo"))</f>
+      </c>
+      <c r="Q58" s="19">
+        <f>IF($P58="","",$C58&amp;"|"&amp;$P58)</f>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="20"/>
@@ -5060,6 +6607,15 @@
       <c r="L59" s="17">
         <f>IF($A59="","",IFERROR(VLOOKUP($C59,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M59" s="20"/>
+      <c r="N59" s="22"/>
+      <c r="O59" s="22"/>
+      <c r="P59" s="17">
+        <f>IF(OR($A59="",$D59&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C59,$C59,$D$2:$D59,"Activo"))</f>
+      </c>
+      <c r="Q59" s="19">
+        <f>IF($P59="","",$C59&amp;"|"&amp;$P59)</f>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="20"/>
@@ -5088,6 +6644,15 @@
       <c r="L60" s="17">
         <f>IF($A60="","",IFERROR(VLOOKUP($C60,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M60" s="20"/>
+      <c r="N60" s="22"/>
+      <c r="O60" s="22"/>
+      <c r="P60" s="17">
+        <f>IF(OR($A60="",$D60&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C60,$C60,$D$2:$D60,"Activo"))</f>
+      </c>
+      <c r="Q60" s="19">
+        <f>IF($P60="","",$C60&amp;"|"&amp;$P60)</f>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="20"/>
@@ -5116,6 +6681,15 @@
       <c r="L61" s="17">
         <f>IF($A61="","",IFERROR(VLOOKUP($C61,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M61" s="20"/>
+      <c r="N61" s="22"/>
+      <c r="O61" s="22"/>
+      <c r="P61" s="17">
+        <f>IF(OR($A61="",$D61&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C61,$C61,$D$2:$D61,"Activo"))</f>
+      </c>
+      <c r="Q61" s="19">
+        <f>IF($P61="","",$C61&amp;"|"&amp;$P61)</f>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="20"/>
@@ -5144,6 +6718,15 @@
       <c r="L62" s="17">
         <f>IF($A62="","",IFERROR(VLOOKUP($C62,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M62" s="20"/>
+      <c r="N62" s="22"/>
+      <c r="O62" s="22"/>
+      <c r="P62" s="17">
+        <f>IF(OR($A62="",$D62&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C62,$C62,$D$2:$D62,"Activo"))</f>
+      </c>
+      <c r="Q62" s="19">
+        <f>IF($P62="","",$C62&amp;"|"&amp;$P62)</f>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="20"/>
@@ -5172,6 +6755,15 @@
       <c r="L63" s="17">
         <f>IF($A63="","",IFERROR(VLOOKUP($C63,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M63" s="20"/>
+      <c r="N63" s="22"/>
+      <c r="O63" s="22"/>
+      <c r="P63" s="17">
+        <f>IF(OR($A63="",$D63&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C63,$C63,$D$2:$D63,"Activo"))</f>
+      </c>
+      <c r="Q63" s="19">
+        <f>IF($P63="","",$C63&amp;"|"&amp;$P63)</f>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="20"/>
@@ -5200,6 +6792,15 @@
       <c r="L64" s="17">
         <f>IF($A64="","",IFERROR(VLOOKUP($C64,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M64" s="20"/>
+      <c r="N64" s="22"/>
+      <c r="O64" s="22"/>
+      <c r="P64" s="17">
+        <f>IF(OR($A64="",$D64&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C64,$C64,$D$2:$D64,"Activo"))</f>
+      </c>
+      <c r="Q64" s="19">
+        <f>IF($P64="","",$C64&amp;"|"&amp;$P64)</f>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="20"/>
@@ -5228,6 +6829,15 @@
       <c r="L65" s="17">
         <f>IF($A65="","",IFERROR(VLOOKUP($C65,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M65" s="20"/>
+      <c r="N65" s="22"/>
+      <c r="O65" s="22"/>
+      <c r="P65" s="17">
+        <f>IF(OR($A65="",$D65&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C65,$C65,$D$2:$D65,"Activo"))</f>
+      </c>
+      <c r="Q65" s="19">
+        <f>IF($P65="","",$C65&amp;"|"&amp;$P65)</f>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="20"/>
@@ -5256,6 +6866,15 @@
       <c r="L66" s="17">
         <f>IF($A66="","",IFERROR(VLOOKUP($C66,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M66" s="20"/>
+      <c r="N66" s="22"/>
+      <c r="O66" s="22"/>
+      <c r="P66" s="17">
+        <f>IF(OR($A66="",$D66&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C66,$C66,$D$2:$D66,"Activo"))</f>
+      </c>
+      <c r="Q66" s="19">
+        <f>IF($P66="","",$C66&amp;"|"&amp;$P66)</f>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="20"/>
@@ -5284,6 +6903,15 @@
       <c r="L67" s="17">
         <f>IF($A67="","",IFERROR(VLOOKUP($C67,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M67" s="20"/>
+      <c r="N67" s="22"/>
+      <c r="O67" s="22"/>
+      <c r="P67" s="17">
+        <f>IF(OR($A67="",$D67&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C67,$C67,$D$2:$D67,"Activo"))</f>
+      </c>
+      <c r="Q67" s="19">
+        <f>IF($P67="","",$C67&amp;"|"&amp;$P67)</f>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="20"/>
@@ -5312,6 +6940,15 @@
       <c r="L68" s="17">
         <f>IF($A68="","",IFERROR(VLOOKUP($C68,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M68" s="20"/>
+      <c r="N68" s="22"/>
+      <c r="O68" s="22"/>
+      <c r="P68" s="17">
+        <f>IF(OR($A68="",$D68&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C68,$C68,$D$2:$D68,"Activo"))</f>
+      </c>
+      <c r="Q68" s="19">
+        <f>IF($P68="","",$C68&amp;"|"&amp;$P68)</f>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="20"/>
@@ -5340,6 +6977,15 @@
       <c r="L69" s="17">
         <f>IF($A69="","",IFERROR(VLOOKUP($C69,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M69" s="20"/>
+      <c r="N69" s="22"/>
+      <c r="O69" s="22"/>
+      <c r="P69" s="17">
+        <f>IF(OR($A69="",$D69&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C69,$C69,$D$2:$D69,"Activo"))</f>
+      </c>
+      <c r="Q69" s="19">
+        <f>IF($P69="","",$C69&amp;"|"&amp;$P69)</f>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="20"/>
@@ -5368,6 +7014,15 @@
       <c r="L70" s="17">
         <f>IF($A70="","",IFERROR(VLOOKUP($C70,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M70" s="20"/>
+      <c r="N70" s="22"/>
+      <c r="O70" s="22"/>
+      <c r="P70" s="17">
+        <f>IF(OR($A70="",$D70&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C70,$C70,$D$2:$D70,"Activo"))</f>
+      </c>
+      <c r="Q70" s="19">
+        <f>IF($P70="","",$C70&amp;"|"&amp;$P70)</f>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="20"/>
@@ -5396,6 +7051,15 @@
       <c r="L71" s="17">
         <f>IF($A71="","",IFERROR(VLOOKUP($C71,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M71" s="20"/>
+      <c r="N71" s="22"/>
+      <c r="O71" s="22"/>
+      <c r="P71" s="17">
+        <f>IF(OR($A71="",$D71&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C71,$C71,$D$2:$D71,"Activo"))</f>
+      </c>
+      <c r="Q71" s="19">
+        <f>IF($P71="","",$C71&amp;"|"&amp;$P71)</f>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="20"/>
@@ -5424,6 +7088,15 @@
       <c r="L72" s="17">
         <f>IF($A72="","",IFERROR(VLOOKUP($C72,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M72" s="20"/>
+      <c r="N72" s="22"/>
+      <c r="O72" s="22"/>
+      <c r="P72" s="17">
+        <f>IF(OR($A72="",$D72&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C72,$C72,$D$2:$D72,"Activo"))</f>
+      </c>
+      <c r="Q72" s="19">
+        <f>IF($P72="","",$C72&amp;"|"&amp;$P72)</f>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="20"/>
@@ -5452,6 +7125,15 @@
       <c r="L73" s="17">
         <f>IF($A73="","",IFERROR(VLOOKUP($C73,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M73" s="20"/>
+      <c r="N73" s="22"/>
+      <c r="O73" s="22"/>
+      <c r="P73" s="17">
+        <f>IF(OR($A73="",$D73&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C73,$C73,$D$2:$D73,"Activo"))</f>
+      </c>
+      <c r="Q73" s="19">
+        <f>IF($P73="","",$C73&amp;"|"&amp;$P73)</f>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="20"/>
@@ -5480,6 +7162,15 @@
       <c r="L74" s="17">
         <f>IF($A74="","",IFERROR(VLOOKUP($C74,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M74" s="20"/>
+      <c r="N74" s="22"/>
+      <c r="O74" s="22"/>
+      <c r="P74" s="17">
+        <f>IF(OR($A74="",$D74&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C74,$C74,$D$2:$D74,"Activo"))</f>
+      </c>
+      <c r="Q74" s="19">
+        <f>IF($P74="","",$C74&amp;"|"&amp;$P74)</f>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="20"/>
@@ -5508,6 +7199,15 @@
       <c r="L75" s="17">
         <f>IF($A75="","",IFERROR(VLOOKUP($C75,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M75" s="20"/>
+      <c r="N75" s="22"/>
+      <c r="O75" s="22"/>
+      <c r="P75" s="17">
+        <f>IF(OR($A75="",$D75&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C75,$C75,$D$2:$D75,"Activo"))</f>
+      </c>
+      <c r="Q75" s="19">
+        <f>IF($P75="","",$C75&amp;"|"&amp;$P75)</f>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="20"/>
@@ -5536,6 +7236,15 @@
       <c r="L76" s="17">
         <f>IF($A76="","",IFERROR(VLOOKUP($C76,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M76" s="20"/>
+      <c r="N76" s="22"/>
+      <c r="O76" s="22"/>
+      <c r="P76" s="17">
+        <f>IF(OR($A76="",$D76&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C76,$C76,$D$2:$D76,"Activo"))</f>
+      </c>
+      <c r="Q76" s="19">
+        <f>IF($P76="","",$C76&amp;"|"&amp;$P76)</f>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="20"/>
@@ -5564,6 +7273,15 @@
       <c r="L77" s="17">
         <f>IF($A77="","",IFERROR(VLOOKUP($C77,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M77" s="20"/>
+      <c r="N77" s="22"/>
+      <c r="O77" s="22"/>
+      <c r="P77" s="17">
+        <f>IF(OR($A77="",$D77&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C77,$C77,$D$2:$D77,"Activo"))</f>
+      </c>
+      <c r="Q77" s="19">
+        <f>IF($P77="","",$C77&amp;"|"&amp;$P77)</f>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="20"/>
@@ -5592,6 +7310,15 @@
       <c r="L78" s="17">
         <f>IF($A78="","",IFERROR(VLOOKUP($C78,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M78" s="20"/>
+      <c r="N78" s="22"/>
+      <c r="O78" s="22"/>
+      <c r="P78" s="17">
+        <f>IF(OR($A78="",$D78&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C78,$C78,$D$2:$D78,"Activo"))</f>
+      </c>
+      <c r="Q78" s="19">
+        <f>IF($P78="","",$C78&amp;"|"&amp;$P78)</f>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="20"/>
@@ -5620,6 +7347,15 @@
       <c r="L79" s="17">
         <f>IF($A79="","",IFERROR(VLOOKUP($C79,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M79" s="20"/>
+      <c r="N79" s="22"/>
+      <c r="O79" s="22"/>
+      <c r="P79" s="17">
+        <f>IF(OR($A79="",$D79&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C79,$C79,$D$2:$D79,"Activo"))</f>
+      </c>
+      <c r="Q79" s="19">
+        <f>IF($P79="","",$C79&amp;"|"&amp;$P79)</f>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="20"/>
@@ -5648,6 +7384,15 @@
       <c r="L80" s="17">
         <f>IF($A80="","",IFERROR(VLOOKUP($C80,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M80" s="20"/>
+      <c r="N80" s="22"/>
+      <c r="O80" s="22"/>
+      <c r="P80" s="17">
+        <f>IF(OR($A80="",$D80&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C80,$C80,$D$2:$D80,"Activo"))</f>
+      </c>
+      <c r="Q80" s="19">
+        <f>IF($P80="","",$C80&amp;"|"&amp;$P80)</f>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="20"/>
@@ -5676,6 +7421,15 @@
       <c r="L81" s="17">
         <f>IF($A81="","",IFERROR(VLOOKUP($C81,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M81" s="20"/>
+      <c r="N81" s="22"/>
+      <c r="O81" s="22"/>
+      <c r="P81" s="17">
+        <f>IF(OR($A81="",$D81&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C81,$C81,$D$2:$D81,"Activo"))</f>
+      </c>
+      <c r="Q81" s="19">
+        <f>IF($P81="","",$C81&amp;"|"&amp;$P81)</f>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="20"/>
@@ -5704,6 +7458,15 @@
       <c r="L82" s="17">
         <f>IF($A82="","",IFERROR(VLOOKUP($C82,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M82" s="20"/>
+      <c r="N82" s="22"/>
+      <c r="O82" s="22"/>
+      <c r="P82" s="17">
+        <f>IF(OR($A82="",$D82&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C82,$C82,$D$2:$D82,"Activo"))</f>
+      </c>
+      <c r="Q82" s="19">
+        <f>IF($P82="","",$C82&amp;"|"&amp;$P82)</f>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="20"/>
@@ -5732,6 +7495,15 @@
       <c r="L83" s="17">
         <f>IF($A83="","",IFERROR(VLOOKUP($C83,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M83" s="20"/>
+      <c r="N83" s="22"/>
+      <c r="O83" s="22"/>
+      <c r="P83" s="17">
+        <f>IF(OR($A83="",$D83&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C83,$C83,$D$2:$D83,"Activo"))</f>
+      </c>
+      <c r="Q83" s="19">
+        <f>IF($P83="","",$C83&amp;"|"&amp;$P83)</f>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="20"/>
@@ -5760,6 +7532,15 @@
       <c r="L84" s="17">
         <f>IF($A84="","",IFERROR(VLOOKUP($C84,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M84" s="20"/>
+      <c r="N84" s="22"/>
+      <c r="O84" s="22"/>
+      <c r="P84" s="17">
+        <f>IF(OR($A84="",$D84&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C84,$C84,$D$2:$D84,"Activo"))</f>
+      </c>
+      <c r="Q84" s="19">
+        <f>IF($P84="","",$C84&amp;"|"&amp;$P84)</f>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="20"/>
@@ -5788,6 +7569,15 @@
       <c r="L85" s="17">
         <f>IF($A85="","",IFERROR(VLOOKUP($C85,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M85" s="20"/>
+      <c r="N85" s="22"/>
+      <c r="O85" s="22"/>
+      <c r="P85" s="17">
+        <f>IF(OR($A85="",$D85&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C85,$C85,$D$2:$D85,"Activo"))</f>
+      </c>
+      <c r="Q85" s="19">
+        <f>IF($P85="","",$C85&amp;"|"&amp;$P85)</f>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="20"/>
@@ -5816,6 +7606,15 @@
       <c r="L86" s="17">
         <f>IF($A86="","",IFERROR(VLOOKUP($C86,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M86" s="20"/>
+      <c r="N86" s="22"/>
+      <c r="O86" s="22"/>
+      <c r="P86" s="17">
+        <f>IF(OR($A86="",$D86&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C86,$C86,$D$2:$D86,"Activo"))</f>
+      </c>
+      <c r="Q86" s="19">
+        <f>IF($P86="","",$C86&amp;"|"&amp;$P86)</f>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="20"/>
@@ -5844,6 +7643,15 @@
       <c r="L87" s="17">
         <f>IF($A87="","",IFERROR(VLOOKUP($C87,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M87" s="20"/>
+      <c r="N87" s="22"/>
+      <c r="O87" s="22"/>
+      <c r="P87" s="17">
+        <f>IF(OR($A87="",$D87&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C87,$C87,$D$2:$D87,"Activo"))</f>
+      </c>
+      <c r="Q87" s="19">
+        <f>IF($P87="","",$C87&amp;"|"&amp;$P87)</f>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="20"/>
@@ -5872,6 +7680,15 @@
       <c r="L88" s="17">
         <f>IF($A88="","",IFERROR(VLOOKUP($C88,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M88" s="20"/>
+      <c r="N88" s="22"/>
+      <c r="O88" s="22"/>
+      <c r="P88" s="17">
+        <f>IF(OR($A88="",$D88&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C88,$C88,$D$2:$D88,"Activo"))</f>
+      </c>
+      <c r="Q88" s="19">
+        <f>IF($P88="","",$C88&amp;"|"&amp;$P88)</f>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="20"/>
@@ -5900,6 +7717,15 @@
       <c r="L89" s="17">
         <f>IF($A89="","",IFERROR(VLOOKUP($C89,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M89" s="20"/>
+      <c r="N89" s="22"/>
+      <c r="O89" s="22"/>
+      <c r="P89" s="17">
+        <f>IF(OR($A89="",$D89&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C89,$C89,$D$2:$D89,"Activo"))</f>
+      </c>
+      <c r="Q89" s="19">
+        <f>IF($P89="","",$C89&amp;"|"&amp;$P89)</f>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="20"/>
@@ -5928,6 +7754,15 @@
       <c r="L90" s="17">
         <f>IF($A90="","",IFERROR(VLOOKUP($C90,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M90" s="20"/>
+      <c r="N90" s="22"/>
+      <c r="O90" s="22"/>
+      <c r="P90" s="17">
+        <f>IF(OR($A90="",$D90&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C90,$C90,$D$2:$D90,"Activo"))</f>
+      </c>
+      <c r="Q90" s="19">
+        <f>IF($P90="","",$C90&amp;"|"&amp;$P90)</f>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="20"/>
@@ -5956,6 +7791,15 @@
       <c r="L91" s="17">
         <f>IF($A91="","",IFERROR(VLOOKUP($C91,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M91" s="20"/>
+      <c r="N91" s="22"/>
+      <c r="O91" s="22"/>
+      <c r="P91" s="17">
+        <f>IF(OR($A91="",$D91&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C91,$C91,$D$2:$D91,"Activo"))</f>
+      </c>
+      <c r="Q91" s="19">
+        <f>IF($P91="","",$C91&amp;"|"&amp;$P91)</f>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="20"/>
@@ -5984,6 +7828,15 @@
       <c r="L92" s="17">
         <f>IF($A92="","",IFERROR(VLOOKUP($C92,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M92" s="20"/>
+      <c r="N92" s="22"/>
+      <c r="O92" s="22"/>
+      <c r="P92" s="17">
+        <f>IF(OR($A92="",$D92&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C92,$C92,$D$2:$D92,"Activo"))</f>
+      </c>
+      <c r="Q92" s="19">
+        <f>IF($P92="","",$C92&amp;"|"&amp;$P92)</f>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="20"/>
@@ -6012,6 +7865,15 @@
       <c r="L93" s="17">
         <f>IF($A93="","",IFERROR(VLOOKUP($C93,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M93" s="20"/>
+      <c r="N93" s="22"/>
+      <c r="O93" s="22"/>
+      <c r="P93" s="17">
+        <f>IF(OR($A93="",$D93&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C93,$C93,$D$2:$D93,"Activo"))</f>
+      </c>
+      <c r="Q93" s="19">
+        <f>IF($P93="","",$C93&amp;"|"&amp;$P93)</f>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="20"/>
@@ -6040,6 +7902,15 @@
       <c r="L94" s="17">
         <f>IF($A94="","",IFERROR(VLOOKUP($C94,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M94" s="20"/>
+      <c r="N94" s="22"/>
+      <c r="O94" s="22"/>
+      <c r="P94" s="17">
+        <f>IF(OR($A94="",$D94&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C94,$C94,$D$2:$D94,"Activo"))</f>
+      </c>
+      <c r="Q94" s="19">
+        <f>IF($P94="","",$C94&amp;"|"&amp;$P94)</f>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="20"/>
@@ -6068,6 +7939,15 @@
       <c r="L95" s="17">
         <f>IF($A95="","",IFERROR(VLOOKUP($C95,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M95" s="20"/>
+      <c r="N95" s="22"/>
+      <c r="O95" s="22"/>
+      <c r="P95" s="17">
+        <f>IF(OR($A95="",$D95&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C95,$C95,$D$2:$D95,"Activo"))</f>
+      </c>
+      <c r="Q95" s="19">
+        <f>IF($P95="","",$C95&amp;"|"&amp;$P95)</f>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="20"/>
@@ -6096,6 +7976,15 @@
       <c r="L96" s="17">
         <f>IF($A96="","",IFERROR(VLOOKUP($C96,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M96" s="20"/>
+      <c r="N96" s="22"/>
+      <c r="O96" s="22"/>
+      <c r="P96" s="17">
+        <f>IF(OR($A96="",$D96&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C96,$C96,$D$2:$D96,"Activo"))</f>
+      </c>
+      <c r="Q96" s="19">
+        <f>IF($P96="","",$C96&amp;"|"&amp;$P96)</f>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="20"/>
@@ -6124,6 +8013,15 @@
       <c r="L97" s="17">
         <f>IF($A97="","",IFERROR(VLOOKUP($C97,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M97" s="20"/>
+      <c r="N97" s="22"/>
+      <c r="O97" s="22"/>
+      <c r="P97" s="17">
+        <f>IF(OR($A97="",$D97&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C97,$C97,$D$2:$D97,"Activo"))</f>
+      </c>
+      <c r="Q97" s="19">
+        <f>IF($P97="","",$C97&amp;"|"&amp;$P97)</f>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="20"/>
@@ -6152,6 +8050,15 @@
       <c r="L98" s="17">
         <f>IF($A98="","",IFERROR(VLOOKUP($C98,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M98" s="20"/>
+      <c r="N98" s="22"/>
+      <c r="O98" s="22"/>
+      <c r="P98" s="17">
+        <f>IF(OR($A98="",$D98&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C98,$C98,$D$2:$D98,"Activo"))</f>
+      </c>
+      <c r="Q98" s="19">
+        <f>IF($P98="","",$C98&amp;"|"&amp;$P98)</f>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="20"/>
@@ -6180,6 +8087,15 @@
       <c r="L99" s="17">
         <f>IF($A99="","",IFERROR(VLOOKUP($C99,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M99" s="20"/>
+      <c r="N99" s="22"/>
+      <c r="O99" s="22"/>
+      <c r="P99" s="17">
+        <f>IF(OR($A99="",$D99&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C99,$C99,$D$2:$D99,"Activo"))</f>
+      </c>
+      <c r="Q99" s="19">
+        <f>IF($P99="","",$C99&amp;"|"&amp;$P99)</f>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="20"/>
@@ -6208,6 +8124,15 @@
       <c r="L100" s="17">
         <f>IF($A100="","",IFERROR(VLOOKUP($C100,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M100" s="20"/>
+      <c r="N100" s="22"/>
+      <c r="O100" s="22"/>
+      <c r="P100" s="17">
+        <f>IF(OR($A100="",$D100&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C100,$C100,$D$2:$D100,"Activo"))</f>
+      </c>
+      <c r="Q100" s="19">
+        <f>IF($P100="","",$C100&amp;"|"&amp;$P100)</f>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="20"/>
@@ -6236,6 +8161,15 @@
       <c r="L101" s="17">
         <f>IF($A101="","",IFERROR(VLOOKUP($C101,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M101" s="20"/>
+      <c r="N101" s="22"/>
+      <c r="O101" s="22"/>
+      <c r="P101" s="17">
+        <f>IF(OR($A101="",$D101&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C101,$C101,$D$2:$D101,"Activo"))</f>
+      </c>
+      <c r="Q101" s="19">
+        <f>IF($P101="","",$C101&amp;"|"&amp;$P101)</f>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="20"/>
@@ -6264,6 +8198,15 @@
       <c r="L102" s="17">
         <f>IF($A102="","",IFERROR(VLOOKUP($C102,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M102" s="20"/>
+      <c r="N102" s="22"/>
+      <c r="O102" s="22"/>
+      <c r="P102" s="17">
+        <f>IF(OR($A102="",$D102&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C102,$C102,$D$2:$D102,"Activo"))</f>
+      </c>
+      <c r="Q102" s="19">
+        <f>IF($P102="","",$C102&amp;"|"&amp;$P102)</f>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="20"/>
@@ -6292,6 +8235,15 @@
       <c r="L103" s="17">
         <f>IF($A103="","",IFERROR(VLOOKUP($C103,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M103" s="20"/>
+      <c r="N103" s="22"/>
+      <c r="O103" s="22"/>
+      <c r="P103" s="17">
+        <f>IF(OR($A103="",$D103&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C103,$C103,$D$2:$D103,"Activo"))</f>
+      </c>
+      <c r="Q103" s="19">
+        <f>IF($P103="","",$C103&amp;"|"&amp;$P103)</f>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="20"/>
@@ -6320,6 +8272,15 @@
       <c r="L104" s="17">
         <f>IF($A104="","",IFERROR(VLOOKUP($C104,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M104" s="20"/>
+      <c r="N104" s="22"/>
+      <c r="O104" s="22"/>
+      <c r="P104" s="17">
+        <f>IF(OR($A104="",$D104&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C104,$C104,$D$2:$D104,"Activo"))</f>
+      </c>
+      <c r="Q104" s="19">
+        <f>IF($P104="","",$C104&amp;"|"&amp;$P104)</f>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="20"/>
@@ -6348,6 +8309,15 @@
       <c r="L105" s="17">
         <f>IF($A105="","",IFERROR(VLOOKUP($C105,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M105" s="20"/>
+      <c r="N105" s="22"/>
+      <c r="O105" s="22"/>
+      <c r="P105" s="17">
+        <f>IF(OR($A105="",$D105&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C105,$C105,$D$2:$D105,"Activo"))</f>
+      </c>
+      <c r="Q105" s="19">
+        <f>IF($P105="","",$C105&amp;"|"&amp;$P105)</f>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="20"/>
@@ -6376,6 +8346,15 @@
       <c r="L106" s="17">
         <f>IF($A106="","",IFERROR(VLOOKUP($C106,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M106" s="20"/>
+      <c r="N106" s="22"/>
+      <c r="O106" s="22"/>
+      <c r="P106" s="17">
+        <f>IF(OR($A106="",$D106&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C106,$C106,$D$2:$D106,"Activo"))</f>
+      </c>
+      <c r="Q106" s="19">
+        <f>IF($P106="","",$C106&amp;"|"&amp;$P106)</f>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="20"/>
@@ -6404,6 +8383,15 @@
       <c r="L107" s="17">
         <f>IF($A107="","",IFERROR(VLOOKUP($C107,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M107" s="20"/>
+      <c r="N107" s="22"/>
+      <c r="O107" s="22"/>
+      <c r="P107" s="17">
+        <f>IF(OR($A107="",$D107&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C107,$C107,$D$2:$D107,"Activo"))</f>
+      </c>
+      <c r="Q107" s="19">
+        <f>IF($P107="","",$C107&amp;"|"&amp;$P107)</f>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="20"/>
@@ -6432,6 +8420,15 @@
       <c r="L108" s="17">
         <f>IF($A108="","",IFERROR(VLOOKUP($C108,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M108" s="20"/>
+      <c r="N108" s="22"/>
+      <c r="O108" s="22"/>
+      <c r="P108" s="17">
+        <f>IF(OR($A108="",$D108&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C108,$C108,$D$2:$D108,"Activo"))</f>
+      </c>
+      <c r="Q108" s="19">
+        <f>IF($P108="","",$C108&amp;"|"&amp;$P108)</f>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="20"/>
@@ -6460,6 +8457,15 @@
       <c r="L109" s="17">
         <f>IF($A109="","",IFERROR(VLOOKUP($C109,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M109" s="20"/>
+      <c r="N109" s="22"/>
+      <c r="O109" s="22"/>
+      <c r="P109" s="17">
+        <f>IF(OR($A109="",$D109&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C109,$C109,$D$2:$D109,"Activo"))</f>
+      </c>
+      <c r="Q109" s="19">
+        <f>IF($P109="","",$C109&amp;"|"&amp;$P109)</f>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="20"/>
@@ -6488,6 +8494,15 @@
       <c r="L110" s="17">
         <f>IF($A110="","",IFERROR(VLOOKUP($C110,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M110" s="20"/>
+      <c r="N110" s="22"/>
+      <c r="O110" s="22"/>
+      <c r="P110" s="17">
+        <f>IF(OR($A110="",$D110&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C110,$C110,$D$2:$D110,"Activo"))</f>
+      </c>
+      <c r="Q110" s="19">
+        <f>IF($P110="","",$C110&amp;"|"&amp;$P110)</f>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="20"/>
@@ -6516,6 +8531,15 @@
       <c r="L111" s="17">
         <f>IF($A111="","",IFERROR(VLOOKUP($C111,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M111" s="20"/>
+      <c r="N111" s="22"/>
+      <c r="O111" s="22"/>
+      <c r="P111" s="17">
+        <f>IF(OR($A111="",$D111&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C111,$C111,$D$2:$D111,"Activo"))</f>
+      </c>
+      <c r="Q111" s="19">
+        <f>IF($P111="","",$C111&amp;"|"&amp;$P111)</f>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="20"/>
@@ -6544,6 +8568,15 @@
       <c r="L112" s="17">
         <f>IF($A112="","",IFERROR(VLOOKUP($C112,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M112" s="20"/>
+      <c r="N112" s="22"/>
+      <c r="O112" s="22"/>
+      <c r="P112" s="17">
+        <f>IF(OR($A112="",$D112&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C112,$C112,$D$2:$D112,"Activo"))</f>
+      </c>
+      <c r="Q112" s="19">
+        <f>IF($P112="","",$C112&amp;"|"&amp;$P112)</f>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="20"/>
@@ -6572,6 +8605,15 @@
       <c r="L113" s="17">
         <f>IF($A113="","",IFERROR(VLOOKUP($C113,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M113" s="20"/>
+      <c r="N113" s="22"/>
+      <c r="O113" s="22"/>
+      <c r="P113" s="17">
+        <f>IF(OR($A113="",$D113&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C113,$C113,$D$2:$D113,"Activo"))</f>
+      </c>
+      <c r="Q113" s="19">
+        <f>IF($P113="","",$C113&amp;"|"&amp;$P113)</f>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="20"/>
@@ -6600,6 +8642,15 @@
       <c r="L114" s="17">
         <f>IF($A114="","",IFERROR(VLOOKUP($C114,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M114" s="20"/>
+      <c r="N114" s="22"/>
+      <c r="O114" s="22"/>
+      <c r="P114" s="17">
+        <f>IF(OR($A114="",$D114&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C114,$C114,$D$2:$D114,"Activo"))</f>
+      </c>
+      <c r="Q114" s="19">
+        <f>IF($P114="","",$C114&amp;"|"&amp;$P114)</f>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="20"/>
@@ -6628,6 +8679,15 @@
       <c r="L115" s="17">
         <f>IF($A115="","",IFERROR(VLOOKUP($C115,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M115" s="20"/>
+      <c r="N115" s="22"/>
+      <c r="O115" s="22"/>
+      <c r="P115" s="17">
+        <f>IF(OR($A115="",$D115&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C115,$C115,$D$2:$D115,"Activo"))</f>
+      </c>
+      <c r="Q115" s="19">
+        <f>IF($P115="","",$C115&amp;"|"&amp;$P115)</f>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="20"/>
@@ -6656,6 +8716,15 @@
       <c r="L116" s="17">
         <f>IF($A116="","",IFERROR(VLOOKUP($C116,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M116" s="20"/>
+      <c r="N116" s="22"/>
+      <c r="O116" s="22"/>
+      <c r="P116" s="17">
+        <f>IF(OR($A116="",$D116&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C116,$C116,$D$2:$D116,"Activo"))</f>
+      </c>
+      <c r="Q116" s="19">
+        <f>IF($P116="","",$C116&amp;"|"&amp;$P116)</f>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="20"/>
@@ -6684,6 +8753,15 @@
       <c r="L117" s="17">
         <f>IF($A117="","",IFERROR(VLOOKUP($C117,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M117" s="20"/>
+      <c r="N117" s="22"/>
+      <c r="O117" s="22"/>
+      <c r="P117" s="17">
+        <f>IF(OR($A117="",$D117&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C117,$C117,$D$2:$D117,"Activo"))</f>
+      </c>
+      <c r="Q117" s="19">
+        <f>IF($P117="","",$C117&amp;"|"&amp;$P117)</f>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="20"/>
@@ -6712,6 +8790,15 @@
       <c r="L118" s="17">
         <f>IF($A118="","",IFERROR(VLOOKUP($C118,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M118" s="20"/>
+      <c r="N118" s="22"/>
+      <c r="O118" s="22"/>
+      <c r="P118" s="17">
+        <f>IF(OR($A118="",$D118&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C118,$C118,$D$2:$D118,"Activo"))</f>
+      </c>
+      <c r="Q118" s="19">
+        <f>IF($P118="","",$C118&amp;"|"&amp;$P118)</f>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="20"/>
@@ -6740,6 +8827,15 @@
       <c r="L119" s="17">
         <f>IF($A119="","",IFERROR(VLOOKUP($C119,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M119" s="20"/>
+      <c r="N119" s="22"/>
+      <c r="O119" s="22"/>
+      <c r="P119" s="17">
+        <f>IF(OR($A119="",$D119&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C119,$C119,$D$2:$D119,"Activo"))</f>
+      </c>
+      <c r="Q119" s="19">
+        <f>IF($P119="","",$C119&amp;"|"&amp;$P119)</f>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="20"/>
@@ -6768,6 +8864,15 @@
       <c r="L120" s="17">
         <f>IF($A120="","",IFERROR(VLOOKUP($C120,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M120" s="20"/>
+      <c r="N120" s="22"/>
+      <c r="O120" s="22"/>
+      <c r="P120" s="17">
+        <f>IF(OR($A120="",$D120&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C120,$C120,$D$2:$D120,"Activo"))</f>
+      </c>
+      <c r="Q120" s="19">
+        <f>IF($P120="","",$C120&amp;"|"&amp;$P120)</f>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="20"/>
@@ -6796,6 +8901,15 @@
       <c r="L121" s="17">
         <f>IF($A121="","",IFERROR(VLOOKUP($C121,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M121" s="20"/>
+      <c r="N121" s="22"/>
+      <c r="O121" s="22"/>
+      <c r="P121" s="17">
+        <f>IF(OR($A121="",$D121&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C121,$C121,$D$2:$D121,"Activo"))</f>
+      </c>
+      <c r="Q121" s="19">
+        <f>IF($P121="","",$C121&amp;"|"&amp;$P121)</f>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="20"/>
@@ -6824,6 +8938,15 @@
       <c r="L122" s="17">
         <f>IF($A122="","",IFERROR(VLOOKUP($C122,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M122" s="20"/>
+      <c r="N122" s="22"/>
+      <c r="O122" s="22"/>
+      <c r="P122" s="17">
+        <f>IF(OR($A122="",$D122&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C122,$C122,$D$2:$D122,"Activo"))</f>
+      </c>
+      <c r="Q122" s="19">
+        <f>IF($P122="","",$C122&amp;"|"&amp;$P122)</f>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="20"/>
@@ -6852,6 +8975,15 @@
       <c r="L123" s="17">
         <f>IF($A123="","",IFERROR(VLOOKUP($C123,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M123" s="20"/>
+      <c r="N123" s="22"/>
+      <c r="O123" s="22"/>
+      <c r="P123" s="17">
+        <f>IF(OR($A123="",$D123&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C123,$C123,$D$2:$D123,"Activo"))</f>
+      </c>
+      <c r="Q123" s="19">
+        <f>IF($P123="","",$C123&amp;"|"&amp;$P123)</f>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="20"/>
@@ -6880,6 +9012,15 @@
       <c r="L124" s="17">
         <f>IF($A124="","",IFERROR(VLOOKUP($C124,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M124" s="20"/>
+      <c r="N124" s="22"/>
+      <c r="O124" s="22"/>
+      <c r="P124" s="17">
+        <f>IF(OR($A124="",$D124&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C124,$C124,$D$2:$D124,"Activo"))</f>
+      </c>
+      <c r="Q124" s="19">
+        <f>IF($P124="","",$C124&amp;"|"&amp;$P124)</f>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="20"/>
@@ -6908,6 +9049,15 @@
       <c r="L125" s="17">
         <f>IF($A125="","",IFERROR(VLOOKUP($C125,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M125" s="20"/>
+      <c r="N125" s="22"/>
+      <c r="O125" s="22"/>
+      <c r="P125" s="17">
+        <f>IF(OR($A125="",$D125&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C125,$C125,$D$2:$D125,"Activo"))</f>
+      </c>
+      <c r="Q125" s="19">
+        <f>IF($P125="","",$C125&amp;"|"&amp;$P125)</f>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="20"/>
@@ -6936,6 +9086,15 @@
       <c r="L126" s="17">
         <f>IF($A126="","",IFERROR(VLOOKUP($C126,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M126" s="20"/>
+      <c r="N126" s="22"/>
+      <c r="O126" s="22"/>
+      <c r="P126" s="17">
+        <f>IF(OR($A126="",$D126&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C126,$C126,$D$2:$D126,"Activo"))</f>
+      </c>
+      <c r="Q126" s="19">
+        <f>IF($P126="","",$C126&amp;"|"&amp;$P126)</f>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="20"/>
@@ -6964,6 +9123,15 @@
       <c r="L127" s="17">
         <f>IF($A127="","",IFERROR(VLOOKUP($C127,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M127" s="20"/>
+      <c r="N127" s="22"/>
+      <c r="O127" s="22"/>
+      <c r="P127" s="17">
+        <f>IF(OR($A127="",$D127&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C127,$C127,$D$2:$D127,"Activo"))</f>
+      </c>
+      <c r="Q127" s="19">
+        <f>IF($P127="","",$C127&amp;"|"&amp;$P127)</f>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="20"/>
@@ -6992,6 +9160,15 @@
       <c r="L128" s="17">
         <f>IF($A128="","",IFERROR(VLOOKUP($C128,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M128" s="20"/>
+      <c r="N128" s="22"/>
+      <c r="O128" s="22"/>
+      <c r="P128" s="17">
+        <f>IF(OR($A128="",$D128&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C128,$C128,$D$2:$D128,"Activo"))</f>
+      </c>
+      <c r="Q128" s="19">
+        <f>IF($P128="","",$C128&amp;"|"&amp;$P128)</f>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="20"/>
@@ -7020,6 +9197,15 @@
       <c r="L129" s="17">
         <f>IF($A129="","",IFERROR(VLOOKUP($C129,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M129" s="20"/>
+      <c r="N129" s="22"/>
+      <c r="O129" s="22"/>
+      <c r="P129" s="17">
+        <f>IF(OR($A129="",$D129&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C129,$C129,$D$2:$D129,"Activo"))</f>
+      </c>
+      <c r="Q129" s="19">
+        <f>IF($P129="","",$C129&amp;"|"&amp;$P129)</f>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="20"/>
@@ -7048,6 +9234,15 @@
       <c r="L130" s="17">
         <f>IF($A130="","",IFERROR(VLOOKUP($C130,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M130" s="20"/>
+      <c r="N130" s="22"/>
+      <c r="O130" s="22"/>
+      <c r="P130" s="17">
+        <f>IF(OR($A130="",$D130&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C130,$C130,$D$2:$D130,"Activo"))</f>
+      </c>
+      <c r="Q130" s="19">
+        <f>IF($P130="","",$C130&amp;"|"&amp;$P130)</f>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="20"/>
@@ -7076,6 +9271,15 @@
       <c r="L131" s="17">
         <f>IF($A131="","",IFERROR(VLOOKUP($C131,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M131" s="20"/>
+      <c r="N131" s="22"/>
+      <c r="O131" s="22"/>
+      <c r="P131" s="17">
+        <f>IF(OR($A131="",$D131&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C131,$C131,$D$2:$D131,"Activo"))</f>
+      </c>
+      <c r="Q131" s="19">
+        <f>IF($P131="","",$C131&amp;"|"&amp;$P131)</f>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="20"/>
@@ -7104,6 +9308,15 @@
       <c r="L132" s="17">
         <f>IF($A132="","",IFERROR(VLOOKUP($C132,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M132" s="20"/>
+      <c r="N132" s="22"/>
+      <c r="O132" s="22"/>
+      <c r="P132" s="17">
+        <f>IF(OR($A132="",$D132&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C132,$C132,$D$2:$D132,"Activo"))</f>
+      </c>
+      <c r="Q132" s="19">
+        <f>IF($P132="","",$C132&amp;"|"&amp;$P132)</f>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="20"/>
@@ -7132,6 +9345,15 @@
       <c r="L133" s="17">
         <f>IF($A133="","",IFERROR(VLOOKUP($C133,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M133" s="20"/>
+      <c r="N133" s="22"/>
+      <c r="O133" s="22"/>
+      <c r="P133" s="17">
+        <f>IF(OR($A133="",$D133&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C133,$C133,$D$2:$D133,"Activo"))</f>
+      </c>
+      <c r="Q133" s="19">
+        <f>IF($P133="","",$C133&amp;"|"&amp;$P133)</f>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="20"/>
@@ -7160,6 +9382,15 @@
       <c r="L134" s="17">
         <f>IF($A134="","",IFERROR(VLOOKUP($C134,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M134" s="20"/>
+      <c r="N134" s="22"/>
+      <c r="O134" s="22"/>
+      <c r="P134" s="17">
+        <f>IF(OR($A134="",$D134&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C134,$C134,$D$2:$D134,"Activo"))</f>
+      </c>
+      <c r="Q134" s="19">
+        <f>IF($P134="","",$C134&amp;"|"&amp;$P134)</f>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="20"/>
@@ -7188,6 +9419,15 @@
       <c r="L135" s="17">
         <f>IF($A135="","",IFERROR(VLOOKUP($C135,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M135" s="20"/>
+      <c r="N135" s="22"/>
+      <c r="O135" s="22"/>
+      <c r="P135" s="17">
+        <f>IF(OR($A135="",$D135&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C135,$C135,$D$2:$D135,"Activo"))</f>
+      </c>
+      <c r="Q135" s="19">
+        <f>IF($P135="","",$C135&amp;"|"&amp;$P135)</f>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="20"/>
@@ -7216,6 +9456,15 @@
       <c r="L136" s="17">
         <f>IF($A136="","",IFERROR(VLOOKUP($C136,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M136" s="20"/>
+      <c r="N136" s="22"/>
+      <c r="O136" s="22"/>
+      <c r="P136" s="17">
+        <f>IF(OR($A136="",$D136&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C136,$C136,$D$2:$D136,"Activo"))</f>
+      </c>
+      <c r="Q136" s="19">
+        <f>IF($P136="","",$C136&amp;"|"&amp;$P136)</f>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="20"/>
@@ -7244,6 +9493,15 @@
       <c r="L137" s="17">
         <f>IF($A137="","",IFERROR(VLOOKUP($C137,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M137" s="20"/>
+      <c r="N137" s="22"/>
+      <c r="O137" s="22"/>
+      <c r="P137" s="17">
+        <f>IF(OR($A137="",$D137&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C137,$C137,$D$2:$D137,"Activo"))</f>
+      </c>
+      <c r="Q137" s="19">
+        <f>IF($P137="","",$C137&amp;"|"&amp;$P137)</f>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="20"/>
@@ -7272,6 +9530,15 @@
       <c r="L138" s="17">
         <f>IF($A138="","",IFERROR(VLOOKUP($C138,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M138" s="20"/>
+      <c r="N138" s="22"/>
+      <c r="O138" s="22"/>
+      <c r="P138" s="17">
+        <f>IF(OR($A138="",$D138&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C138,$C138,$D$2:$D138,"Activo"))</f>
+      </c>
+      <c r="Q138" s="19">
+        <f>IF($P138="","",$C138&amp;"|"&amp;$P138)</f>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="20"/>
@@ -7300,6 +9567,15 @@
       <c r="L139" s="17">
         <f>IF($A139="","",IFERROR(VLOOKUP($C139,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M139" s="20"/>
+      <c r="N139" s="22"/>
+      <c r="O139" s="22"/>
+      <c r="P139" s="17">
+        <f>IF(OR($A139="",$D139&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C139,$C139,$D$2:$D139,"Activo"))</f>
+      </c>
+      <c r="Q139" s="19">
+        <f>IF($P139="","",$C139&amp;"|"&amp;$P139)</f>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="20"/>
@@ -7328,6 +9604,15 @@
       <c r="L140" s="17">
         <f>IF($A140="","",IFERROR(VLOOKUP($C140,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M140" s="20"/>
+      <c r="N140" s="22"/>
+      <c r="O140" s="22"/>
+      <c r="P140" s="17">
+        <f>IF(OR($A140="",$D140&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C140,$C140,$D$2:$D140,"Activo"))</f>
+      </c>
+      <c r="Q140" s="19">
+        <f>IF($P140="","",$C140&amp;"|"&amp;$P140)</f>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="20"/>
@@ -7356,6 +9641,15 @@
       <c r="L141" s="17">
         <f>IF($A141="","",IFERROR(VLOOKUP($C141,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M141" s="20"/>
+      <c r="N141" s="22"/>
+      <c r="O141" s="22"/>
+      <c r="P141" s="17">
+        <f>IF(OR($A141="",$D141&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C141,$C141,$D$2:$D141,"Activo"))</f>
+      </c>
+      <c r="Q141" s="19">
+        <f>IF($P141="","",$C141&amp;"|"&amp;$P141)</f>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="20"/>
@@ -7384,6 +9678,15 @@
       <c r="L142" s="17">
         <f>IF($A142="","",IFERROR(VLOOKUP($C142,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M142" s="20"/>
+      <c r="N142" s="22"/>
+      <c r="O142" s="22"/>
+      <c r="P142" s="17">
+        <f>IF(OR($A142="",$D142&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C142,$C142,$D$2:$D142,"Activo"))</f>
+      </c>
+      <c r="Q142" s="19">
+        <f>IF($P142="","",$C142&amp;"|"&amp;$P142)</f>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="20"/>
@@ -7412,6 +9715,15 @@
       <c r="L143" s="17">
         <f>IF($A143="","",IFERROR(VLOOKUP($C143,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M143" s="20"/>
+      <c r="N143" s="22"/>
+      <c r="O143" s="22"/>
+      <c r="P143" s="17">
+        <f>IF(OR($A143="",$D143&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C143,$C143,$D$2:$D143,"Activo"))</f>
+      </c>
+      <c r="Q143" s="19">
+        <f>IF($P143="","",$C143&amp;"|"&amp;$P143)</f>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="20"/>
@@ -7440,6 +9752,15 @@
       <c r="L144" s="17">
         <f>IF($A144="","",IFERROR(VLOOKUP($C144,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M144" s="20"/>
+      <c r="N144" s="22"/>
+      <c r="O144" s="22"/>
+      <c r="P144" s="17">
+        <f>IF(OR($A144="",$D144&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C144,$C144,$D$2:$D144,"Activo"))</f>
+      </c>
+      <c r="Q144" s="19">
+        <f>IF($P144="","",$C144&amp;"|"&amp;$P144)</f>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="20"/>
@@ -7468,6 +9789,15 @@
       <c r="L145" s="17">
         <f>IF($A145="","",IFERROR(VLOOKUP($C145,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M145" s="20"/>
+      <c r="N145" s="22"/>
+      <c r="O145" s="22"/>
+      <c r="P145" s="17">
+        <f>IF(OR($A145="",$D145&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C145,$C145,$D$2:$D145,"Activo"))</f>
+      </c>
+      <c r="Q145" s="19">
+        <f>IF($P145="","",$C145&amp;"|"&amp;$P145)</f>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="20"/>
@@ -7496,6 +9826,15 @@
       <c r="L146" s="17">
         <f>IF($A146="","",IFERROR(VLOOKUP($C146,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M146" s="20"/>
+      <c r="N146" s="22"/>
+      <c r="O146" s="22"/>
+      <c r="P146" s="17">
+        <f>IF(OR($A146="",$D146&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C146,$C146,$D$2:$D146,"Activo"))</f>
+      </c>
+      <c r="Q146" s="19">
+        <f>IF($P146="","",$C146&amp;"|"&amp;$P146)</f>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="20"/>
@@ -7524,6 +9863,15 @@
       <c r="L147" s="17">
         <f>IF($A147="","",IFERROR(VLOOKUP($C147,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M147" s="20"/>
+      <c r="N147" s="22"/>
+      <c r="O147" s="22"/>
+      <c r="P147" s="17">
+        <f>IF(OR($A147="",$D147&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C147,$C147,$D$2:$D147,"Activo"))</f>
+      </c>
+      <c r="Q147" s="19">
+        <f>IF($P147="","",$C147&amp;"|"&amp;$P147)</f>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="20"/>
@@ -7552,6 +9900,15 @@
       <c r="L148" s="17">
         <f>IF($A148="","",IFERROR(VLOOKUP($C148,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M148" s="20"/>
+      <c r="N148" s="22"/>
+      <c r="O148" s="22"/>
+      <c r="P148" s="17">
+        <f>IF(OR($A148="",$D148&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C148,$C148,$D$2:$D148,"Activo"))</f>
+      </c>
+      <c r="Q148" s="19">
+        <f>IF($P148="","",$C148&amp;"|"&amp;$P148)</f>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="20"/>
@@ -7580,6 +9937,15 @@
       <c r="L149" s="17">
         <f>IF($A149="","",IFERROR(VLOOKUP($C149,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M149" s="20"/>
+      <c r="N149" s="22"/>
+      <c r="O149" s="22"/>
+      <c r="P149" s="17">
+        <f>IF(OR($A149="",$D149&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C149,$C149,$D$2:$D149,"Activo"))</f>
+      </c>
+      <c r="Q149" s="19">
+        <f>IF($P149="","",$C149&amp;"|"&amp;$P149)</f>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="20"/>
@@ -7608,6 +9974,15 @@
       <c r="L150" s="17">
         <f>IF($A150="","",IFERROR(VLOOKUP($C150,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M150" s="20"/>
+      <c r="N150" s="22"/>
+      <c r="O150" s="22"/>
+      <c r="P150" s="17">
+        <f>IF(OR($A150="",$D150&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C150,$C150,$D$2:$D150,"Activo"))</f>
+      </c>
+      <c r="Q150" s="19">
+        <f>IF($P150="","",$C150&amp;"|"&amp;$P150)</f>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="20"/>
@@ -7636,6 +10011,15 @@
       <c r="L151" s="17">
         <f>IF($A151="","",IFERROR(VLOOKUP($C151,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M151" s="20"/>
+      <c r="N151" s="22"/>
+      <c r="O151" s="22"/>
+      <c r="P151" s="17">
+        <f>IF(OR($A151="",$D151&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C151,$C151,$D$2:$D151,"Activo"))</f>
+      </c>
+      <c r="Q151" s="19">
+        <f>IF($P151="","",$C151&amp;"|"&amp;$P151)</f>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="20"/>
@@ -7664,6 +10048,15 @@
       <c r="L152" s="17">
         <f>IF($A152="","",IFERROR(VLOOKUP($C152,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M152" s="20"/>
+      <c r="N152" s="22"/>
+      <c r="O152" s="22"/>
+      <c r="P152" s="17">
+        <f>IF(OR($A152="",$D152&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C152,$C152,$D$2:$D152,"Activo"))</f>
+      </c>
+      <c r="Q152" s="19">
+        <f>IF($P152="","",$C152&amp;"|"&amp;$P152)</f>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="20"/>
@@ -7692,6 +10085,15 @@
       <c r="L153" s="17">
         <f>IF($A153="","",IFERROR(VLOOKUP($C153,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M153" s="20"/>
+      <c r="N153" s="22"/>
+      <c r="O153" s="22"/>
+      <c r="P153" s="17">
+        <f>IF(OR($A153="",$D153&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C153,$C153,$D$2:$D153,"Activo"))</f>
+      </c>
+      <c r="Q153" s="19">
+        <f>IF($P153="","",$C153&amp;"|"&amp;$P153)</f>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="20"/>
@@ -7720,6 +10122,15 @@
       <c r="L154" s="17">
         <f>IF($A154="","",IFERROR(VLOOKUP($C154,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M154" s="20"/>
+      <c r="N154" s="22"/>
+      <c r="O154" s="22"/>
+      <c r="P154" s="17">
+        <f>IF(OR($A154="",$D154&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C154,$C154,$D$2:$D154,"Activo"))</f>
+      </c>
+      <c r="Q154" s="19">
+        <f>IF($P154="","",$C154&amp;"|"&amp;$P154)</f>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="20"/>
@@ -7748,6 +10159,15 @@
       <c r="L155" s="17">
         <f>IF($A155="","",IFERROR(VLOOKUP($C155,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M155" s="20"/>
+      <c r="N155" s="22"/>
+      <c r="O155" s="22"/>
+      <c r="P155" s="17">
+        <f>IF(OR($A155="",$D155&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C155,$C155,$D$2:$D155,"Activo"))</f>
+      </c>
+      <c r="Q155" s="19">
+        <f>IF($P155="","",$C155&amp;"|"&amp;$P155)</f>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="20"/>
@@ -7776,6 +10196,15 @@
       <c r="L156" s="17">
         <f>IF($A156="","",IFERROR(VLOOKUP($C156,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M156" s="20"/>
+      <c r="N156" s="22"/>
+      <c r="O156" s="22"/>
+      <c r="P156" s="17">
+        <f>IF(OR($A156="",$D156&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C156,$C156,$D$2:$D156,"Activo"))</f>
+      </c>
+      <c r="Q156" s="19">
+        <f>IF($P156="","",$C156&amp;"|"&amp;$P156)</f>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="20"/>
@@ -7804,6 +10233,15 @@
       <c r="L157" s="17">
         <f>IF($A157="","",IFERROR(VLOOKUP($C157,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M157" s="20"/>
+      <c r="N157" s="22"/>
+      <c r="O157" s="22"/>
+      <c r="P157" s="17">
+        <f>IF(OR($A157="",$D157&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C157,$C157,$D$2:$D157,"Activo"))</f>
+      </c>
+      <c r="Q157" s="19">
+        <f>IF($P157="","",$C157&amp;"|"&amp;$P157)</f>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="20"/>
@@ -7832,6 +10270,15 @@
       <c r="L158" s="17">
         <f>IF($A158="","",IFERROR(VLOOKUP($C158,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M158" s="20"/>
+      <c r="N158" s="22"/>
+      <c r="O158" s="22"/>
+      <c r="P158" s="17">
+        <f>IF(OR($A158="",$D158&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C158,$C158,$D$2:$D158,"Activo"))</f>
+      </c>
+      <c r="Q158" s="19">
+        <f>IF($P158="","",$C158&amp;"|"&amp;$P158)</f>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="20"/>
@@ -7860,6 +10307,15 @@
       <c r="L159" s="17">
         <f>IF($A159="","",IFERROR(VLOOKUP($C159,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M159" s="20"/>
+      <c r="N159" s="22"/>
+      <c r="O159" s="22"/>
+      <c r="P159" s="17">
+        <f>IF(OR($A159="",$D159&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C159,$C159,$D$2:$D159,"Activo"))</f>
+      </c>
+      <c r="Q159" s="19">
+        <f>IF($P159="","",$C159&amp;"|"&amp;$P159)</f>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="20"/>
@@ -7888,6 +10344,15 @@
       <c r="L160" s="17">
         <f>IF($A160="","",IFERROR(VLOOKUP($C160,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M160" s="20"/>
+      <c r="N160" s="22"/>
+      <c r="O160" s="22"/>
+      <c r="P160" s="17">
+        <f>IF(OR($A160="",$D160&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C160,$C160,$D$2:$D160,"Activo"))</f>
+      </c>
+      <c r="Q160" s="19">
+        <f>IF($P160="","",$C160&amp;"|"&amp;$P160)</f>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="20"/>
@@ -7916,6 +10381,15 @@
       <c r="L161" s="17">
         <f>IF($A161="","",IFERROR(VLOOKUP($C161,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M161" s="20"/>
+      <c r="N161" s="22"/>
+      <c r="O161" s="22"/>
+      <c r="P161" s="17">
+        <f>IF(OR($A161="",$D161&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C161,$C161,$D$2:$D161,"Activo"))</f>
+      </c>
+      <c r="Q161" s="19">
+        <f>IF($P161="","",$C161&amp;"|"&amp;$P161)</f>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="20"/>
@@ -7944,6 +10418,15 @@
       <c r="L162" s="17">
         <f>IF($A162="","",IFERROR(VLOOKUP($C162,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M162" s="20"/>
+      <c r="N162" s="22"/>
+      <c r="O162" s="22"/>
+      <c r="P162" s="17">
+        <f>IF(OR($A162="",$D162&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C162,$C162,$D$2:$D162,"Activo"))</f>
+      </c>
+      <c r="Q162" s="19">
+        <f>IF($P162="","",$C162&amp;"|"&amp;$P162)</f>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="20"/>
@@ -7972,6 +10455,15 @@
       <c r="L163" s="17">
         <f>IF($A163="","",IFERROR(VLOOKUP($C163,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M163" s="20"/>
+      <c r="N163" s="22"/>
+      <c r="O163" s="22"/>
+      <c r="P163" s="17">
+        <f>IF(OR($A163="",$D163&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C163,$C163,$D$2:$D163,"Activo"))</f>
+      </c>
+      <c r="Q163" s="19">
+        <f>IF($P163="","",$C163&amp;"|"&amp;$P163)</f>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="20"/>
@@ -8000,6 +10492,15 @@
       <c r="L164" s="17">
         <f>IF($A164="","",IFERROR(VLOOKUP($C164,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M164" s="20"/>
+      <c r="N164" s="22"/>
+      <c r="O164" s="22"/>
+      <c r="P164" s="17">
+        <f>IF(OR($A164="",$D164&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C164,$C164,$D$2:$D164,"Activo"))</f>
+      </c>
+      <c r="Q164" s="19">
+        <f>IF($P164="","",$C164&amp;"|"&amp;$P164)</f>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="20"/>
@@ -8028,6 +10529,15 @@
       <c r="L165" s="17">
         <f>IF($A165="","",IFERROR(VLOOKUP($C165,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M165" s="20"/>
+      <c r="N165" s="22"/>
+      <c r="O165" s="22"/>
+      <c r="P165" s="17">
+        <f>IF(OR($A165="",$D165&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C165,$C165,$D$2:$D165,"Activo"))</f>
+      </c>
+      <c r="Q165" s="19">
+        <f>IF($P165="","",$C165&amp;"|"&amp;$P165)</f>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="20"/>
@@ -8056,6 +10566,15 @@
       <c r="L166" s="17">
         <f>IF($A166="","",IFERROR(VLOOKUP($C166,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M166" s="20"/>
+      <c r="N166" s="22"/>
+      <c r="O166" s="22"/>
+      <c r="P166" s="17">
+        <f>IF(OR($A166="",$D166&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C166,$C166,$D$2:$D166,"Activo"))</f>
+      </c>
+      <c r="Q166" s="19">
+        <f>IF($P166="","",$C166&amp;"|"&amp;$P166)</f>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="20"/>
@@ -8084,6 +10603,15 @@
       <c r="L167" s="17">
         <f>IF($A167="","",IFERROR(VLOOKUP($C167,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M167" s="20"/>
+      <c r="N167" s="22"/>
+      <c r="O167" s="22"/>
+      <c r="P167" s="17">
+        <f>IF(OR($A167="",$D167&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C167,$C167,$D$2:$D167,"Activo"))</f>
+      </c>
+      <c r="Q167" s="19">
+        <f>IF($P167="","",$C167&amp;"|"&amp;$P167)</f>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="20"/>
@@ -8112,6 +10640,15 @@
       <c r="L168" s="17">
         <f>IF($A168="","",IFERROR(VLOOKUP($C168,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M168" s="20"/>
+      <c r="N168" s="22"/>
+      <c r="O168" s="22"/>
+      <c r="P168" s="17">
+        <f>IF(OR($A168="",$D168&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C168,$C168,$D$2:$D168,"Activo"))</f>
+      </c>
+      <c r="Q168" s="19">
+        <f>IF($P168="","",$C168&amp;"|"&amp;$P168)</f>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="20"/>
@@ -8140,6 +10677,15 @@
       <c r="L169" s="17">
         <f>IF($A169="","",IFERROR(VLOOKUP($C169,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M169" s="20"/>
+      <c r="N169" s="22"/>
+      <c r="O169" s="22"/>
+      <c r="P169" s="17">
+        <f>IF(OR($A169="",$D169&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C169,$C169,$D$2:$D169,"Activo"))</f>
+      </c>
+      <c r="Q169" s="19">
+        <f>IF($P169="","",$C169&amp;"|"&amp;$P169)</f>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="20"/>
@@ -8168,6 +10714,15 @@
       <c r="L170" s="17">
         <f>IF($A170="","",IFERROR(VLOOKUP($C170,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M170" s="20"/>
+      <c r="N170" s="22"/>
+      <c r="O170" s="22"/>
+      <c r="P170" s="17">
+        <f>IF(OR($A170="",$D170&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C170,$C170,$D$2:$D170,"Activo"))</f>
+      </c>
+      <c r="Q170" s="19">
+        <f>IF($P170="","",$C170&amp;"|"&amp;$P170)</f>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="20"/>
@@ -8196,6 +10751,15 @@
       <c r="L171" s="17">
         <f>IF($A171="","",IFERROR(VLOOKUP($C171,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M171" s="20"/>
+      <c r="N171" s="22"/>
+      <c r="O171" s="22"/>
+      <c r="P171" s="17">
+        <f>IF(OR($A171="",$D171&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C171,$C171,$D$2:$D171,"Activo"))</f>
+      </c>
+      <c r="Q171" s="19">
+        <f>IF($P171="","",$C171&amp;"|"&amp;$P171)</f>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="20"/>
@@ -8224,6 +10788,15 @@
       <c r="L172" s="17">
         <f>IF($A172="","",IFERROR(VLOOKUP($C172,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M172" s="20"/>
+      <c r="N172" s="22"/>
+      <c r="O172" s="22"/>
+      <c r="P172" s="17">
+        <f>IF(OR($A172="",$D172&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C172,$C172,$D$2:$D172,"Activo"))</f>
+      </c>
+      <c r="Q172" s="19">
+        <f>IF($P172="","",$C172&amp;"|"&amp;$P172)</f>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="20"/>
@@ -8252,6 +10825,15 @@
       <c r="L173" s="17">
         <f>IF($A173="","",IFERROR(VLOOKUP($C173,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M173" s="20"/>
+      <c r="N173" s="22"/>
+      <c r="O173" s="22"/>
+      <c r="P173" s="17">
+        <f>IF(OR($A173="",$D173&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C173,$C173,$D$2:$D173,"Activo"))</f>
+      </c>
+      <c r="Q173" s="19">
+        <f>IF($P173="","",$C173&amp;"|"&amp;$P173)</f>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="20"/>
@@ -8280,6 +10862,15 @@
       <c r="L174" s="17">
         <f>IF($A174="","",IFERROR(VLOOKUP($C174,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M174" s="20"/>
+      <c r="N174" s="22"/>
+      <c r="O174" s="22"/>
+      <c r="P174" s="17">
+        <f>IF(OR($A174="",$D174&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C174,$C174,$D$2:$D174,"Activo"))</f>
+      </c>
+      <c r="Q174" s="19">
+        <f>IF($P174="","",$C174&amp;"|"&amp;$P174)</f>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="20"/>
@@ -8308,6 +10899,15 @@
       <c r="L175" s="17">
         <f>IF($A175="","",IFERROR(VLOOKUP($C175,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M175" s="20"/>
+      <c r="N175" s="22"/>
+      <c r="O175" s="22"/>
+      <c r="P175" s="17">
+        <f>IF(OR($A175="",$D175&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C175,$C175,$D$2:$D175,"Activo"))</f>
+      </c>
+      <c r="Q175" s="19">
+        <f>IF($P175="","",$C175&amp;"|"&amp;$P175)</f>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="20"/>
@@ -8336,6 +10936,15 @@
       <c r="L176" s="17">
         <f>IF($A176="","",IFERROR(VLOOKUP($C176,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M176" s="20"/>
+      <c r="N176" s="22"/>
+      <c r="O176" s="22"/>
+      <c r="P176" s="17">
+        <f>IF(OR($A176="",$D176&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C176,$C176,$D$2:$D176,"Activo"))</f>
+      </c>
+      <c r="Q176" s="19">
+        <f>IF($P176="","",$C176&amp;"|"&amp;$P176)</f>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="20"/>
@@ -8364,6 +10973,15 @@
       <c r="L177" s="17">
         <f>IF($A177="","",IFERROR(VLOOKUP($C177,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M177" s="20"/>
+      <c r="N177" s="22"/>
+      <c r="O177" s="22"/>
+      <c r="P177" s="17">
+        <f>IF(OR($A177="",$D177&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C177,$C177,$D$2:$D177,"Activo"))</f>
+      </c>
+      <c r="Q177" s="19">
+        <f>IF($P177="","",$C177&amp;"|"&amp;$P177)</f>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="20"/>
@@ -8392,6 +11010,15 @@
       <c r="L178" s="17">
         <f>IF($A178="","",IFERROR(VLOOKUP($C178,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M178" s="20"/>
+      <c r="N178" s="22"/>
+      <c r="O178" s="22"/>
+      <c r="P178" s="17">
+        <f>IF(OR($A178="",$D178&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C178,$C178,$D$2:$D178,"Activo"))</f>
+      </c>
+      <c r="Q178" s="19">
+        <f>IF($P178="","",$C178&amp;"|"&amp;$P178)</f>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="20"/>
@@ -8420,6 +11047,15 @@
       <c r="L179" s="17">
         <f>IF($A179="","",IFERROR(VLOOKUP($C179,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M179" s="20"/>
+      <c r="N179" s="22"/>
+      <c r="O179" s="22"/>
+      <c r="P179" s="17">
+        <f>IF(OR($A179="",$D179&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C179,$C179,$D$2:$D179,"Activo"))</f>
+      </c>
+      <c r="Q179" s="19">
+        <f>IF($P179="","",$C179&amp;"|"&amp;$P179)</f>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="20"/>
@@ -8448,6 +11084,15 @@
       <c r="L180" s="17">
         <f>IF($A180="","",IFERROR(VLOOKUP($C180,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M180" s="20"/>
+      <c r="N180" s="22"/>
+      <c r="O180" s="22"/>
+      <c r="P180" s="17">
+        <f>IF(OR($A180="",$D180&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C180,$C180,$D$2:$D180,"Activo"))</f>
+      </c>
+      <c r="Q180" s="19">
+        <f>IF($P180="","",$C180&amp;"|"&amp;$P180)</f>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="20"/>
@@ -8476,6 +11121,15 @@
       <c r="L181" s="17">
         <f>IF($A181="","",IFERROR(VLOOKUP($C181,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M181" s="20"/>
+      <c r="N181" s="22"/>
+      <c r="O181" s="22"/>
+      <c r="P181" s="17">
+        <f>IF(OR($A181="",$D181&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C181,$C181,$D$2:$D181,"Activo"))</f>
+      </c>
+      <c r="Q181" s="19">
+        <f>IF($P181="","",$C181&amp;"|"&amp;$P181)</f>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="20"/>
@@ -8504,6 +11158,15 @@
       <c r="L182" s="17">
         <f>IF($A182="","",IFERROR(VLOOKUP($C182,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M182" s="20"/>
+      <c r="N182" s="22"/>
+      <c r="O182" s="22"/>
+      <c r="P182" s="17">
+        <f>IF(OR($A182="",$D182&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C182,$C182,$D$2:$D182,"Activo"))</f>
+      </c>
+      <c r="Q182" s="19">
+        <f>IF($P182="","",$C182&amp;"|"&amp;$P182)</f>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="20"/>
@@ -8532,6 +11195,15 @@
       <c r="L183" s="17">
         <f>IF($A183="","",IFERROR(VLOOKUP($C183,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M183" s="20"/>
+      <c r="N183" s="22"/>
+      <c r="O183" s="22"/>
+      <c r="P183" s="17">
+        <f>IF(OR($A183="",$D183&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C183,$C183,$D$2:$D183,"Activo"))</f>
+      </c>
+      <c r="Q183" s="19">
+        <f>IF($P183="","",$C183&amp;"|"&amp;$P183)</f>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="20"/>
@@ -8560,6 +11232,15 @@
       <c r="L184" s="17">
         <f>IF($A184="","",IFERROR(VLOOKUP($C184,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M184" s="20"/>
+      <c r="N184" s="22"/>
+      <c r="O184" s="22"/>
+      <c r="P184" s="17">
+        <f>IF(OR($A184="",$D184&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C184,$C184,$D$2:$D184,"Activo"))</f>
+      </c>
+      <c r="Q184" s="19">
+        <f>IF($P184="","",$C184&amp;"|"&amp;$P184)</f>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="20"/>
@@ -8588,6 +11269,15 @@
       <c r="L185" s="17">
         <f>IF($A185="","",IFERROR(VLOOKUP($C185,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M185" s="20"/>
+      <c r="N185" s="22"/>
+      <c r="O185" s="22"/>
+      <c r="P185" s="17">
+        <f>IF(OR($A185="",$D185&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C185,$C185,$D$2:$D185,"Activo"))</f>
+      </c>
+      <c r="Q185" s="19">
+        <f>IF($P185="","",$C185&amp;"|"&amp;$P185)</f>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="20"/>
@@ -8616,6 +11306,15 @@
       <c r="L186" s="17">
         <f>IF($A186="","",IFERROR(VLOOKUP($C186,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M186" s="20"/>
+      <c r="N186" s="22"/>
+      <c r="O186" s="22"/>
+      <c r="P186" s="17">
+        <f>IF(OR($A186="",$D186&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C186,$C186,$D$2:$D186,"Activo"))</f>
+      </c>
+      <c r="Q186" s="19">
+        <f>IF($P186="","",$C186&amp;"|"&amp;$P186)</f>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="20"/>
@@ -8644,6 +11343,15 @@
       <c r="L187" s="17">
         <f>IF($A187="","",IFERROR(VLOOKUP($C187,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M187" s="20"/>
+      <c r="N187" s="22"/>
+      <c r="O187" s="22"/>
+      <c r="P187" s="17">
+        <f>IF(OR($A187="",$D187&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C187,$C187,$D$2:$D187,"Activo"))</f>
+      </c>
+      <c r="Q187" s="19">
+        <f>IF($P187="","",$C187&amp;"|"&amp;$P187)</f>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="20"/>
@@ -8672,6 +11380,15 @@
       <c r="L188" s="17">
         <f>IF($A188="","",IFERROR(VLOOKUP($C188,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M188" s="20"/>
+      <c r="N188" s="22"/>
+      <c r="O188" s="22"/>
+      <c r="P188" s="17">
+        <f>IF(OR($A188="",$D188&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C188,$C188,$D$2:$D188,"Activo"))</f>
+      </c>
+      <c r="Q188" s="19">
+        <f>IF($P188="","",$C188&amp;"|"&amp;$P188)</f>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="20"/>
@@ -8700,6 +11417,15 @@
       <c r="L189" s="17">
         <f>IF($A189="","",IFERROR(VLOOKUP($C189,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M189" s="20"/>
+      <c r="N189" s="22"/>
+      <c r="O189" s="22"/>
+      <c r="P189" s="17">
+        <f>IF(OR($A189="",$D189&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C189,$C189,$D$2:$D189,"Activo"))</f>
+      </c>
+      <c r="Q189" s="19">
+        <f>IF($P189="","",$C189&amp;"|"&amp;$P189)</f>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="20"/>
@@ -8728,6 +11454,15 @@
       <c r="L190" s="17">
         <f>IF($A190="","",IFERROR(VLOOKUP($C190,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M190" s="20"/>
+      <c r="N190" s="22"/>
+      <c r="O190" s="22"/>
+      <c r="P190" s="17">
+        <f>IF(OR($A190="",$D190&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C190,$C190,$D$2:$D190,"Activo"))</f>
+      </c>
+      <c r="Q190" s="19">
+        <f>IF($P190="","",$C190&amp;"|"&amp;$P190)</f>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="20"/>
@@ -8756,6 +11491,15 @@
       <c r="L191" s="17">
         <f>IF($A191="","",IFERROR(VLOOKUP($C191,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M191" s="20"/>
+      <c r="N191" s="22"/>
+      <c r="O191" s="22"/>
+      <c r="P191" s="17">
+        <f>IF(OR($A191="",$D191&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C191,$C191,$D$2:$D191,"Activo"))</f>
+      </c>
+      <c r="Q191" s="19">
+        <f>IF($P191="","",$C191&amp;"|"&amp;$P191)</f>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="20"/>
@@ -8784,6 +11528,15 @@
       <c r="L192" s="17">
         <f>IF($A192="","",IFERROR(VLOOKUP($C192,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M192" s="20"/>
+      <c r="N192" s="22"/>
+      <c r="O192" s="22"/>
+      <c r="P192" s="17">
+        <f>IF(OR($A192="",$D192&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C192,$C192,$D$2:$D192,"Activo"))</f>
+      </c>
+      <c r="Q192" s="19">
+        <f>IF($P192="","",$C192&amp;"|"&amp;$P192)</f>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="20"/>
@@ -8812,6 +11565,15 @@
       <c r="L193" s="17">
         <f>IF($A193="","",IFERROR(VLOOKUP($C193,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M193" s="20"/>
+      <c r="N193" s="22"/>
+      <c r="O193" s="22"/>
+      <c r="P193" s="17">
+        <f>IF(OR($A193="",$D193&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C193,$C193,$D$2:$D193,"Activo"))</f>
+      </c>
+      <c r="Q193" s="19">
+        <f>IF($P193="","",$C193&amp;"|"&amp;$P193)</f>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="20"/>
@@ -8840,6 +11602,15 @@
       <c r="L194" s="17">
         <f>IF($A194="","",IFERROR(VLOOKUP($C194,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M194" s="20"/>
+      <c r="N194" s="22"/>
+      <c r="O194" s="22"/>
+      <c r="P194" s="17">
+        <f>IF(OR($A194="",$D194&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C194,$C194,$D$2:$D194,"Activo"))</f>
+      </c>
+      <c r="Q194" s="19">
+        <f>IF($P194="","",$C194&amp;"|"&amp;$P194)</f>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="20"/>
@@ -8868,6 +11639,15 @@
       <c r="L195" s="17">
         <f>IF($A195="","",IFERROR(VLOOKUP($C195,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M195" s="20"/>
+      <c r="N195" s="22"/>
+      <c r="O195" s="22"/>
+      <c r="P195" s="17">
+        <f>IF(OR($A195="",$D195&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C195,$C195,$D$2:$D195,"Activo"))</f>
+      </c>
+      <c r="Q195" s="19">
+        <f>IF($P195="","",$C195&amp;"|"&amp;$P195)</f>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="20"/>
@@ -8896,6 +11676,15 @@
       <c r="L196" s="17">
         <f>IF($A196="","",IFERROR(VLOOKUP($C196,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M196" s="20"/>
+      <c r="N196" s="22"/>
+      <c r="O196" s="22"/>
+      <c r="P196" s="17">
+        <f>IF(OR($A196="",$D196&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C196,$C196,$D$2:$D196,"Activo"))</f>
+      </c>
+      <c r="Q196" s="19">
+        <f>IF($P196="","",$C196&amp;"|"&amp;$P196)</f>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="20"/>
@@ -8924,6 +11713,15 @@
       <c r="L197" s="17">
         <f>IF($A197="","",IFERROR(VLOOKUP($C197,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M197" s="20"/>
+      <c r="N197" s="22"/>
+      <c r="O197" s="22"/>
+      <c r="P197" s="17">
+        <f>IF(OR($A197="",$D197&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C197,$C197,$D$2:$D197,"Activo"))</f>
+      </c>
+      <c r="Q197" s="19">
+        <f>IF($P197="","",$C197&amp;"|"&amp;$P197)</f>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="20"/>
@@ -8952,6 +11750,15 @@
       <c r="L198" s="17">
         <f>IF($A198="","",IFERROR(VLOOKUP($C198,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M198" s="20"/>
+      <c r="N198" s="22"/>
+      <c r="O198" s="22"/>
+      <c r="P198" s="17">
+        <f>IF(OR($A198="",$D198&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C198,$C198,$D$2:$D198,"Activo"))</f>
+      </c>
+      <c r="Q198" s="19">
+        <f>IF($P198="","",$C198&amp;"|"&amp;$P198)</f>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="20"/>
@@ -8980,6 +11787,15 @@
       <c r="L199" s="17">
         <f>IF($A199="","",IFERROR(VLOOKUP($C199,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M199" s="20"/>
+      <c r="N199" s="22"/>
+      <c r="O199" s="22"/>
+      <c r="P199" s="17">
+        <f>IF(OR($A199="",$D199&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C199,$C199,$D$2:$D199,"Activo"))</f>
+      </c>
+      <c r="Q199" s="19">
+        <f>IF($P199="","",$C199&amp;"|"&amp;$P199)</f>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="20"/>
@@ -9008,6 +11824,15 @@
       <c r="L200" s="17">
         <f>IF($A200="","",IFERROR(VLOOKUP($C200,'Config'!$D$2:$E$8,2,FALSE),0))</f>
       </c>
+      <c r="M200" s="20"/>
+      <c r="N200" s="22"/>
+      <c r="O200" s="22"/>
+      <c r="P200" s="17">
+        <f>IF(OR($A200="",$D200&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C200,$C200,$D$2:$D200,"Activo"))</f>
+      </c>
+      <c r="Q200" s="19">
+        <f>IF($P200="","",$C200&amp;"|"&amp;$P200)</f>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="20"/>
@@ -9035,6 +11860,15 @@
       </c>
       <c r="L201" s="17">
         <f>IF($A201="","",IFERROR(VLOOKUP($C201,'Config'!$D$2:$E$8,2,FALSE),0))</f>
+      </c>
+      <c r="M201" s="20"/>
+      <c r="N201" s="22"/>
+      <c r="O201" s="22"/>
+      <c r="P201" s="17">
+        <f>IF(OR($A201="",$D201&lt;&gt;"Activo"),"",COUNTIFS($C$2:$C201,$C201,$D$2:$D201,"Activo"))</f>
+      </c>
+      <c r="Q201" s="19">
+        <f>IF($P201="","",$C201&amp;"|"&amp;$P201)</f>
       </c>
     </row>
   </sheetData>
@@ -37439,7 +40273,7 @@
           <t xml:space="preserve">N°:</t>
         </is>
       </c>
-      <c r="E2" s="39">
+      <c r="E2" s="44">
         <f>'Config'!$B$8&amp;TEXT('Config'!$B$9,"0000")</f>
       </c>
     </row>

</xml_diff>

<commit_message>
Catalogo Venta: FILTER+SORT para mostrar todos los productos sin filas en blanco
Co-authored-by: inversionescrypto8-hash <290796894+inversionescrypto8-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/generator/Sistema_Gestion_Inventario.xlsx
+++ b/generator/Sistema_Gestion_Inventario.xlsx
@@ -3419,13 +3419,31 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D205"/>
+  <dimension ref="A1:H255"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.00" customWidth="1"/>
     <col min="2" max="2" width="30.00" customWidth="1"/>
     <col min="3" max="3" width="30.00" customWidth="1"/>
     <col min="4" max="4" width="20.00" customWidth="1"/>
+    <col min="8" max="8" width="10.00" customWidth="1" hidden="1"/>
+    <col min="9" max="9" width="10.00" customWidth="1" hidden="1"/>
+    <col min="10" max="10" width="10.00" customWidth="1" hidden="1"/>
+    <col min="11" max="11" width="10.00" customWidth="1" hidden="1"/>
+    <col min="12" max="12" width="10.00" customWidth="1" hidden="1"/>
+    <col min="13" max="13" width="10.00" customWidth="1" hidden="1"/>
+    <col min="14" max="14" width="10.00" customWidth="1" hidden="1"/>
+    <col min="15" max="15" width="10.00" customWidth="1" hidden="1"/>
+    <col min="16" max="16" width="10.00" customWidth="1" hidden="1"/>
+    <col min="17" max="17" width="10.00" customWidth="1" hidden="1"/>
+    <col min="18" max="18" width="10.00" customWidth="1" hidden="1"/>
+    <col min="19" max="19" width="10.00" customWidth="1" hidden="1"/>
+    <col min="20" max="20" width="10.00" customWidth="1" hidden="1"/>
+    <col min="21" max="21" width="10.00" customWidth="1" hidden="1"/>
+    <col min="22" max="22" width="10.00" customWidth="1" hidden="1"/>
+    <col min="23" max="23" width="10.00" customWidth="1" hidden="1"/>
+    <col min="24" max="24" width="10.00" customWidth="1" hidden="1"/>
+    <col min="25" max="25" width="10.00" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="44.00" customHeight="1">
@@ -3484,2802 +3502,3505 @@
     </row>
     <row r="6" ht="90.00" customHeight="1">
       <c r="A6" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H6="","",IFERROR(IMAGE($T6,1),""))</f>
       </c>
       <c r="B6" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H6="","",$I6)</f>
       </c>
       <c r="C6" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H6="","",IF($Y6="","Cód: "&amp;$H6,"Medidas: "&amp;$Y6&amp;"  ·  Cód: "&amp;$H6))</f>
       </c>
       <c r="D6" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;1,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H6="","",IF($D$3="Mayor",$V6,$U6))</f>
+      </c>
+      <c r="H6" s="41">
+        <f>IFERROR(SORT(FILTER('Catálogo'!$A$2:$R$2000,('Catálogo'!$A$2:$A$2000&lt;&gt;"")*('Catálogo'!$D$2:$D$2000&lt;&gt;"Inactivo")*(($B$3="TODAS")+('Catálogo'!$C$2:$C$2000=$B$3))),3,TRUE,18,TRUE,2,TRUE),"")</f>
       </c>
     </row>
     <row r="7" ht="90.00" customHeight="1">
       <c r="A7" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H7="","",IFERROR(IMAGE($T7,1),""))</f>
       </c>
       <c r="B7" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H7="","",$I7)</f>
       </c>
       <c r="C7" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H7="","",IF($Y7="","Cód: "&amp;$H7,"Medidas: "&amp;$Y7&amp;"  ·  Cód: "&amp;$H7))</f>
       </c>
       <c r="D7" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;2,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H7="","",IF($D$3="Mayor",$V7,$U7))</f>
       </c>
     </row>
     <row r="8" ht="90.00" customHeight="1">
       <c r="A8" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H8="","",IFERROR(IMAGE($T8,1),""))</f>
       </c>
       <c r="B8" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H8="","",$I8)</f>
       </c>
       <c r="C8" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H8="","",IF($Y8="","Cód: "&amp;$H8,"Medidas: "&amp;$Y8&amp;"  ·  Cód: "&amp;$H8))</f>
       </c>
       <c r="D8" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;3,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H8="","",IF($D$3="Mayor",$V8,$U8))</f>
       </c>
     </row>
     <row r="9" ht="90.00" customHeight="1">
       <c r="A9" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H9="","",IFERROR(IMAGE($T9,1),""))</f>
       </c>
       <c r="B9" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H9="","",$I9)</f>
       </c>
       <c r="C9" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H9="","",IF($Y9="","Cód: "&amp;$H9,"Medidas: "&amp;$Y9&amp;"  ·  Cód: "&amp;$H9))</f>
       </c>
       <c r="D9" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;4,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H9="","",IF($D$3="Mayor",$V9,$U9))</f>
       </c>
     </row>
     <row r="10" ht="90.00" customHeight="1">
       <c r="A10" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H10="","",IFERROR(IMAGE($T10,1),""))</f>
       </c>
       <c r="B10" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H10="","",$I10)</f>
       </c>
       <c r="C10" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H10="","",IF($Y10="","Cód: "&amp;$H10,"Medidas: "&amp;$Y10&amp;"  ·  Cód: "&amp;$H10))</f>
       </c>
       <c r="D10" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;5,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H10="","",IF($D$3="Mayor",$V10,$U10))</f>
       </c>
     </row>
     <row r="11" ht="90.00" customHeight="1">
       <c r="A11" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H11="","",IFERROR(IMAGE($T11,1),""))</f>
       </c>
       <c r="B11" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H11="","",$I11)</f>
       </c>
       <c r="C11" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H11="","",IF($Y11="","Cód: "&amp;$H11,"Medidas: "&amp;$Y11&amp;"  ·  Cód: "&amp;$H11))</f>
       </c>
       <c r="D11" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;6,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H11="","",IF($D$3="Mayor",$V11,$U11))</f>
       </c>
     </row>
     <row r="12" ht="90.00" customHeight="1">
       <c r="A12" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H12="","",IFERROR(IMAGE($T12,1),""))</f>
       </c>
       <c r="B12" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H12="","",$I12)</f>
       </c>
       <c r="C12" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H12="","",IF($Y12="","Cód: "&amp;$H12,"Medidas: "&amp;$Y12&amp;"  ·  Cód: "&amp;$H12))</f>
       </c>
       <c r="D12" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;7,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H12="","",IF($D$3="Mayor",$V12,$U12))</f>
       </c>
     </row>
     <row r="13" ht="90.00" customHeight="1">
       <c r="A13" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H13="","",IFERROR(IMAGE($T13,1),""))</f>
       </c>
       <c r="B13" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H13="","",$I13)</f>
       </c>
       <c r="C13" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H13="","",IF($Y13="","Cód: "&amp;$H13,"Medidas: "&amp;$Y13&amp;"  ·  Cód: "&amp;$H13))</f>
       </c>
       <c r="D13" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;8,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H13="","",IF($D$3="Mayor",$V13,$U13))</f>
       </c>
     </row>
     <row r="14" ht="90.00" customHeight="1">
       <c r="A14" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H14="","",IFERROR(IMAGE($T14,1),""))</f>
       </c>
       <c r="B14" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H14="","",$I14)</f>
       </c>
       <c r="C14" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H14="","",IF($Y14="","Cód: "&amp;$H14,"Medidas: "&amp;$Y14&amp;"  ·  Cód: "&amp;$H14))</f>
       </c>
       <c r="D14" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;9,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H14="","",IF($D$3="Mayor",$V14,$U14))</f>
       </c>
     </row>
     <row r="15" ht="90.00" customHeight="1">
       <c r="A15" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H15="","",IFERROR(IMAGE($T15,1),""))</f>
       </c>
       <c r="B15" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H15="","",$I15)</f>
       </c>
       <c r="C15" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H15="","",IF($Y15="","Cód: "&amp;$H15,"Medidas: "&amp;$Y15&amp;"  ·  Cód: "&amp;$H15))</f>
       </c>
       <c r="D15" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;10,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H15="","",IF($D$3="Mayor",$V15,$U15))</f>
       </c>
     </row>
     <row r="16" ht="90.00" customHeight="1">
       <c r="A16" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H16="","",IFERROR(IMAGE($T16,1),""))</f>
       </c>
       <c r="B16" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H16="","",$I16)</f>
       </c>
       <c r="C16" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H16="","",IF($Y16="","Cód: "&amp;$H16,"Medidas: "&amp;$Y16&amp;"  ·  Cód: "&amp;$H16))</f>
       </c>
       <c r="D16" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;11,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H16="","",IF($D$3="Mayor",$V16,$U16))</f>
       </c>
     </row>
     <row r="17" ht="90.00" customHeight="1">
       <c r="A17" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H17="","",IFERROR(IMAGE($T17,1),""))</f>
       </c>
       <c r="B17" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H17="","",$I17)</f>
       </c>
       <c r="C17" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H17="","",IF($Y17="","Cód: "&amp;$H17,"Medidas: "&amp;$Y17&amp;"  ·  Cód: "&amp;$H17))</f>
       </c>
       <c r="D17" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;12,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H17="","",IF($D$3="Mayor",$V17,$U17))</f>
       </c>
     </row>
     <row r="18" ht="90.00" customHeight="1">
       <c r="A18" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H18="","",IFERROR(IMAGE($T18,1),""))</f>
       </c>
       <c r="B18" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H18="","",$I18)</f>
       </c>
       <c r="C18" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H18="","",IF($Y18="","Cód: "&amp;$H18,"Medidas: "&amp;$Y18&amp;"  ·  Cód: "&amp;$H18))</f>
       </c>
       <c r="D18" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;13,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H18="","",IF($D$3="Mayor",$V18,$U18))</f>
       </c>
     </row>
     <row r="19" ht="90.00" customHeight="1">
       <c r="A19" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H19="","",IFERROR(IMAGE($T19,1),""))</f>
       </c>
       <c r="B19" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H19="","",$I19)</f>
       </c>
       <c r="C19" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H19="","",IF($Y19="","Cód: "&amp;$H19,"Medidas: "&amp;$Y19&amp;"  ·  Cód: "&amp;$H19))</f>
       </c>
       <c r="D19" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;14,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H19="","",IF($D$3="Mayor",$V19,$U19))</f>
       </c>
     </row>
     <row r="20" ht="90.00" customHeight="1">
       <c r="A20" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H20="","",IFERROR(IMAGE($T20,1),""))</f>
       </c>
       <c r="B20" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H20="","",$I20)</f>
       </c>
       <c r="C20" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H20="","",IF($Y20="","Cód: "&amp;$H20,"Medidas: "&amp;$Y20&amp;"  ·  Cód: "&amp;$H20))</f>
       </c>
       <c r="D20" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;15,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H20="","",IF($D$3="Mayor",$V20,$U20))</f>
       </c>
     </row>
     <row r="21" ht="90.00" customHeight="1">
       <c r="A21" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H21="","",IFERROR(IMAGE($T21,1),""))</f>
       </c>
       <c r="B21" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H21="","",$I21)</f>
       </c>
       <c r="C21" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H21="","",IF($Y21="","Cód: "&amp;$H21,"Medidas: "&amp;$Y21&amp;"  ·  Cód: "&amp;$H21))</f>
       </c>
       <c r="D21" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;16,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H21="","",IF($D$3="Mayor",$V21,$U21))</f>
       </c>
     </row>
     <row r="22" ht="90.00" customHeight="1">
       <c r="A22" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H22="","",IFERROR(IMAGE($T22,1),""))</f>
       </c>
       <c r="B22" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H22="","",$I22)</f>
       </c>
       <c r="C22" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H22="","",IF($Y22="","Cód: "&amp;$H22,"Medidas: "&amp;$Y22&amp;"  ·  Cód: "&amp;$H22))</f>
       </c>
       <c r="D22" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;17,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H22="","",IF($D$3="Mayor",$V22,$U22))</f>
       </c>
     </row>
     <row r="23" ht="90.00" customHeight="1">
       <c r="A23" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H23="","",IFERROR(IMAGE($T23,1),""))</f>
       </c>
       <c r="B23" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H23="","",$I23)</f>
       </c>
       <c r="C23" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H23="","",IF($Y23="","Cód: "&amp;$H23,"Medidas: "&amp;$Y23&amp;"  ·  Cód: "&amp;$H23))</f>
       </c>
       <c r="D23" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;18,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H23="","",IF($D$3="Mayor",$V23,$U23))</f>
       </c>
     </row>
     <row r="24" ht="90.00" customHeight="1">
       <c r="A24" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H24="","",IFERROR(IMAGE($T24,1),""))</f>
       </c>
       <c r="B24" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H24="","",$I24)</f>
       </c>
       <c r="C24" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H24="","",IF($Y24="","Cód: "&amp;$H24,"Medidas: "&amp;$Y24&amp;"  ·  Cód: "&amp;$H24))</f>
       </c>
       <c r="D24" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;19,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H24="","",IF($D$3="Mayor",$V24,$U24))</f>
       </c>
     </row>
     <row r="25" ht="90.00" customHeight="1">
       <c r="A25" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H25="","",IFERROR(IMAGE($T25,1),""))</f>
       </c>
       <c r="B25" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H25="","",$I25)</f>
       </c>
       <c r="C25" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H25="","",IF($Y25="","Cód: "&amp;$H25,"Medidas: "&amp;$Y25&amp;"  ·  Cód: "&amp;$H25))</f>
       </c>
       <c r="D25" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;20,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H25="","",IF($D$3="Mayor",$V25,$U25))</f>
       </c>
     </row>
     <row r="26" ht="90.00" customHeight="1">
       <c r="A26" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H26="","",IFERROR(IMAGE($T26,1),""))</f>
       </c>
       <c r="B26" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H26="","",$I26)</f>
       </c>
       <c r="C26" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H26="","",IF($Y26="","Cód: "&amp;$H26,"Medidas: "&amp;$Y26&amp;"  ·  Cód: "&amp;$H26))</f>
       </c>
       <c r="D26" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;21,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H26="","",IF($D$3="Mayor",$V26,$U26))</f>
       </c>
     </row>
     <row r="27" ht="90.00" customHeight="1">
       <c r="A27" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H27="","",IFERROR(IMAGE($T27,1),""))</f>
       </c>
       <c r="B27" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H27="","",$I27)</f>
       </c>
       <c r="C27" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H27="","",IF($Y27="","Cód: "&amp;$H27,"Medidas: "&amp;$Y27&amp;"  ·  Cód: "&amp;$H27))</f>
       </c>
       <c r="D27" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;22,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H27="","",IF($D$3="Mayor",$V27,$U27))</f>
       </c>
     </row>
     <row r="28" ht="90.00" customHeight="1">
       <c r="A28" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H28="","",IFERROR(IMAGE($T28,1),""))</f>
       </c>
       <c r="B28" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H28="","",$I28)</f>
       </c>
       <c r="C28" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H28="","",IF($Y28="","Cód: "&amp;$H28,"Medidas: "&amp;$Y28&amp;"  ·  Cód: "&amp;$H28))</f>
       </c>
       <c r="D28" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;23,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H28="","",IF($D$3="Mayor",$V28,$U28))</f>
       </c>
     </row>
     <row r="29" ht="90.00" customHeight="1">
       <c r="A29" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H29="","",IFERROR(IMAGE($T29,1),""))</f>
       </c>
       <c r="B29" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H29="","",$I29)</f>
       </c>
       <c r="C29" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H29="","",IF($Y29="","Cód: "&amp;$H29,"Medidas: "&amp;$Y29&amp;"  ·  Cód: "&amp;$H29))</f>
       </c>
       <c r="D29" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;24,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H29="","",IF($D$3="Mayor",$V29,$U29))</f>
       </c>
     </row>
     <row r="30" ht="90.00" customHeight="1">
       <c r="A30" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H30="","",IFERROR(IMAGE($T30,1),""))</f>
       </c>
       <c r="B30" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H30="","",$I30)</f>
       </c>
       <c r="C30" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H30="","",IF($Y30="","Cód: "&amp;$H30,"Medidas: "&amp;$Y30&amp;"  ·  Cód: "&amp;$H30))</f>
       </c>
       <c r="D30" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;25,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H30="","",IF($D$3="Mayor",$V30,$U30))</f>
       </c>
     </row>
     <row r="31" ht="90.00" customHeight="1">
       <c r="A31" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H31="","",IFERROR(IMAGE($T31,1),""))</f>
       </c>
       <c r="B31" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H31="","",$I31)</f>
       </c>
       <c r="C31" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H31="","",IF($Y31="","Cód: "&amp;$H31,"Medidas: "&amp;$Y31&amp;"  ·  Cód: "&amp;$H31))</f>
       </c>
       <c r="D31" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;26,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H31="","",IF($D$3="Mayor",$V31,$U31))</f>
       </c>
     </row>
     <row r="32" ht="90.00" customHeight="1">
       <c r="A32" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H32="","",IFERROR(IMAGE($T32,1),""))</f>
       </c>
       <c r="B32" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H32="","",$I32)</f>
       </c>
       <c r="C32" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H32="","",IF($Y32="","Cód: "&amp;$H32,"Medidas: "&amp;$Y32&amp;"  ·  Cód: "&amp;$H32))</f>
       </c>
       <c r="D32" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;27,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H32="","",IF($D$3="Mayor",$V32,$U32))</f>
       </c>
     </row>
     <row r="33" ht="90.00" customHeight="1">
       <c r="A33" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H33="","",IFERROR(IMAGE($T33,1),""))</f>
       </c>
       <c r="B33" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H33="","",$I33)</f>
       </c>
       <c r="C33" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H33="","",IF($Y33="","Cód: "&amp;$H33,"Medidas: "&amp;$Y33&amp;"  ·  Cód: "&amp;$H33))</f>
       </c>
       <c r="D33" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;28,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H33="","",IF($D$3="Mayor",$V33,$U33))</f>
       </c>
     </row>
     <row r="34" ht="90.00" customHeight="1">
       <c r="A34" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H34="","",IFERROR(IMAGE($T34,1),""))</f>
       </c>
       <c r="B34" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H34="","",$I34)</f>
       </c>
       <c r="C34" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H34="","",IF($Y34="","Cód: "&amp;$H34,"Medidas: "&amp;$Y34&amp;"  ·  Cód: "&amp;$H34))</f>
       </c>
       <c r="D34" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;29,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H34="","",IF($D$3="Mayor",$V34,$U34))</f>
       </c>
     </row>
     <row r="35" ht="90.00" customHeight="1">
       <c r="A35" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H35="","",IFERROR(IMAGE($T35,1),""))</f>
       </c>
       <c r="B35" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H35="","",$I35)</f>
       </c>
       <c r="C35" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H35="","",IF($Y35="","Cód: "&amp;$H35,"Medidas: "&amp;$Y35&amp;"  ·  Cód: "&amp;$H35))</f>
       </c>
       <c r="D35" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;30,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H35="","",IF($D$3="Mayor",$V35,$U35))</f>
       </c>
     </row>
     <row r="36" ht="90.00" customHeight="1">
       <c r="A36" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H36="","",IFERROR(IMAGE($T36,1),""))</f>
       </c>
       <c r="B36" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H36="","",$I36)</f>
       </c>
       <c r="C36" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H36="","",IF($Y36="","Cód: "&amp;$H36,"Medidas: "&amp;$Y36&amp;"  ·  Cód: "&amp;$H36))</f>
       </c>
       <c r="D36" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;31,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H36="","",IF($D$3="Mayor",$V36,$U36))</f>
       </c>
     </row>
     <row r="37" ht="90.00" customHeight="1">
       <c r="A37" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H37="","",IFERROR(IMAGE($T37,1),""))</f>
       </c>
       <c r="B37" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H37="","",$I37)</f>
       </c>
       <c r="C37" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H37="","",IF($Y37="","Cód: "&amp;$H37,"Medidas: "&amp;$Y37&amp;"  ·  Cód: "&amp;$H37))</f>
       </c>
       <c r="D37" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;32,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H37="","",IF($D$3="Mayor",$V37,$U37))</f>
       </c>
     </row>
     <row r="38" ht="90.00" customHeight="1">
       <c r="A38" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H38="","",IFERROR(IMAGE($T38,1),""))</f>
       </c>
       <c r="B38" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H38="","",$I38)</f>
       </c>
       <c r="C38" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H38="","",IF($Y38="","Cód: "&amp;$H38,"Medidas: "&amp;$Y38&amp;"  ·  Cód: "&amp;$H38))</f>
       </c>
       <c r="D38" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;33,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H38="","",IF($D$3="Mayor",$V38,$U38))</f>
       </c>
     </row>
     <row r="39" ht="90.00" customHeight="1">
       <c r="A39" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H39="","",IFERROR(IMAGE($T39,1),""))</f>
       </c>
       <c r="B39" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H39="","",$I39)</f>
       </c>
       <c r="C39" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H39="","",IF($Y39="","Cód: "&amp;$H39,"Medidas: "&amp;$Y39&amp;"  ·  Cód: "&amp;$H39))</f>
       </c>
       <c r="D39" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;34,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H39="","",IF($D$3="Mayor",$V39,$U39))</f>
       </c>
     </row>
     <row r="40" ht="90.00" customHeight="1">
       <c r="A40" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H40="","",IFERROR(IMAGE($T40,1),""))</f>
       </c>
       <c r="B40" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H40="","",$I40)</f>
       </c>
       <c r="C40" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H40="","",IF($Y40="","Cód: "&amp;$H40,"Medidas: "&amp;$Y40&amp;"  ·  Cód: "&amp;$H40))</f>
       </c>
       <c r="D40" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;35,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H40="","",IF($D$3="Mayor",$V40,$U40))</f>
       </c>
     </row>
     <row r="41" ht="90.00" customHeight="1">
       <c r="A41" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H41="","",IFERROR(IMAGE($T41,1),""))</f>
       </c>
       <c r="B41" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H41="","",$I41)</f>
       </c>
       <c r="C41" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H41="","",IF($Y41="","Cód: "&amp;$H41,"Medidas: "&amp;$Y41&amp;"  ·  Cód: "&amp;$H41))</f>
       </c>
       <c r="D41" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;36,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H41="","",IF($D$3="Mayor",$V41,$U41))</f>
       </c>
     </row>
     <row r="42" ht="90.00" customHeight="1">
       <c r="A42" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H42="","",IFERROR(IMAGE($T42,1),""))</f>
       </c>
       <c r="B42" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H42="","",$I42)</f>
       </c>
       <c r="C42" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H42="","",IF($Y42="","Cód: "&amp;$H42,"Medidas: "&amp;$Y42&amp;"  ·  Cód: "&amp;$H42))</f>
       </c>
       <c r="D42" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;37,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H42="","",IF($D$3="Mayor",$V42,$U42))</f>
       </c>
     </row>
     <row r="43" ht="90.00" customHeight="1">
       <c r="A43" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H43="","",IFERROR(IMAGE($T43,1),""))</f>
       </c>
       <c r="B43" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H43="","",$I43)</f>
       </c>
       <c r="C43" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H43="","",IF($Y43="","Cód: "&amp;$H43,"Medidas: "&amp;$Y43&amp;"  ·  Cód: "&amp;$H43))</f>
       </c>
       <c r="D43" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;38,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H43="","",IF($D$3="Mayor",$V43,$U43))</f>
       </c>
     </row>
     <row r="44" ht="90.00" customHeight="1">
       <c r="A44" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H44="","",IFERROR(IMAGE($T44,1),""))</f>
       </c>
       <c r="B44" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H44="","",$I44)</f>
       </c>
       <c r="C44" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H44="","",IF($Y44="","Cód: "&amp;$H44,"Medidas: "&amp;$Y44&amp;"  ·  Cód: "&amp;$H44))</f>
       </c>
       <c r="D44" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;39,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H44="","",IF($D$3="Mayor",$V44,$U44))</f>
       </c>
     </row>
     <row r="45" ht="90.00" customHeight="1">
       <c r="A45" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H45="","",IFERROR(IMAGE($T45,1),""))</f>
       </c>
       <c r="B45" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H45="","",$I45)</f>
       </c>
       <c r="C45" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H45="","",IF($Y45="","Cód: "&amp;$H45,"Medidas: "&amp;$Y45&amp;"  ·  Cód: "&amp;$H45))</f>
       </c>
       <c r="D45" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;40,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H45="","",IF($D$3="Mayor",$V45,$U45))</f>
       </c>
     </row>
     <row r="46" ht="90.00" customHeight="1">
       <c r="A46" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H46="","",IFERROR(IMAGE($T46,1),""))</f>
       </c>
       <c r="B46" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H46="","",$I46)</f>
       </c>
       <c r="C46" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H46="","",IF($Y46="","Cód: "&amp;$H46,"Medidas: "&amp;$Y46&amp;"  ·  Cód: "&amp;$H46))</f>
       </c>
       <c r="D46" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;41,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H46="","",IF($D$3="Mayor",$V46,$U46))</f>
       </c>
     </row>
     <row r="47" ht="90.00" customHeight="1">
       <c r="A47" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H47="","",IFERROR(IMAGE($T47,1),""))</f>
       </c>
       <c r="B47" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H47="","",$I47)</f>
       </c>
       <c r="C47" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H47="","",IF($Y47="","Cód: "&amp;$H47,"Medidas: "&amp;$Y47&amp;"  ·  Cód: "&amp;$H47))</f>
       </c>
       <c r="D47" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;42,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H47="","",IF($D$3="Mayor",$V47,$U47))</f>
       </c>
     </row>
     <row r="48" ht="90.00" customHeight="1">
       <c r="A48" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H48="","",IFERROR(IMAGE($T48,1),""))</f>
       </c>
       <c r="B48" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H48="","",$I48)</f>
       </c>
       <c r="C48" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H48="","",IF($Y48="","Cód: "&amp;$H48,"Medidas: "&amp;$Y48&amp;"  ·  Cód: "&amp;$H48))</f>
       </c>
       <c r="D48" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;43,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H48="","",IF($D$3="Mayor",$V48,$U48))</f>
       </c>
     </row>
     <row r="49" ht="90.00" customHeight="1">
       <c r="A49" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H49="","",IFERROR(IMAGE($T49,1),""))</f>
       </c>
       <c r="B49" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H49="","",$I49)</f>
       </c>
       <c r="C49" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H49="","",IF($Y49="","Cód: "&amp;$H49,"Medidas: "&amp;$Y49&amp;"  ·  Cód: "&amp;$H49))</f>
       </c>
       <c r="D49" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;44,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H49="","",IF($D$3="Mayor",$V49,$U49))</f>
       </c>
     </row>
     <row r="50" ht="90.00" customHeight="1">
       <c r="A50" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H50="","",IFERROR(IMAGE($T50,1),""))</f>
       </c>
       <c r="B50" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H50="","",$I50)</f>
       </c>
       <c r="C50" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H50="","",IF($Y50="","Cód: "&amp;$H50,"Medidas: "&amp;$Y50&amp;"  ·  Cód: "&amp;$H50))</f>
       </c>
       <c r="D50" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;45,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H50="","",IF($D$3="Mayor",$V50,$U50))</f>
       </c>
     </row>
     <row r="51" ht="90.00" customHeight="1">
       <c r="A51" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H51="","",IFERROR(IMAGE($T51,1),""))</f>
       </c>
       <c r="B51" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H51="","",$I51)</f>
       </c>
       <c r="C51" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H51="","",IF($Y51="","Cód: "&amp;$H51,"Medidas: "&amp;$Y51&amp;"  ·  Cód: "&amp;$H51))</f>
       </c>
       <c r="D51" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;46,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H51="","",IF($D$3="Mayor",$V51,$U51))</f>
       </c>
     </row>
     <row r="52" ht="90.00" customHeight="1">
       <c r="A52" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H52="","",IFERROR(IMAGE($T52,1),""))</f>
       </c>
       <c r="B52" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H52="","",$I52)</f>
       </c>
       <c r="C52" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H52="","",IF($Y52="","Cód: "&amp;$H52,"Medidas: "&amp;$Y52&amp;"  ·  Cód: "&amp;$H52))</f>
       </c>
       <c r="D52" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;47,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H52="","",IF($D$3="Mayor",$V52,$U52))</f>
       </c>
     </row>
     <row r="53" ht="90.00" customHeight="1">
       <c r="A53" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H53="","",IFERROR(IMAGE($T53,1),""))</f>
       </c>
       <c r="B53" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H53="","",$I53)</f>
       </c>
       <c r="C53" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H53="","",IF($Y53="","Cód: "&amp;$H53,"Medidas: "&amp;$Y53&amp;"  ·  Cód: "&amp;$H53))</f>
       </c>
       <c r="D53" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;48,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H53="","",IF($D$3="Mayor",$V53,$U53))</f>
       </c>
     </row>
     <row r="54" ht="90.00" customHeight="1">
       <c r="A54" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H54="","",IFERROR(IMAGE($T54,1),""))</f>
       </c>
       <c r="B54" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H54="","",$I54)</f>
       </c>
       <c r="C54" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H54="","",IF($Y54="","Cód: "&amp;$H54,"Medidas: "&amp;$Y54&amp;"  ·  Cód: "&amp;$H54))</f>
       </c>
       <c r="D54" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;49,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H54="","",IF($D$3="Mayor",$V54,$U54))</f>
       </c>
     </row>
     <row r="55" ht="90.00" customHeight="1">
       <c r="A55" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H55="","",IFERROR(IMAGE($T55,1),""))</f>
       </c>
       <c r="B55" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H55="","",$I55)</f>
       </c>
       <c r="C55" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H55="","",IF($Y55="","Cód: "&amp;$H55,"Medidas: "&amp;$Y55&amp;"  ·  Cód: "&amp;$H55))</f>
       </c>
       <c r="D55" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;50,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H55="","",IF($D$3="Mayor",$V55,$U55))</f>
       </c>
     </row>
     <row r="56" ht="90.00" customHeight="1">
       <c r="A56" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H56="","",IFERROR(IMAGE($T56,1),""))</f>
       </c>
       <c r="B56" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H56="","",$I56)</f>
       </c>
       <c r="C56" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H56="","",IF($Y56="","Cód: "&amp;$H56,"Medidas: "&amp;$Y56&amp;"  ·  Cód: "&amp;$H56))</f>
       </c>
       <c r="D56" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;51,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H56="","",IF($D$3="Mayor",$V56,$U56))</f>
       </c>
     </row>
     <row r="57" ht="90.00" customHeight="1">
       <c r="A57" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H57="","",IFERROR(IMAGE($T57,1),""))</f>
       </c>
       <c r="B57" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H57="","",$I57)</f>
       </c>
       <c r="C57" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H57="","",IF($Y57="","Cód: "&amp;$H57,"Medidas: "&amp;$Y57&amp;"  ·  Cód: "&amp;$H57))</f>
       </c>
       <c r="D57" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;52,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H57="","",IF($D$3="Mayor",$V57,$U57))</f>
       </c>
     </row>
     <row r="58" ht="90.00" customHeight="1">
       <c r="A58" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H58="","",IFERROR(IMAGE($T58,1),""))</f>
       </c>
       <c r="B58" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H58="","",$I58)</f>
       </c>
       <c r="C58" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H58="","",IF($Y58="","Cód: "&amp;$H58,"Medidas: "&amp;$Y58&amp;"  ·  Cód: "&amp;$H58))</f>
       </c>
       <c r="D58" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;53,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H58="","",IF($D$3="Mayor",$V58,$U58))</f>
       </c>
     </row>
     <row r="59" ht="90.00" customHeight="1">
       <c r="A59" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H59="","",IFERROR(IMAGE($T59,1),""))</f>
       </c>
       <c r="B59" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H59="","",$I59)</f>
       </c>
       <c r="C59" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H59="","",IF($Y59="","Cód: "&amp;$H59,"Medidas: "&amp;$Y59&amp;"  ·  Cód: "&amp;$H59))</f>
       </c>
       <c r="D59" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;54,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H59="","",IF($D$3="Mayor",$V59,$U59))</f>
       </c>
     </row>
     <row r="60" ht="90.00" customHeight="1">
       <c r="A60" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H60="","",IFERROR(IMAGE($T60,1),""))</f>
       </c>
       <c r="B60" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H60="","",$I60)</f>
       </c>
       <c r="C60" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H60="","",IF($Y60="","Cód: "&amp;$H60,"Medidas: "&amp;$Y60&amp;"  ·  Cód: "&amp;$H60))</f>
       </c>
       <c r="D60" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;55,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H60="","",IF($D$3="Mayor",$V60,$U60))</f>
       </c>
     </row>
     <row r="61" ht="90.00" customHeight="1">
       <c r="A61" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H61="","",IFERROR(IMAGE($T61,1),""))</f>
       </c>
       <c r="B61" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H61="","",$I61)</f>
       </c>
       <c r="C61" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H61="","",IF($Y61="","Cód: "&amp;$H61,"Medidas: "&amp;$Y61&amp;"  ·  Cód: "&amp;$H61))</f>
       </c>
       <c r="D61" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;56,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H61="","",IF($D$3="Mayor",$V61,$U61))</f>
       </c>
     </row>
     <row r="62" ht="90.00" customHeight="1">
       <c r="A62" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H62="","",IFERROR(IMAGE($T62,1),""))</f>
       </c>
       <c r="B62" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H62="","",$I62)</f>
       </c>
       <c r="C62" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H62="","",IF($Y62="","Cód: "&amp;$H62,"Medidas: "&amp;$Y62&amp;"  ·  Cód: "&amp;$H62))</f>
       </c>
       <c r="D62" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;57,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H62="","",IF($D$3="Mayor",$V62,$U62))</f>
       </c>
     </row>
     <row r="63" ht="90.00" customHeight="1">
       <c r="A63" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H63="","",IFERROR(IMAGE($T63,1),""))</f>
       </c>
       <c r="B63" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H63="","",$I63)</f>
       </c>
       <c r="C63" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H63="","",IF($Y63="","Cód: "&amp;$H63,"Medidas: "&amp;$Y63&amp;"  ·  Cód: "&amp;$H63))</f>
       </c>
       <c r="D63" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;58,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H63="","",IF($D$3="Mayor",$V63,$U63))</f>
       </c>
     </row>
     <row r="64" ht="90.00" customHeight="1">
       <c r="A64" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H64="","",IFERROR(IMAGE($T64,1),""))</f>
       </c>
       <c r="B64" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H64="","",$I64)</f>
       </c>
       <c r="C64" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H64="","",IF($Y64="","Cód: "&amp;$H64,"Medidas: "&amp;$Y64&amp;"  ·  Cód: "&amp;$H64))</f>
       </c>
       <c r="D64" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;59,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H64="","",IF($D$3="Mayor",$V64,$U64))</f>
       </c>
     </row>
     <row r="65" ht="90.00" customHeight="1">
       <c r="A65" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H65="","",IFERROR(IMAGE($T65,1),""))</f>
       </c>
       <c r="B65" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H65="","",$I65)</f>
       </c>
       <c r="C65" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H65="","",IF($Y65="","Cód: "&amp;$H65,"Medidas: "&amp;$Y65&amp;"  ·  Cód: "&amp;$H65))</f>
       </c>
       <c r="D65" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;60,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H65="","",IF($D$3="Mayor",$V65,$U65))</f>
       </c>
     </row>
     <row r="66" ht="90.00" customHeight="1">
       <c r="A66" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H66="","",IFERROR(IMAGE($T66,1),""))</f>
       </c>
       <c r="B66" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H66="","",$I66)</f>
       </c>
       <c r="C66" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H66="","",IF($Y66="","Cód: "&amp;$H66,"Medidas: "&amp;$Y66&amp;"  ·  Cód: "&amp;$H66))</f>
       </c>
       <c r="D66" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;61,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H66="","",IF($D$3="Mayor",$V66,$U66))</f>
       </c>
     </row>
     <row r="67" ht="90.00" customHeight="1">
       <c r="A67" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H67="","",IFERROR(IMAGE($T67,1),""))</f>
       </c>
       <c r="B67" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H67="","",$I67)</f>
       </c>
       <c r="C67" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H67="","",IF($Y67="","Cód: "&amp;$H67,"Medidas: "&amp;$Y67&amp;"  ·  Cód: "&amp;$H67))</f>
       </c>
       <c r="D67" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;62,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H67="","",IF($D$3="Mayor",$V67,$U67))</f>
       </c>
     </row>
     <row r="68" ht="90.00" customHeight="1">
       <c r="A68" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H68="","",IFERROR(IMAGE($T68,1),""))</f>
       </c>
       <c r="B68" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H68="","",$I68)</f>
       </c>
       <c r="C68" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H68="","",IF($Y68="","Cód: "&amp;$H68,"Medidas: "&amp;$Y68&amp;"  ·  Cód: "&amp;$H68))</f>
       </c>
       <c r="D68" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;63,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H68="","",IF($D$3="Mayor",$V68,$U68))</f>
       </c>
     </row>
     <row r="69" ht="90.00" customHeight="1">
       <c r="A69" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H69="","",IFERROR(IMAGE($T69,1),""))</f>
       </c>
       <c r="B69" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H69="","",$I69)</f>
       </c>
       <c r="C69" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H69="","",IF($Y69="","Cód: "&amp;$H69,"Medidas: "&amp;$Y69&amp;"  ·  Cód: "&amp;$H69))</f>
       </c>
       <c r="D69" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;64,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H69="","",IF($D$3="Mayor",$V69,$U69))</f>
       </c>
     </row>
     <row r="70" ht="90.00" customHeight="1">
       <c r="A70" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H70="","",IFERROR(IMAGE($T70,1),""))</f>
       </c>
       <c r="B70" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H70="","",$I70)</f>
       </c>
       <c r="C70" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H70="","",IF($Y70="","Cód: "&amp;$H70,"Medidas: "&amp;$Y70&amp;"  ·  Cód: "&amp;$H70))</f>
       </c>
       <c r="D70" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;65,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H70="","",IF($D$3="Mayor",$V70,$U70))</f>
       </c>
     </row>
     <row r="71" ht="90.00" customHeight="1">
       <c r="A71" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H71="","",IFERROR(IMAGE($T71,1),""))</f>
       </c>
       <c r="B71" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H71="","",$I71)</f>
       </c>
       <c r="C71" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H71="","",IF($Y71="","Cód: "&amp;$H71,"Medidas: "&amp;$Y71&amp;"  ·  Cód: "&amp;$H71))</f>
       </c>
       <c r="D71" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;66,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H71="","",IF($D$3="Mayor",$V71,$U71))</f>
       </c>
     </row>
     <row r="72" ht="90.00" customHeight="1">
       <c r="A72" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H72="","",IFERROR(IMAGE($T72,1),""))</f>
       </c>
       <c r="B72" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H72="","",$I72)</f>
       </c>
       <c r="C72" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H72="","",IF($Y72="","Cód: "&amp;$H72,"Medidas: "&amp;$Y72&amp;"  ·  Cód: "&amp;$H72))</f>
       </c>
       <c r="D72" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;67,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H72="","",IF($D$3="Mayor",$V72,$U72))</f>
       </c>
     </row>
     <row r="73" ht="90.00" customHeight="1">
       <c r="A73" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H73="","",IFERROR(IMAGE($T73,1),""))</f>
       </c>
       <c r="B73" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H73="","",$I73)</f>
       </c>
       <c r="C73" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H73="","",IF($Y73="","Cód: "&amp;$H73,"Medidas: "&amp;$Y73&amp;"  ·  Cód: "&amp;$H73))</f>
       </c>
       <c r="D73" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;68,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H73="","",IF($D$3="Mayor",$V73,$U73))</f>
       </c>
     </row>
     <row r="74" ht="90.00" customHeight="1">
       <c r="A74" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H74="","",IFERROR(IMAGE($T74,1),""))</f>
       </c>
       <c r="B74" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H74="","",$I74)</f>
       </c>
       <c r="C74" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H74="","",IF($Y74="","Cód: "&amp;$H74,"Medidas: "&amp;$Y74&amp;"  ·  Cód: "&amp;$H74))</f>
       </c>
       <c r="D74" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;69,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H74="","",IF($D$3="Mayor",$V74,$U74))</f>
       </c>
     </row>
     <row r="75" ht="90.00" customHeight="1">
       <c r="A75" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H75="","",IFERROR(IMAGE($T75,1),""))</f>
       </c>
       <c r="B75" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H75="","",$I75)</f>
       </c>
       <c r="C75" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H75="","",IF($Y75="","Cód: "&amp;$H75,"Medidas: "&amp;$Y75&amp;"  ·  Cód: "&amp;$H75))</f>
       </c>
       <c r="D75" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;70,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H75="","",IF($D$3="Mayor",$V75,$U75))</f>
       </c>
     </row>
     <row r="76" ht="90.00" customHeight="1">
       <c r="A76" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H76="","",IFERROR(IMAGE($T76,1),""))</f>
       </c>
       <c r="B76" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H76="","",$I76)</f>
       </c>
       <c r="C76" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H76="","",IF($Y76="","Cód: "&amp;$H76,"Medidas: "&amp;$Y76&amp;"  ·  Cód: "&amp;$H76))</f>
       </c>
       <c r="D76" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;71,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H76="","",IF($D$3="Mayor",$V76,$U76))</f>
       </c>
     </row>
     <row r="77" ht="90.00" customHeight="1">
       <c r="A77" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H77="","",IFERROR(IMAGE($T77,1),""))</f>
       </c>
       <c r="B77" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H77="","",$I77)</f>
       </c>
       <c r="C77" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H77="","",IF($Y77="","Cód: "&amp;$H77,"Medidas: "&amp;$Y77&amp;"  ·  Cód: "&amp;$H77))</f>
       </c>
       <c r="D77" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;72,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H77="","",IF($D$3="Mayor",$V77,$U77))</f>
       </c>
     </row>
     <row r="78" ht="90.00" customHeight="1">
       <c r="A78" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H78="","",IFERROR(IMAGE($T78,1),""))</f>
       </c>
       <c r="B78" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H78="","",$I78)</f>
       </c>
       <c r="C78" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H78="","",IF($Y78="","Cód: "&amp;$H78,"Medidas: "&amp;$Y78&amp;"  ·  Cód: "&amp;$H78))</f>
       </c>
       <c r="D78" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;73,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H78="","",IF($D$3="Mayor",$V78,$U78))</f>
       </c>
     </row>
     <row r="79" ht="90.00" customHeight="1">
       <c r="A79" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H79="","",IFERROR(IMAGE($T79,1),""))</f>
       </c>
       <c r="B79" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H79="","",$I79)</f>
       </c>
       <c r="C79" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H79="","",IF($Y79="","Cód: "&amp;$H79,"Medidas: "&amp;$Y79&amp;"  ·  Cód: "&amp;$H79))</f>
       </c>
       <c r="D79" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;74,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H79="","",IF($D$3="Mayor",$V79,$U79))</f>
       </c>
     </row>
     <row r="80" ht="90.00" customHeight="1">
       <c r="A80" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H80="","",IFERROR(IMAGE($T80,1),""))</f>
       </c>
       <c r="B80" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H80="","",$I80)</f>
       </c>
       <c r="C80" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H80="","",IF($Y80="","Cód: "&amp;$H80,"Medidas: "&amp;$Y80&amp;"  ·  Cód: "&amp;$H80))</f>
       </c>
       <c r="D80" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;75,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H80="","",IF($D$3="Mayor",$V80,$U80))</f>
       </c>
     </row>
     <row r="81" ht="90.00" customHeight="1">
       <c r="A81" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H81="","",IFERROR(IMAGE($T81,1),""))</f>
       </c>
       <c r="B81" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H81="","",$I81)</f>
       </c>
       <c r="C81" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H81="","",IF($Y81="","Cód: "&amp;$H81,"Medidas: "&amp;$Y81&amp;"  ·  Cód: "&amp;$H81))</f>
       </c>
       <c r="D81" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;76,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H81="","",IF($D$3="Mayor",$V81,$U81))</f>
       </c>
     </row>
     <row r="82" ht="90.00" customHeight="1">
       <c r="A82" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H82="","",IFERROR(IMAGE($T82,1),""))</f>
       </c>
       <c r="B82" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H82="","",$I82)</f>
       </c>
       <c r="C82" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H82="","",IF($Y82="","Cód: "&amp;$H82,"Medidas: "&amp;$Y82&amp;"  ·  Cód: "&amp;$H82))</f>
       </c>
       <c r="D82" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;77,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H82="","",IF($D$3="Mayor",$V82,$U82))</f>
       </c>
     </row>
     <row r="83" ht="90.00" customHeight="1">
       <c r="A83" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H83="","",IFERROR(IMAGE($T83,1),""))</f>
       </c>
       <c r="B83" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H83="","",$I83)</f>
       </c>
       <c r="C83" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H83="","",IF($Y83="","Cód: "&amp;$H83,"Medidas: "&amp;$Y83&amp;"  ·  Cód: "&amp;$H83))</f>
       </c>
       <c r="D83" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;78,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H83="","",IF($D$3="Mayor",$V83,$U83))</f>
       </c>
     </row>
     <row r="84" ht="90.00" customHeight="1">
       <c r="A84" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H84="","",IFERROR(IMAGE($T84,1),""))</f>
       </c>
       <c r="B84" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H84="","",$I84)</f>
       </c>
       <c r="C84" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H84="","",IF($Y84="","Cód: "&amp;$H84,"Medidas: "&amp;$Y84&amp;"  ·  Cód: "&amp;$H84))</f>
       </c>
       <c r="D84" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;79,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H84="","",IF($D$3="Mayor",$V84,$U84))</f>
       </c>
     </row>
     <row r="85" ht="90.00" customHeight="1">
       <c r="A85" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H85="","",IFERROR(IMAGE($T85,1),""))</f>
       </c>
       <c r="B85" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H85="","",$I85)</f>
       </c>
       <c r="C85" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H85="","",IF($Y85="","Cód: "&amp;$H85,"Medidas: "&amp;$Y85&amp;"  ·  Cód: "&amp;$H85))</f>
       </c>
       <c r="D85" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;80,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H85="","",IF($D$3="Mayor",$V85,$U85))</f>
       </c>
     </row>
     <row r="86" ht="90.00" customHeight="1">
       <c r="A86" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H86="","",IFERROR(IMAGE($T86,1),""))</f>
       </c>
       <c r="B86" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H86="","",$I86)</f>
       </c>
       <c r="C86" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H86="","",IF($Y86="","Cód: "&amp;$H86,"Medidas: "&amp;$Y86&amp;"  ·  Cód: "&amp;$H86))</f>
       </c>
       <c r="D86" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;81,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H86="","",IF($D$3="Mayor",$V86,$U86))</f>
       </c>
     </row>
     <row r="87" ht="90.00" customHeight="1">
       <c r="A87" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H87="","",IFERROR(IMAGE($T87,1),""))</f>
       </c>
       <c r="B87" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H87="","",$I87)</f>
       </c>
       <c r="C87" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H87="","",IF($Y87="","Cód: "&amp;$H87,"Medidas: "&amp;$Y87&amp;"  ·  Cód: "&amp;$H87))</f>
       </c>
       <c r="D87" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;82,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H87="","",IF($D$3="Mayor",$V87,$U87))</f>
       </c>
     </row>
     <row r="88" ht="90.00" customHeight="1">
       <c r="A88" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H88="","",IFERROR(IMAGE($T88,1),""))</f>
       </c>
       <c r="B88" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H88="","",$I88)</f>
       </c>
       <c r="C88" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H88="","",IF($Y88="","Cód: "&amp;$H88,"Medidas: "&amp;$Y88&amp;"  ·  Cód: "&amp;$H88))</f>
       </c>
       <c r="D88" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;83,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H88="","",IF($D$3="Mayor",$V88,$U88))</f>
       </c>
     </row>
     <row r="89" ht="90.00" customHeight="1">
       <c r="A89" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H89="","",IFERROR(IMAGE($T89,1),""))</f>
       </c>
       <c r="B89" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H89="","",$I89)</f>
       </c>
       <c r="C89" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H89="","",IF($Y89="","Cód: "&amp;$H89,"Medidas: "&amp;$Y89&amp;"  ·  Cód: "&amp;$H89))</f>
       </c>
       <c r="D89" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;84,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H89="","",IF($D$3="Mayor",$V89,$U89))</f>
       </c>
     </row>
     <row r="90" ht="90.00" customHeight="1">
       <c r="A90" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H90="","",IFERROR(IMAGE($T90,1),""))</f>
       </c>
       <c r="B90" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H90="","",$I90)</f>
       </c>
       <c r="C90" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H90="","",IF($Y90="","Cód: "&amp;$H90,"Medidas: "&amp;$Y90&amp;"  ·  Cód: "&amp;$H90))</f>
       </c>
       <c r="D90" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;85,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H90="","",IF($D$3="Mayor",$V90,$U90))</f>
       </c>
     </row>
     <row r="91" ht="90.00" customHeight="1">
       <c r="A91" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H91="","",IFERROR(IMAGE($T91,1),""))</f>
       </c>
       <c r="B91" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H91="","",$I91)</f>
       </c>
       <c r="C91" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H91="","",IF($Y91="","Cód: "&amp;$H91,"Medidas: "&amp;$Y91&amp;"  ·  Cód: "&amp;$H91))</f>
       </c>
       <c r="D91" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;86,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H91="","",IF($D$3="Mayor",$V91,$U91))</f>
       </c>
     </row>
     <row r="92" ht="90.00" customHeight="1">
       <c r="A92" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H92="","",IFERROR(IMAGE($T92,1),""))</f>
       </c>
       <c r="B92" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H92="","",$I92)</f>
       </c>
       <c r="C92" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H92="","",IF($Y92="","Cód: "&amp;$H92,"Medidas: "&amp;$Y92&amp;"  ·  Cód: "&amp;$H92))</f>
       </c>
       <c r="D92" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;87,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H92="","",IF($D$3="Mayor",$V92,$U92))</f>
       </c>
     </row>
     <row r="93" ht="90.00" customHeight="1">
       <c r="A93" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H93="","",IFERROR(IMAGE($T93,1),""))</f>
       </c>
       <c r="B93" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H93="","",$I93)</f>
       </c>
       <c r="C93" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H93="","",IF($Y93="","Cód: "&amp;$H93,"Medidas: "&amp;$Y93&amp;"  ·  Cód: "&amp;$H93))</f>
       </c>
       <c r="D93" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;88,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H93="","",IF($D$3="Mayor",$V93,$U93))</f>
       </c>
     </row>
     <row r="94" ht="90.00" customHeight="1">
       <c r="A94" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H94="","",IFERROR(IMAGE($T94,1),""))</f>
       </c>
       <c r="B94" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H94="","",$I94)</f>
       </c>
       <c r="C94" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H94="","",IF($Y94="","Cód: "&amp;$H94,"Medidas: "&amp;$Y94&amp;"  ·  Cód: "&amp;$H94))</f>
       </c>
       <c r="D94" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;89,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H94="","",IF($D$3="Mayor",$V94,$U94))</f>
       </c>
     </row>
     <row r="95" ht="90.00" customHeight="1">
       <c r="A95" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H95="","",IFERROR(IMAGE($T95,1),""))</f>
       </c>
       <c r="B95" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H95="","",$I95)</f>
       </c>
       <c r="C95" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H95="","",IF($Y95="","Cód: "&amp;$H95,"Medidas: "&amp;$Y95&amp;"  ·  Cód: "&amp;$H95))</f>
       </c>
       <c r="D95" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;90,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H95="","",IF($D$3="Mayor",$V95,$U95))</f>
       </c>
     </row>
     <row r="96" ht="90.00" customHeight="1">
       <c r="A96" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H96="","",IFERROR(IMAGE($T96,1),""))</f>
       </c>
       <c r="B96" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H96="","",$I96)</f>
       </c>
       <c r="C96" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H96="","",IF($Y96="","Cód: "&amp;$H96,"Medidas: "&amp;$Y96&amp;"  ·  Cód: "&amp;$H96))</f>
       </c>
       <c r="D96" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;91,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H96="","",IF($D$3="Mayor",$V96,$U96))</f>
       </c>
     </row>
     <row r="97" ht="90.00" customHeight="1">
       <c r="A97" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H97="","",IFERROR(IMAGE($T97,1),""))</f>
       </c>
       <c r="B97" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H97="","",$I97)</f>
       </c>
       <c r="C97" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H97="","",IF($Y97="","Cód: "&amp;$H97,"Medidas: "&amp;$Y97&amp;"  ·  Cód: "&amp;$H97))</f>
       </c>
       <c r="D97" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;92,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H97="","",IF($D$3="Mayor",$V97,$U97))</f>
       </c>
     </row>
     <row r="98" ht="90.00" customHeight="1">
       <c r="A98" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H98="","",IFERROR(IMAGE($T98,1),""))</f>
       </c>
       <c r="B98" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H98="","",$I98)</f>
       </c>
       <c r="C98" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H98="","",IF($Y98="","Cód: "&amp;$H98,"Medidas: "&amp;$Y98&amp;"  ·  Cód: "&amp;$H98))</f>
       </c>
       <c r="D98" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;93,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H98="","",IF($D$3="Mayor",$V98,$U98))</f>
       </c>
     </row>
     <row r="99" ht="90.00" customHeight="1">
       <c r="A99" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H99="","",IFERROR(IMAGE($T99,1),""))</f>
       </c>
       <c r="B99" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H99="","",$I99)</f>
       </c>
       <c r="C99" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H99="","",IF($Y99="","Cód: "&amp;$H99,"Medidas: "&amp;$Y99&amp;"  ·  Cód: "&amp;$H99))</f>
       </c>
       <c r="D99" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;94,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H99="","",IF($D$3="Mayor",$V99,$U99))</f>
       </c>
     </row>
     <row r="100" ht="90.00" customHeight="1">
       <c r="A100" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H100="","",IFERROR(IMAGE($T100,1),""))</f>
       </c>
       <c r="B100" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H100="","",$I100)</f>
       </c>
       <c r="C100" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H100="","",IF($Y100="","Cód: "&amp;$H100,"Medidas: "&amp;$Y100&amp;"  ·  Cód: "&amp;$H100))</f>
       </c>
       <c r="D100" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;95,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H100="","",IF($D$3="Mayor",$V100,$U100))</f>
       </c>
     </row>
     <row r="101" ht="90.00" customHeight="1">
       <c r="A101" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H101="","",IFERROR(IMAGE($T101,1),""))</f>
       </c>
       <c r="B101" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H101="","",$I101)</f>
       </c>
       <c r="C101" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H101="","",IF($Y101="","Cód: "&amp;$H101,"Medidas: "&amp;$Y101&amp;"  ·  Cód: "&amp;$H101))</f>
       </c>
       <c r="D101" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;96,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H101="","",IF($D$3="Mayor",$V101,$U101))</f>
       </c>
     </row>
     <row r="102" ht="90.00" customHeight="1">
       <c r="A102" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H102="","",IFERROR(IMAGE($T102,1),""))</f>
       </c>
       <c r="B102" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H102="","",$I102)</f>
       </c>
       <c r="C102" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H102="","",IF($Y102="","Cód: "&amp;$H102,"Medidas: "&amp;$Y102&amp;"  ·  Cód: "&amp;$H102))</f>
       </c>
       <c r="D102" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;97,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H102="","",IF($D$3="Mayor",$V102,$U102))</f>
       </c>
     </row>
     <row r="103" ht="90.00" customHeight="1">
       <c r="A103" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H103="","",IFERROR(IMAGE($T103,1),""))</f>
       </c>
       <c r="B103" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H103="","",$I103)</f>
       </c>
       <c r="C103" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H103="","",IF($Y103="","Cód: "&amp;$H103,"Medidas: "&amp;$Y103&amp;"  ·  Cód: "&amp;$H103))</f>
       </c>
       <c r="D103" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;98,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H103="","",IF($D$3="Mayor",$V103,$U103))</f>
       </c>
     </row>
     <row r="104" ht="90.00" customHeight="1">
       <c r="A104" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H104="","",IFERROR(IMAGE($T104,1),""))</f>
       </c>
       <c r="B104" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H104="","",$I104)</f>
       </c>
       <c r="C104" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H104="","",IF($Y104="","Cód: "&amp;$H104,"Medidas: "&amp;$Y104&amp;"  ·  Cód: "&amp;$H104))</f>
       </c>
       <c r="D104" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;99,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H104="","",IF($D$3="Mayor",$V104,$U104))</f>
       </c>
     </row>
     <row r="105" ht="90.00" customHeight="1">
       <c r="A105" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H105="","",IFERROR(IMAGE($T105,1),""))</f>
       </c>
       <c r="B105" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H105="","",$I105)</f>
       </c>
       <c r="C105" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H105="","",IF($Y105="","Cód: "&amp;$H105,"Medidas: "&amp;$Y105&amp;"  ·  Cód: "&amp;$H105))</f>
       </c>
       <c r="D105" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;100,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H105="","",IF($D$3="Mayor",$V105,$U105))</f>
       </c>
     </row>
     <row r="106" ht="90.00" customHeight="1">
       <c r="A106" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H106="","",IFERROR(IMAGE($T106,1),""))</f>
       </c>
       <c r="B106" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H106="","",$I106)</f>
       </c>
       <c r="C106" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H106="","",IF($Y106="","Cód: "&amp;$H106,"Medidas: "&amp;$Y106&amp;"  ·  Cód: "&amp;$H106))</f>
       </c>
       <c r="D106" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;101,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H106="","",IF($D$3="Mayor",$V106,$U106))</f>
       </c>
     </row>
     <row r="107" ht="90.00" customHeight="1">
       <c r="A107" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H107="","",IFERROR(IMAGE($T107,1),""))</f>
       </c>
       <c r="B107" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H107="","",$I107)</f>
       </c>
       <c r="C107" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H107="","",IF($Y107="","Cód: "&amp;$H107,"Medidas: "&amp;$Y107&amp;"  ·  Cód: "&amp;$H107))</f>
       </c>
       <c r="D107" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;102,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H107="","",IF($D$3="Mayor",$V107,$U107))</f>
       </c>
     </row>
     <row r="108" ht="90.00" customHeight="1">
       <c r="A108" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H108="","",IFERROR(IMAGE($T108,1),""))</f>
       </c>
       <c r="B108" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H108="","",$I108)</f>
       </c>
       <c r="C108" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H108="","",IF($Y108="","Cód: "&amp;$H108,"Medidas: "&amp;$Y108&amp;"  ·  Cód: "&amp;$H108))</f>
       </c>
       <c r="D108" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;103,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H108="","",IF($D$3="Mayor",$V108,$U108))</f>
       </c>
     </row>
     <row r="109" ht="90.00" customHeight="1">
       <c r="A109" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H109="","",IFERROR(IMAGE($T109,1),""))</f>
       </c>
       <c r="B109" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H109="","",$I109)</f>
       </c>
       <c r="C109" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H109="","",IF($Y109="","Cód: "&amp;$H109,"Medidas: "&amp;$Y109&amp;"  ·  Cód: "&amp;$H109))</f>
       </c>
       <c r="D109" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;104,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H109="","",IF($D$3="Mayor",$V109,$U109))</f>
       </c>
     </row>
     <row r="110" ht="90.00" customHeight="1">
       <c r="A110" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H110="","",IFERROR(IMAGE($T110,1),""))</f>
       </c>
       <c r="B110" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H110="","",$I110)</f>
       </c>
       <c r="C110" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H110="","",IF($Y110="","Cód: "&amp;$H110,"Medidas: "&amp;$Y110&amp;"  ·  Cód: "&amp;$H110))</f>
       </c>
       <c r="D110" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;105,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H110="","",IF($D$3="Mayor",$V110,$U110))</f>
       </c>
     </row>
     <row r="111" ht="90.00" customHeight="1">
       <c r="A111" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H111="","",IFERROR(IMAGE($T111,1),""))</f>
       </c>
       <c r="B111" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H111="","",$I111)</f>
       </c>
       <c r="C111" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H111="","",IF($Y111="","Cód: "&amp;$H111,"Medidas: "&amp;$Y111&amp;"  ·  Cód: "&amp;$H111))</f>
       </c>
       <c r="D111" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;106,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H111="","",IF($D$3="Mayor",$V111,$U111))</f>
       </c>
     </row>
     <row r="112" ht="90.00" customHeight="1">
       <c r="A112" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H112="","",IFERROR(IMAGE($T112,1),""))</f>
       </c>
       <c r="B112" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H112="","",$I112)</f>
       </c>
       <c r="C112" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H112="","",IF($Y112="","Cód: "&amp;$H112,"Medidas: "&amp;$Y112&amp;"  ·  Cód: "&amp;$H112))</f>
       </c>
       <c r="D112" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;107,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H112="","",IF($D$3="Mayor",$V112,$U112))</f>
       </c>
     </row>
     <row r="113" ht="90.00" customHeight="1">
       <c r="A113" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H113="","",IFERROR(IMAGE($T113,1),""))</f>
       </c>
       <c r="B113" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H113="","",$I113)</f>
       </c>
       <c r="C113" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H113="","",IF($Y113="","Cód: "&amp;$H113,"Medidas: "&amp;$Y113&amp;"  ·  Cód: "&amp;$H113))</f>
       </c>
       <c r="D113" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;108,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H113="","",IF($D$3="Mayor",$V113,$U113))</f>
       </c>
     </row>
     <row r="114" ht="90.00" customHeight="1">
       <c r="A114" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H114="","",IFERROR(IMAGE($T114,1),""))</f>
       </c>
       <c r="B114" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H114="","",$I114)</f>
       </c>
       <c r="C114" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H114="","",IF($Y114="","Cód: "&amp;$H114,"Medidas: "&amp;$Y114&amp;"  ·  Cód: "&amp;$H114))</f>
       </c>
       <c r="D114" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;109,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H114="","",IF($D$3="Mayor",$V114,$U114))</f>
       </c>
     </row>
     <row r="115" ht="90.00" customHeight="1">
       <c r="A115" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H115="","",IFERROR(IMAGE($T115,1),""))</f>
       </c>
       <c r="B115" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H115="","",$I115)</f>
       </c>
       <c r="C115" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H115="","",IF($Y115="","Cód: "&amp;$H115,"Medidas: "&amp;$Y115&amp;"  ·  Cód: "&amp;$H115))</f>
       </c>
       <c r="D115" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;110,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H115="","",IF($D$3="Mayor",$V115,$U115))</f>
       </c>
     </row>
     <row r="116" ht="90.00" customHeight="1">
       <c r="A116" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H116="","",IFERROR(IMAGE($T116,1),""))</f>
       </c>
       <c r="B116" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H116="","",$I116)</f>
       </c>
       <c r="C116" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H116="","",IF($Y116="","Cód: "&amp;$H116,"Medidas: "&amp;$Y116&amp;"  ·  Cód: "&amp;$H116))</f>
       </c>
       <c r="D116" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;111,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H116="","",IF($D$3="Mayor",$V116,$U116))</f>
       </c>
     </row>
     <row r="117" ht="90.00" customHeight="1">
       <c r="A117" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H117="","",IFERROR(IMAGE($T117,1),""))</f>
       </c>
       <c r="B117" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H117="","",$I117)</f>
       </c>
       <c r="C117" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H117="","",IF($Y117="","Cód: "&amp;$H117,"Medidas: "&amp;$Y117&amp;"  ·  Cód: "&amp;$H117))</f>
       </c>
       <c r="D117" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;112,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H117="","",IF($D$3="Mayor",$V117,$U117))</f>
       </c>
     </row>
     <row r="118" ht="90.00" customHeight="1">
       <c r="A118" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H118="","",IFERROR(IMAGE($T118,1),""))</f>
       </c>
       <c r="B118" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H118="","",$I118)</f>
       </c>
       <c r="C118" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H118="","",IF($Y118="","Cód: "&amp;$H118,"Medidas: "&amp;$Y118&amp;"  ·  Cód: "&amp;$H118))</f>
       </c>
       <c r="D118" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;113,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H118="","",IF($D$3="Mayor",$V118,$U118))</f>
       </c>
     </row>
     <row r="119" ht="90.00" customHeight="1">
       <c r="A119" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H119="","",IFERROR(IMAGE($T119,1),""))</f>
       </c>
       <c r="B119" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H119="","",$I119)</f>
       </c>
       <c r="C119" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H119="","",IF($Y119="","Cód: "&amp;$H119,"Medidas: "&amp;$Y119&amp;"  ·  Cód: "&amp;$H119))</f>
       </c>
       <c r="D119" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;114,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H119="","",IF($D$3="Mayor",$V119,$U119))</f>
       </c>
     </row>
     <row r="120" ht="90.00" customHeight="1">
       <c r="A120" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H120="","",IFERROR(IMAGE($T120,1),""))</f>
       </c>
       <c r="B120" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H120="","",$I120)</f>
       </c>
       <c r="C120" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H120="","",IF($Y120="","Cód: "&amp;$H120,"Medidas: "&amp;$Y120&amp;"  ·  Cód: "&amp;$H120))</f>
       </c>
       <c r="D120" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;115,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H120="","",IF($D$3="Mayor",$V120,$U120))</f>
       </c>
     </row>
     <row r="121" ht="90.00" customHeight="1">
       <c r="A121" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H121="","",IFERROR(IMAGE($T121,1),""))</f>
       </c>
       <c r="B121" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H121="","",$I121)</f>
       </c>
       <c r="C121" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H121="","",IF($Y121="","Cód: "&amp;$H121,"Medidas: "&amp;$Y121&amp;"  ·  Cód: "&amp;$H121))</f>
       </c>
       <c r="D121" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;116,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H121="","",IF($D$3="Mayor",$V121,$U121))</f>
       </c>
     </row>
     <row r="122" ht="90.00" customHeight="1">
       <c r="A122" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H122="","",IFERROR(IMAGE($T122,1),""))</f>
       </c>
       <c r="B122" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H122="","",$I122)</f>
       </c>
       <c r="C122" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H122="","",IF($Y122="","Cód: "&amp;$H122,"Medidas: "&amp;$Y122&amp;"  ·  Cód: "&amp;$H122))</f>
       </c>
       <c r="D122" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;117,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H122="","",IF($D$3="Mayor",$V122,$U122))</f>
       </c>
     </row>
     <row r="123" ht="90.00" customHeight="1">
       <c r="A123" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H123="","",IFERROR(IMAGE($T123,1),""))</f>
       </c>
       <c r="B123" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H123="","",$I123)</f>
       </c>
       <c r="C123" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H123="","",IF($Y123="","Cód: "&amp;$H123,"Medidas: "&amp;$Y123&amp;"  ·  Cód: "&amp;$H123))</f>
       </c>
       <c r="D123" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;118,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H123="","",IF($D$3="Mayor",$V123,$U123))</f>
       </c>
     </row>
     <row r="124" ht="90.00" customHeight="1">
       <c r="A124" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H124="","",IFERROR(IMAGE($T124,1),""))</f>
       </c>
       <c r="B124" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H124="","",$I124)</f>
       </c>
       <c r="C124" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H124="","",IF($Y124="","Cód: "&amp;$H124,"Medidas: "&amp;$Y124&amp;"  ·  Cód: "&amp;$H124))</f>
       </c>
       <c r="D124" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;119,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H124="","",IF($D$3="Mayor",$V124,$U124))</f>
       </c>
     </row>
     <row r="125" ht="90.00" customHeight="1">
       <c r="A125" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H125="","",IFERROR(IMAGE($T125,1),""))</f>
       </c>
       <c r="B125" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H125="","",$I125)</f>
       </c>
       <c r="C125" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H125="","",IF($Y125="","Cód: "&amp;$H125,"Medidas: "&amp;$Y125&amp;"  ·  Cód: "&amp;$H125))</f>
       </c>
       <c r="D125" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;120,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H125="","",IF($D$3="Mayor",$V125,$U125))</f>
       </c>
     </row>
     <row r="126" ht="90.00" customHeight="1">
       <c r="A126" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H126="","",IFERROR(IMAGE($T126,1),""))</f>
       </c>
       <c r="B126" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H126="","",$I126)</f>
       </c>
       <c r="C126" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H126="","",IF($Y126="","Cód: "&amp;$H126,"Medidas: "&amp;$Y126&amp;"  ·  Cód: "&amp;$H126))</f>
       </c>
       <c r="D126" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;121,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H126="","",IF($D$3="Mayor",$V126,$U126))</f>
       </c>
     </row>
     <row r="127" ht="90.00" customHeight="1">
       <c r="A127" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H127="","",IFERROR(IMAGE($T127,1),""))</f>
       </c>
       <c r="B127" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H127="","",$I127)</f>
       </c>
       <c r="C127" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H127="","",IF($Y127="","Cód: "&amp;$H127,"Medidas: "&amp;$Y127&amp;"  ·  Cód: "&amp;$H127))</f>
       </c>
       <c r="D127" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;122,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H127="","",IF($D$3="Mayor",$V127,$U127))</f>
       </c>
     </row>
     <row r="128" ht="90.00" customHeight="1">
       <c r="A128" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H128="","",IFERROR(IMAGE($T128,1),""))</f>
       </c>
       <c r="B128" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H128="","",$I128)</f>
       </c>
       <c r="C128" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H128="","",IF($Y128="","Cód: "&amp;$H128,"Medidas: "&amp;$Y128&amp;"  ·  Cód: "&amp;$H128))</f>
       </c>
       <c r="D128" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;123,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H128="","",IF($D$3="Mayor",$V128,$U128))</f>
       </c>
     </row>
     <row r="129" ht="90.00" customHeight="1">
       <c r="A129" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H129="","",IFERROR(IMAGE($T129,1),""))</f>
       </c>
       <c r="B129" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H129="","",$I129)</f>
       </c>
       <c r="C129" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H129="","",IF($Y129="","Cód: "&amp;$H129,"Medidas: "&amp;$Y129&amp;"  ·  Cód: "&amp;$H129))</f>
       </c>
       <c r="D129" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;124,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H129="","",IF($D$3="Mayor",$V129,$U129))</f>
       </c>
     </row>
     <row r="130" ht="90.00" customHeight="1">
       <c r="A130" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H130="","",IFERROR(IMAGE($T130,1),""))</f>
       </c>
       <c r="B130" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H130="","",$I130)</f>
       </c>
       <c r="C130" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H130="","",IF($Y130="","Cód: "&amp;$H130,"Medidas: "&amp;$Y130&amp;"  ·  Cód: "&amp;$H130))</f>
       </c>
       <c r="D130" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;125,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H130="","",IF($D$3="Mayor",$V130,$U130))</f>
       </c>
     </row>
     <row r="131" ht="90.00" customHeight="1">
       <c r="A131" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H131="","",IFERROR(IMAGE($T131,1),""))</f>
       </c>
       <c r="B131" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H131="","",$I131)</f>
       </c>
       <c r="C131" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H131="","",IF($Y131="","Cód: "&amp;$H131,"Medidas: "&amp;$Y131&amp;"  ·  Cód: "&amp;$H131))</f>
       </c>
       <c r="D131" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;126,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H131="","",IF($D$3="Mayor",$V131,$U131))</f>
       </c>
     </row>
     <row r="132" ht="90.00" customHeight="1">
       <c r="A132" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H132="","",IFERROR(IMAGE($T132,1),""))</f>
       </c>
       <c r="B132" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H132="","",$I132)</f>
       </c>
       <c r="C132" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H132="","",IF($Y132="","Cód: "&amp;$H132,"Medidas: "&amp;$Y132&amp;"  ·  Cód: "&amp;$H132))</f>
       </c>
       <c r="D132" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;127,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H132="","",IF($D$3="Mayor",$V132,$U132))</f>
       </c>
     </row>
     <row r="133" ht="90.00" customHeight="1">
       <c r="A133" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H133="","",IFERROR(IMAGE($T133,1),""))</f>
       </c>
       <c r="B133" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H133="","",$I133)</f>
       </c>
       <c r="C133" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H133="","",IF($Y133="","Cód: "&amp;$H133,"Medidas: "&amp;$Y133&amp;"  ·  Cód: "&amp;$H133))</f>
       </c>
       <c r="D133" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;128,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H133="","",IF($D$3="Mayor",$V133,$U133))</f>
       </c>
     </row>
     <row r="134" ht="90.00" customHeight="1">
       <c r="A134" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H134="","",IFERROR(IMAGE($T134,1),""))</f>
       </c>
       <c r="B134" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H134="","",$I134)</f>
       </c>
       <c r="C134" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H134="","",IF($Y134="","Cód: "&amp;$H134,"Medidas: "&amp;$Y134&amp;"  ·  Cód: "&amp;$H134))</f>
       </c>
       <c r="D134" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;129,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H134="","",IF($D$3="Mayor",$V134,$U134))</f>
       </c>
     </row>
     <row r="135" ht="90.00" customHeight="1">
       <c r="A135" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H135="","",IFERROR(IMAGE($T135,1),""))</f>
       </c>
       <c r="B135" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H135="","",$I135)</f>
       </c>
       <c r="C135" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H135="","",IF($Y135="","Cód: "&amp;$H135,"Medidas: "&amp;$Y135&amp;"  ·  Cód: "&amp;$H135))</f>
       </c>
       <c r="D135" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;130,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H135="","",IF($D$3="Mayor",$V135,$U135))</f>
       </c>
     </row>
     <row r="136" ht="90.00" customHeight="1">
       <c r="A136" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H136="","",IFERROR(IMAGE($T136,1),""))</f>
       </c>
       <c r="B136" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H136="","",$I136)</f>
       </c>
       <c r="C136" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H136="","",IF($Y136="","Cód: "&amp;$H136,"Medidas: "&amp;$Y136&amp;"  ·  Cód: "&amp;$H136))</f>
       </c>
       <c r="D136" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;131,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H136="","",IF($D$3="Mayor",$V136,$U136))</f>
       </c>
     </row>
     <row r="137" ht="90.00" customHeight="1">
       <c r="A137" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H137="","",IFERROR(IMAGE($T137,1),""))</f>
       </c>
       <c r="B137" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H137="","",$I137)</f>
       </c>
       <c r="C137" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H137="","",IF($Y137="","Cód: "&amp;$H137,"Medidas: "&amp;$Y137&amp;"  ·  Cód: "&amp;$H137))</f>
       </c>
       <c r="D137" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;132,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H137="","",IF($D$3="Mayor",$V137,$U137))</f>
       </c>
     </row>
     <row r="138" ht="90.00" customHeight="1">
       <c r="A138" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H138="","",IFERROR(IMAGE($T138,1),""))</f>
       </c>
       <c r="B138" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H138="","",$I138)</f>
       </c>
       <c r="C138" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H138="","",IF($Y138="","Cód: "&amp;$H138,"Medidas: "&amp;$Y138&amp;"  ·  Cód: "&amp;$H138))</f>
       </c>
       <c r="D138" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;133,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H138="","",IF($D$3="Mayor",$V138,$U138))</f>
       </c>
     </row>
     <row r="139" ht="90.00" customHeight="1">
       <c r="A139" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H139="","",IFERROR(IMAGE($T139,1),""))</f>
       </c>
       <c r="B139" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H139="","",$I139)</f>
       </c>
       <c r="C139" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H139="","",IF($Y139="","Cód: "&amp;$H139,"Medidas: "&amp;$Y139&amp;"  ·  Cód: "&amp;$H139))</f>
       </c>
       <c r="D139" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;134,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H139="","",IF($D$3="Mayor",$V139,$U139))</f>
       </c>
     </row>
     <row r="140" ht="90.00" customHeight="1">
       <c r="A140" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H140="","",IFERROR(IMAGE($T140,1),""))</f>
       </c>
       <c r="B140" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H140="","",$I140)</f>
       </c>
       <c r="C140" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H140="","",IF($Y140="","Cód: "&amp;$H140,"Medidas: "&amp;$Y140&amp;"  ·  Cód: "&amp;$H140))</f>
       </c>
       <c r="D140" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;135,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H140="","",IF($D$3="Mayor",$V140,$U140))</f>
       </c>
     </row>
     <row r="141" ht="90.00" customHeight="1">
       <c r="A141" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H141="","",IFERROR(IMAGE($T141,1),""))</f>
       </c>
       <c r="B141" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H141="","",$I141)</f>
       </c>
       <c r="C141" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H141="","",IF($Y141="","Cód: "&amp;$H141,"Medidas: "&amp;$Y141&amp;"  ·  Cód: "&amp;$H141))</f>
       </c>
       <c r="D141" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;136,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H141="","",IF($D$3="Mayor",$V141,$U141))</f>
       </c>
     </row>
     <row r="142" ht="90.00" customHeight="1">
       <c r="A142" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H142="","",IFERROR(IMAGE($T142,1),""))</f>
       </c>
       <c r="B142" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H142="","",$I142)</f>
       </c>
       <c r="C142" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H142="","",IF($Y142="","Cód: "&amp;$H142,"Medidas: "&amp;$Y142&amp;"  ·  Cód: "&amp;$H142))</f>
       </c>
       <c r="D142" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;137,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H142="","",IF($D$3="Mayor",$V142,$U142))</f>
       </c>
     </row>
     <row r="143" ht="90.00" customHeight="1">
       <c r="A143" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H143="","",IFERROR(IMAGE($T143,1),""))</f>
       </c>
       <c r="B143" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H143="","",$I143)</f>
       </c>
       <c r="C143" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H143="","",IF($Y143="","Cód: "&amp;$H143,"Medidas: "&amp;$Y143&amp;"  ·  Cód: "&amp;$H143))</f>
       </c>
       <c r="D143" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;138,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H143="","",IF($D$3="Mayor",$V143,$U143))</f>
       </c>
     </row>
     <row r="144" ht="90.00" customHeight="1">
       <c r="A144" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H144="","",IFERROR(IMAGE($T144,1),""))</f>
       </c>
       <c r="B144" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H144="","",$I144)</f>
       </c>
       <c r="C144" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H144="","",IF($Y144="","Cód: "&amp;$H144,"Medidas: "&amp;$Y144&amp;"  ·  Cód: "&amp;$H144))</f>
       </c>
       <c r="D144" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;139,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H144="","",IF($D$3="Mayor",$V144,$U144))</f>
       </c>
     </row>
     <row r="145" ht="90.00" customHeight="1">
       <c r="A145" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H145="","",IFERROR(IMAGE($T145,1),""))</f>
       </c>
       <c r="B145" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H145="","",$I145)</f>
       </c>
       <c r="C145" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H145="","",IF($Y145="","Cód: "&amp;$H145,"Medidas: "&amp;$Y145&amp;"  ·  Cód: "&amp;$H145))</f>
       </c>
       <c r="D145" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;140,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H145="","",IF($D$3="Mayor",$V145,$U145))</f>
       </c>
     </row>
     <row r="146" ht="90.00" customHeight="1">
       <c r="A146" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H146="","",IFERROR(IMAGE($T146,1),""))</f>
       </c>
       <c r="B146" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H146="","",$I146)</f>
       </c>
       <c r="C146" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H146="","",IF($Y146="","Cód: "&amp;$H146,"Medidas: "&amp;$Y146&amp;"  ·  Cód: "&amp;$H146))</f>
       </c>
       <c r="D146" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;141,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H146="","",IF($D$3="Mayor",$V146,$U146))</f>
       </c>
     </row>
     <row r="147" ht="90.00" customHeight="1">
       <c r="A147" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H147="","",IFERROR(IMAGE($T147,1),""))</f>
       </c>
       <c r="B147" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H147="","",$I147)</f>
       </c>
       <c r="C147" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H147="","",IF($Y147="","Cód: "&amp;$H147,"Medidas: "&amp;$Y147&amp;"  ·  Cód: "&amp;$H147))</f>
       </c>
       <c r="D147" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;142,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H147="","",IF($D$3="Mayor",$V147,$U147))</f>
       </c>
     </row>
     <row r="148" ht="90.00" customHeight="1">
       <c r="A148" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H148="","",IFERROR(IMAGE($T148,1),""))</f>
       </c>
       <c r="B148" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H148="","",$I148)</f>
       </c>
       <c r="C148" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H148="","",IF($Y148="","Cód: "&amp;$H148,"Medidas: "&amp;$Y148&amp;"  ·  Cód: "&amp;$H148))</f>
       </c>
       <c r="D148" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;143,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H148="","",IF($D$3="Mayor",$V148,$U148))</f>
       </c>
     </row>
     <row r="149" ht="90.00" customHeight="1">
       <c r="A149" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H149="","",IFERROR(IMAGE($T149,1),""))</f>
       </c>
       <c r="B149" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H149="","",$I149)</f>
       </c>
       <c r="C149" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H149="","",IF($Y149="","Cód: "&amp;$H149,"Medidas: "&amp;$Y149&amp;"  ·  Cód: "&amp;$H149))</f>
       </c>
       <c r="D149" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;144,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H149="","",IF($D$3="Mayor",$V149,$U149))</f>
       </c>
     </row>
     <row r="150" ht="90.00" customHeight="1">
       <c r="A150" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H150="","",IFERROR(IMAGE($T150,1),""))</f>
       </c>
       <c r="B150" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H150="","",$I150)</f>
       </c>
       <c r="C150" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H150="","",IF($Y150="","Cód: "&amp;$H150,"Medidas: "&amp;$Y150&amp;"  ·  Cód: "&amp;$H150))</f>
       </c>
       <c r="D150" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;145,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H150="","",IF($D$3="Mayor",$V150,$U150))</f>
       </c>
     </row>
     <row r="151" ht="90.00" customHeight="1">
       <c r="A151" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H151="","",IFERROR(IMAGE($T151,1),""))</f>
       </c>
       <c r="B151" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H151="","",$I151)</f>
       </c>
       <c r="C151" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H151="","",IF($Y151="","Cód: "&amp;$H151,"Medidas: "&amp;$Y151&amp;"  ·  Cód: "&amp;$H151))</f>
       </c>
       <c r="D151" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;146,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H151="","",IF($D$3="Mayor",$V151,$U151))</f>
       </c>
     </row>
     <row r="152" ht="90.00" customHeight="1">
       <c r="A152" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H152="","",IFERROR(IMAGE($T152,1),""))</f>
       </c>
       <c r="B152" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H152="","",$I152)</f>
       </c>
       <c r="C152" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H152="","",IF($Y152="","Cód: "&amp;$H152,"Medidas: "&amp;$Y152&amp;"  ·  Cód: "&amp;$H152))</f>
       </c>
       <c r="D152" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;147,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H152="","",IF($D$3="Mayor",$V152,$U152))</f>
       </c>
     </row>
     <row r="153" ht="90.00" customHeight="1">
       <c r="A153" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H153="","",IFERROR(IMAGE($T153,1),""))</f>
       </c>
       <c r="B153" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H153="","",$I153)</f>
       </c>
       <c r="C153" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H153="","",IF($Y153="","Cód: "&amp;$H153,"Medidas: "&amp;$Y153&amp;"  ·  Cód: "&amp;$H153))</f>
       </c>
       <c r="D153" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;148,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H153="","",IF($D$3="Mayor",$V153,$U153))</f>
       </c>
     </row>
     <row r="154" ht="90.00" customHeight="1">
       <c r="A154" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H154="","",IFERROR(IMAGE($T154,1),""))</f>
       </c>
       <c r="B154" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H154="","",$I154)</f>
       </c>
       <c r="C154" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H154="","",IF($Y154="","Cód: "&amp;$H154,"Medidas: "&amp;$Y154&amp;"  ·  Cód: "&amp;$H154))</f>
       </c>
       <c r="D154" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;149,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H154="","",IF($D$3="Mayor",$V154,$U154))</f>
       </c>
     </row>
     <row r="155" ht="90.00" customHeight="1">
       <c r="A155" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H155="","",IFERROR(IMAGE($T155,1),""))</f>
       </c>
       <c r="B155" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H155="","",$I155)</f>
       </c>
       <c r="C155" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H155="","",IF($Y155="","Cód: "&amp;$H155,"Medidas: "&amp;$Y155&amp;"  ·  Cód: "&amp;$H155))</f>
       </c>
       <c r="D155" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;150,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H155="","",IF($D$3="Mayor",$V155,$U155))</f>
       </c>
     </row>
     <row r="156" ht="90.00" customHeight="1">
       <c r="A156" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H156="","",IFERROR(IMAGE($T156,1),""))</f>
       </c>
       <c r="B156" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H156="","",$I156)</f>
       </c>
       <c r="C156" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H156="","",IF($Y156="","Cód: "&amp;$H156,"Medidas: "&amp;$Y156&amp;"  ·  Cód: "&amp;$H156))</f>
       </c>
       <c r="D156" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;151,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H156="","",IF($D$3="Mayor",$V156,$U156))</f>
       </c>
     </row>
     <row r="157" ht="90.00" customHeight="1">
       <c r="A157" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H157="","",IFERROR(IMAGE($T157,1),""))</f>
       </c>
       <c r="B157" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H157="","",$I157)</f>
       </c>
       <c r="C157" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H157="","",IF($Y157="","Cód: "&amp;$H157,"Medidas: "&amp;$Y157&amp;"  ·  Cód: "&amp;$H157))</f>
       </c>
       <c r="D157" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;152,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H157="","",IF($D$3="Mayor",$V157,$U157))</f>
       </c>
     </row>
     <row r="158" ht="90.00" customHeight="1">
       <c r="A158" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H158="","",IFERROR(IMAGE($T158,1),""))</f>
       </c>
       <c r="B158" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H158="","",$I158)</f>
       </c>
       <c r="C158" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H158="","",IF($Y158="","Cód: "&amp;$H158,"Medidas: "&amp;$Y158&amp;"  ·  Cód: "&amp;$H158))</f>
       </c>
       <c r="D158" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;153,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H158="","",IF($D$3="Mayor",$V158,$U158))</f>
       </c>
     </row>
     <row r="159" ht="90.00" customHeight="1">
       <c r="A159" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H159="","",IFERROR(IMAGE($T159,1),""))</f>
       </c>
       <c r="B159" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H159="","",$I159)</f>
       </c>
       <c r="C159" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H159="","",IF($Y159="","Cód: "&amp;$H159,"Medidas: "&amp;$Y159&amp;"  ·  Cód: "&amp;$H159))</f>
       </c>
       <c r="D159" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;154,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H159="","",IF($D$3="Mayor",$V159,$U159))</f>
       </c>
     </row>
     <row r="160" ht="90.00" customHeight="1">
       <c r="A160" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H160="","",IFERROR(IMAGE($T160,1),""))</f>
       </c>
       <c r="B160" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H160="","",$I160)</f>
       </c>
       <c r="C160" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H160="","",IF($Y160="","Cód: "&amp;$H160,"Medidas: "&amp;$Y160&amp;"  ·  Cód: "&amp;$H160))</f>
       </c>
       <c r="D160" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;155,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H160="","",IF($D$3="Mayor",$V160,$U160))</f>
       </c>
     </row>
     <row r="161" ht="90.00" customHeight="1">
       <c r="A161" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H161="","",IFERROR(IMAGE($T161,1),""))</f>
       </c>
       <c r="B161" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H161="","",$I161)</f>
       </c>
       <c r="C161" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H161="","",IF($Y161="","Cód: "&amp;$H161,"Medidas: "&amp;$Y161&amp;"  ·  Cód: "&amp;$H161))</f>
       </c>
       <c r="D161" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;156,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H161="","",IF($D$3="Mayor",$V161,$U161))</f>
       </c>
     </row>
     <row r="162" ht="90.00" customHeight="1">
       <c r="A162" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H162="","",IFERROR(IMAGE($T162,1),""))</f>
       </c>
       <c r="B162" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H162="","",$I162)</f>
       </c>
       <c r="C162" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H162="","",IF($Y162="","Cód: "&amp;$H162,"Medidas: "&amp;$Y162&amp;"  ·  Cód: "&amp;$H162))</f>
       </c>
       <c r="D162" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;157,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H162="","",IF($D$3="Mayor",$V162,$U162))</f>
       </c>
     </row>
     <row r="163" ht="90.00" customHeight="1">
       <c r="A163" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H163="","",IFERROR(IMAGE($T163,1),""))</f>
       </c>
       <c r="B163" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H163="","",$I163)</f>
       </c>
       <c r="C163" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H163="","",IF($Y163="","Cód: "&amp;$H163,"Medidas: "&amp;$Y163&amp;"  ·  Cód: "&amp;$H163))</f>
       </c>
       <c r="D163" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;158,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H163="","",IF($D$3="Mayor",$V163,$U163))</f>
       </c>
     </row>
     <row r="164" ht="90.00" customHeight="1">
       <c r="A164" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H164="","",IFERROR(IMAGE($T164,1),""))</f>
       </c>
       <c r="B164" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H164="","",$I164)</f>
       </c>
       <c r="C164" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H164="","",IF($Y164="","Cód: "&amp;$H164,"Medidas: "&amp;$Y164&amp;"  ·  Cód: "&amp;$H164))</f>
       </c>
       <c r="D164" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;159,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H164="","",IF($D$3="Mayor",$V164,$U164))</f>
       </c>
     </row>
     <row r="165" ht="90.00" customHeight="1">
       <c r="A165" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H165="","",IFERROR(IMAGE($T165,1),""))</f>
       </c>
       <c r="B165" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H165="","",$I165)</f>
       </c>
       <c r="C165" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H165="","",IF($Y165="","Cód: "&amp;$H165,"Medidas: "&amp;$Y165&amp;"  ·  Cód: "&amp;$H165))</f>
       </c>
       <c r="D165" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;160,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H165="","",IF($D$3="Mayor",$V165,$U165))</f>
       </c>
     </row>
     <row r="166" ht="90.00" customHeight="1">
       <c r="A166" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H166="","",IFERROR(IMAGE($T166,1),""))</f>
       </c>
       <c r="B166" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H166="","",$I166)</f>
       </c>
       <c r="C166" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H166="","",IF($Y166="","Cód: "&amp;$H166,"Medidas: "&amp;$Y166&amp;"  ·  Cód: "&amp;$H166))</f>
       </c>
       <c r="D166" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;161,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H166="","",IF($D$3="Mayor",$V166,$U166))</f>
       </c>
     </row>
     <row r="167" ht="90.00" customHeight="1">
       <c r="A167" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H167="","",IFERROR(IMAGE($T167,1),""))</f>
       </c>
       <c r="B167" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H167="","",$I167)</f>
       </c>
       <c r="C167" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H167="","",IF($Y167="","Cód: "&amp;$H167,"Medidas: "&amp;$Y167&amp;"  ·  Cód: "&amp;$H167))</f>
       </c>
       <c r="D167" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;162,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H167="","",IF($D$3="Mayor",$V167,$U167))</f>
       </c>
     </row>
     <row r="168" ht="90.00" customHeight="1">
       <c r="A168" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H168="","",IFERROR(IMAGE($T168,1),""))</f>
       </c>
       <c r="B168" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H168="","",$I168)</f>
       </c>
       <c r="C168" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H168="","",IF($Y168="","Cód: "&amp;$H168,"Medidas: "&amp;$Y168&amp;"  ·  Cód: "&amp;$H168))</f>
       </c>
       <c r="D168" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;163,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H168="","",IF($D$3="Mayor",$V168,$U168))</f>
       </c>
     </row>
     <row r="169" ht="90.00" customHeight="1">
       <c r="A169" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H169="","",IFERROR(IMAGE($T169,1),""))</f>
       </c>
       <c r="B169" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H169="","",$I169)</f>
       </c>
       <c r="C169" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H169="","",IF($Y169="","Cód: "&amp;$H169,"Medidas: "&amp;$Y169&amp;"  ·  Cód: "&amp;$H169))</f>
       </c>
       <c r="D169" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;164,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H169="","",IF($D$3="Mayor",$V169,$U169))</f>
       </c>
     </row>
     <row r="170" ht="90.00" customHeight="1">
       <c r="A170" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H170="","",IFERROR(IMAGE($T170,1),""))</f>
       </c>
       <c r="B170" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H170="","",$I170)</f>
       </c>
       <c r="C170" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H170="","",IF($Y170="","Cód: "&amp;$H170,"Medidas: "&amp;$Y170&amp;"  ·  Cód: "&amp;$H170))</f>
       </c>
       <c r="D170" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;165,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H170="","",IF($D$3="Mayor",$V170,$U170))</f>
       </c>
     </row>
     <row r="171" ht="90.00" customHeight="1">
       <c r="A171" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H171="","",IFERROR(IMAGE($T171,1),""))</f>
       </c>
       <c r="B171" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H171="","",$I171)</f>
       </c>
       <c r="C171" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H171="","",IF($Y171="","Cód: "&amp;$H171,"Medidas: "&amp;$Y171&amp;"  ·  Cód: "&amp;$H171))</f>
       </c>
       <c r="D171" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;166,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H171="","",IF($D$3="Mayor",$V171,$U171))</f>
       </c>
     </row>
     <row r="172" ht="90.00" customHeight="1">
       <c r="A172" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H172="","",IFERROR(IMAGE($T172,1),""))</f>
       </c>
       <c r="B172" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H172="","",$I172)</f>
       </c>
       <c r="C172" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H172="","",IF($Y172="","Cód: "&amp;$H172,"Medidas: "&amp;$Y172&amp;"  ·  Cód: "&amp;$H172))</f>
       </c>
       <c r="D172" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;167,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H172="","",IF($D$3="Mayor",$V172,$U172))</f>
       </c>
     </row>
     <row r="173" ht="90.00" customHeight="1">
       <c r="A173" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H173="","",IFERROR(IMAGE($T173,1),""))</f>
       </c>
       <c r="B173" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H173="","",$I173)</f>
       </c>
       <c r="C173" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H173="","",IF($Y173="","Cód: "&amp;$H173,"Medidas: "&amp;$Y173&amp;"  ·  Cód: "&amp;$H173))</f>
       </c>
       <c r="D173" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;168,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H173="","",IF($D$3="Mayor",$V173,$U173))</f>
       </c>
     </row>
     <row r="174" ht="90.00" customHeight="1">
       <c r="A174" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H174="","",IFERROR(IMAGE($T174,1),""))</f>
       </c>
       <c r="B174" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H174="","",$I174)</f>
       </c>
       <c r="C174" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H174="","",IF($Y174="","Cód: "&amp;$H174,"Medidas: "&amp;$Y174&amp;"  ·  Cód: "&amp;$H174))</f>
       </c>
       <c r="D174" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;169,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H174="","",IF($D$3="Mayor",$V174,$U174))</f>
       </c>
     </row>
     <row r="175" ht="90.00" customHeight="1">
       <c r="A175" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H175="","",IFERROR(IMAGE($T175,1),""))</f>
       </c>
       <c r="B175" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H175="","",$I175)</f>
       </c>
       <c r="C175" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H175="","",IF($Y175="","Cód: "&amp;$H175,"Medidas: "&amp;$Y175&amp;"  ·  Cód: "&amp;$H175))</f>
       </c>
       <c r="D175" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;170,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H175="","",IF($D$3="Mayor",$V175,$U175))</f>
       </c>
     </row>
     <row r="176" ht="90.00" customHeight="1">
       <c r="A176" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H176="","",IFERROR(IMAGE($T176,1),""))</f>
       </c>
       <c r="B176" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H176="","",$I176)</f>
       </c>
       <c r="C176" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H176="","",IF($Y176="","Cód: "&amp;$H176,"Medidas: "&amp;$Y176&amp;"  ·  Cód: "&amp;$H176))</f>
       </c>
       <c r="D176" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;171,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H176="","",IF($D$3="Mayor",$V176,$U176))</f>
       </c>
     </row>
     <row r="177" ht="90.00" customHeight="1">
       <c r="A177" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H177="","",IFERROR(IMAGE($T177,1),""))</f>
       </c>
       <c r="B177" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H177="","",$I177)</f>
       </c>
       <c r="C177" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H177="","",IF($Y177="","Cód: "&amp;$H177,"Medidas: "&amp;$Y177&amp;"  ·  Cód: "&amp;$H177))</f>
       </c>
       <c r="D177" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;172,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H177="","",IF($D$3="Mayor",$V177,$U177))</f>
       </c>
     </row>
     <row r="178" ht="90.00" customHeight="1">
       <c r="A178" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H178="","",IFERROR(IMAGE($T178,1),""))</f>
       </c>
       <c r="B178" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H178="","",$I178)</f>
       </c>
       <c r="C178" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H178="","",IF($Y178="","Cód: "&amp;$H178,"Medidas: "&amp;$Y178&amp;"  ·  Cód: "&amp;$H178))</f>
       </c>
       <c r="D178" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;173,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H178="","",IF($D$3="Mayor",$V178,$U178))</f>
       </c>
     </row>
     <row r="179" ht="90.00" customHeight="1">
       <c r="A179" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H179="","",IFERROR(IMAGE($T179,1),""))</f>
       </c>
       <c r="B179" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H179="","",$I179)</f>
       </c>
       <c r="C179" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H179="","",IF($Y179="","Cód: "&amp;$H179,"Medidas: "&amp;$Y179&amp;"  ·  Cód: "&amp;$H179))</f>
       </c>
       <c r="D179" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;174,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H179="","",IF($D$3="Mayor",$V179,$U179))</f>
       </c>
     </row>
     <row r="180" ht="90.00" customHeight="1">
       <c r="A180" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H180="","",IFERROR(IMAGE($T180,1),""))</f>
       </c>
       <c r="B180" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H180="","",$I180)</f>
       </c>
       <c r="C180" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H180="","",IF($Y180="","Cód: "&amp;$H180,"Medidas: "&amp;$Y180&amp;"  ·  Cód: "&amp;$H180))</f>
       </c>
       <c r="D180" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;175,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H180="","",IF($D$3="Mayor",$V180,$U180))</f>
       </c>
     </row>
     <row r="181" ht="90.00" customHeight="1">
       <c r="A181" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H181="","",IFERROR(IMAGE($T181,1),""))</f>
       </c>
       <c r="B181" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H181="","",$I181)</f>
       </c>
       <c r="C181" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H181="","",IF($Y181="","Cód: "&amp;$H181,"Medidas: "&amp;$Y181&amp;"  ·  Cód: "&amp;$H181))</f>
       </c>
       <c r="D181" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;176,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H181="","",IF($D$3="Mayor",$V181,$U181))</f>
       </c>
     </row>
     <row r="182" ht="90.00" customHeight="1">
       <c r="A182" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H182="","",IFERROR(IMAGE($T182,1),""))</f>
       </c>
       <c r="B182" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H182="","",$I182)</f>
       </c>
       <c r="C182" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H182="","",IF($Y182="","Cód: "&amp;$H182,"Medidas: "&amp;$Y182&amp;"  ·  Cód: "&amp;$H182))</f>
       </c>
       <c r="D182" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;177,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H182="","",IF($D$3="Mayor",$V182,$U182))</f>
       </c>
     </row>
     <row r="183" ht="90.00" customHeight="1">
       <c r="A183" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H183="","",IFERROR(IMAGE($T183,1),""))</f>
       </c>
       <c r="B183" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H183="","",$I183)</f>
       </c>
       <c r="C183" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H183="","",IF($Y183="","Cód: "&amp;$H183,"Medidas: "&amp;$Y183&amp;"  ·  Cód: "&amp;$H183))</f>
       </c>
       <c r="D183" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;178,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H183="","",IF($D$3="Mayor",$V183,$U183))</f>
       </c>
     </row>
     <row r="184" ht="90.00" customHeight="1">
       <c r="A184" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H184="","",IFERROR(IMAGE($T184,1),""))</f>
       </c>
       <c r="B184" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H184="","",$I184)</f>
       </c>
       <c r="C184" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H184="","",IF($Y184="","Cód: "&amp;$H184,"Medidas: "&amp;$Y184&amp;"  ·  Cód: "&amp;$H184))</f>
       </c>
       <c r="D184" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;179,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H184="","",IF($D$3="Mayor",$V184,$U184))</f>
       </c>
     </row>
     <row r="185" ht="90.00" customHeight="1">
       <c r="A185" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H185="","",IFERROR(IMAGE($T185,1),""))</f>
       </c>
       <c r="B185" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H185="","",$I185)</f>
       </c>
       <c r="C185" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H185="","",IF($Y185="","Cód: "&amp;$H185,"Medidas: "&amp;$Y185&amp;"  ·  Cód: "&amp;$H185))</f>
       </c>
       <c r="D185" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;180,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H185="","",IF($D$3="Mayor",$V185,$U185))</f>
       </c>
     </row>
     <row r="186" ht="90.00" customHeight="1">
       <c r="A186" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H186="","",IFERROR(IMAGE($T186,1),""))</f>
       </c>
       <c r="B186" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H186="","",$I186)</f>
       </c>
       <c r="C186" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H186="","",IF($Y186="","Cód: "&amp;$H186,"Medidas: "&amp;$Y186&amp;"  ·  Cód: "&amp;$H186))</f>
       </c>
       <c r="D186" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;181,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H186="","",IF($D$3="Mayor",$V186,$U186))</f>
       </c>
     </row>
     <row r="187" ht="90.00" customHeight="1">
       <c r="A187" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H187="","",IFERROR(IMAGE($T187,1),""))</f>
       </c>
       <c r="B187" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H187="","",$I187)</f>
       </c>
       <c r="C187" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H187="","",IF($Y187="","Cód: "&amp;$H187,"Medidas: "&amp;$Y187&amp;"  ·  Cód: "&amp;$H187))</f>
       </c>
       <c r="D187" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;182,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H187="","",IF($D$3="Mayor",$V187,$U187))</f>
       </c>
     </row>
     <row r="188" ht="90.00" customHeight="1">
       <c r="A188" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H188="","",IFERROR(IMAGE($T188,1),""))</f>
       </c>
       <c r="B188" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H188="","",$I188)</f>
       </c>
       <c r="C188" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H188="","",IF($Y188="","Cód: "&amp;$H188,"Medidas: "&amp;$Y188&amp;"  ·  Cód: "&amp;$H188))</f>
       </c>
       <c r="D188" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;183,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H188="","",IF($D$3="Mayor",$V188,$U188))</f>
       </c>
     </row>
     <row r="189" ht="90.00" customHeight="1">
       <c r="A189" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H189="","",IFERROR(IMAGE($T189,1),""))</f>
       </c>
       <c r="B189" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H189="","",$I189)</f>
       </c>
       <c r="C189" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H189="","",IF($Y189="","Cód: "&amp;$H189,"Medidas: "&amp;$Y189&amp;"  ·  Cód: "&amp;$H189))</f>
       </c>
       <c r="D189" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;184,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H189="","",IF($D$3="Mayor",$V189,$U189))</f>
       </c>
     </row>
     <row r="190" ht="90.00" customHeight="1">
       <c r="A190" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H190="","",IFERROR(IMAGE($T190,1),""))</f>
       </c>
       <c r="B190" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H190="","",$I190)</f>
       </c>
       <c r="C190" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H190="","",IF($Y190="","Cód: "&amp;$H190,"Medidas: "&amp;$Y190&amp;"  ·  Cód: "&amp;$H190))</f>
       </c>
       <c r="D190" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;185,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H190="","",IF($D$3="Mayor",$V190,$U190))</f>
       </c>
     </row>
     <row r="191" ht="90.00" customHeight="1">
       <c r="A191" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H191="","",IFERROR(IMAGE($T191,1),""))</f>
       </c>
       <c r="B191" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H191="","",$I191)</f>
       </c>
       <c r="C191" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H191="","",IF($Y191="","Cód: "&amp;$H191,"Medidas: "&amp;$Y191&amp;"  ·  Cód: "&amp;$H191))</f>
       </c>
       <c r="D191" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;186,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H191="","",IF($D$3="Mayor",$V191,$U191))</f>
       </c>
     </row>
     <row r="192" ht="90.00" customHeight="1">
       <c r="A192" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H192="","",IFERROR(IMAGE($T192,1),""))</f>
       </c>
       <c r="B192" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H192="","",$I192)</f>
       </c>
       <c r="C192" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H192="","",IF($Y192="","Cód: "&amp;$H192,"Medidas: "&amp;$Y192&amp;"  ·  Cód: "&amp;$H192))</f>
       </c>
       <c r="D192" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;187,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H192="","",IF($D$3="Mayor",$V192,$U192))</f>
       </c>
     </row>
     <row r="193" ht="90.00" customHeight="1">
       <c r="A193" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H193="","",IFERROR(IMAGE($T193,1),""))</f>
       </c>
       <c r="B193" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H193="","",$I193)</f>
       </c>
       <c r="C193" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H193="","",IF($Y193="","Cód: "&amp;$H193,"Medidas: "&amp;$Y193&amp;"  ·  Cód: "&amp;$H193))</f>
       </c>
       <c r="D193" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;188,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H193="","",IF($D$3="Mayor",$V193,$U193))</f>
       </c>
     </row>
     <row r="194" ht="90.00" customHeight="1">
       <c r="A194" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H194="","",IFERROR(IMAGE($T194,1),""))</f>
       </c>
       <c r="B194" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H194="","",$I194)</f>
       </c>
       <c r="C194" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H194="","",IF($Y194="","Cód: "&amp;$H194,"Medidas: "&amp;$Y194&amp;"  ·  Cód: "&amp;$H194))</f>
       </c>
       <c r="D194" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;189,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H194="","",IF($D$3="Mayor",$V194,$U194))</f>
       </c>
     </row>
     <row r="195" ht="90.00" customHeight="1">
       <c r="A195" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H195="","",IFERROR(IMAGE($T195,1),""))</f>
       </c>
       <c r="B195" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H195="","",$I195)</f>
       </c>
       <c r="C195" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H195="","",IF($Y195="","Cód: "&amp;$H195,"Medidas: "&amp;$Y195&amp;"  ·  Cód: "&amp;$H195))</f>
       </c>
       <c r="D195" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;190,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H195="","",IF($D$3="Mayor",$V195,$U195))</f>
       </c>
     </row>
     <row r="196" ht="90.00" customHeight="1">
       <c r="A196" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H196="","",IFERROR(IMAGE($T196,1),""))</f>
       </c>
       <c r="B196" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H196="","",$I196)</f>
       </c>
       <c r="C196" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H196="","",IF($Y196="","Cód: "&amp;$H196,"Medidas: "&amp;$Y196&amp;"  ·  Cód: "&amp;$H196))</f>
       </c>
       <c r="D196" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;191,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H196="","",IF($D$3="Mayor",$V196,$U196))</f>
       </c>
     </row>
     <row r="197" ht="90.00" customHeight="1">
       <c r="A197" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H197="","",IFERROR(IMAGE($T197,1),""))</f>
       </c>
       <c r="B197" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H197="","",$I197)</f>
       </c>
       <c r="C197" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H197="","",IF($Y197="","Cód: "&amp;$H197,"Medidas: "&amp;$Y197&amp;"  ·  Cód: "&amp;$H197))</f>
       </c>
       <c r="D197" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;192,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H197="","",IF($D$3="Mayor",$V197,$U197))</f>
       </c>
     </row>
     <row r="198" ht="90.00" customHeight="1">
       <c r="A198" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H198="","",IFERROR(IMAGE($T198,1),""))</f>
       </c>
       <c r="B198" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H198="","",$I198)</f>
       </c>
       <c r="C198" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H198="","",IF($Y198="","Cód: "&amp;$H198,"Medidas: "&amp;$Y198&amp;"  ·  Cód: "&amp;$H198))</f>
       </c>
       <c r="D198" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;193,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H198="","",IF($D$3="Mayor",$V198,$U198))</f>
       </c>
     </row>
     <row r="199" ht="90.00" customHeight="1">
       <c r="A199" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H199="","",IFERROR(IMAGE($T199,1),""))</f>
       </c>
       <c r="B199" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H199="","",$I199)</f>
       </c>
       <c r="C199" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H199="","",IF($Y199="","Cód: "&amp;$H199,"Medidas: "&amp;$Y199&amp;"  ·  Cód: "&amp;$H199))</f>
       </c>
       <c r="D199" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;194,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H199="","",IF($D$3="Mayor",$V199,$U199))</f>
       </c>
     </row>
     <row r="200" ht="90.00" customHeight="1">
       <c r="A200" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H200="","",IFERROR(IMAGE($T200,1),""))</f>
       </c>
       <c r="B200" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H200="","",$I200)</f>
       </c>
       <c r="C200" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H200="","",IF($Y200="","Cód: "&amp;$H200,"Medidas: "&amp;$Y200&amp;"  ·  Cód: "&amp;$H200))</f>
       </c>
       <c r="D200" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;195,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H200="","",IF($D$3="Mayor",$V200,$U200))</f>
       </c>
     </row>
     <row r="201" ht="90.00" customHeight="1">
       <c r="A201" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H201="","",IFERROR(IMAGE($T201,1),""))</f>
       </c>
       <c r="B201" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H201="","",$I201)</f>
       </c>
       <c r="C201" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H201="","",IF($Y201="","Cód: "&amp;$H201,"Medidas: "&amp;$Y201&amp;"  ·  Cód: "&amp;$H201))</f>
       </c>
       <c r="D201" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;196,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H201="","",IF($D$3="Mayor",$V201,$U201))</f>
       </c>
     </row>
     <row r="202" ht="90.00" customHeight="1">
       <c r="A202" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H202="","",IFERROR(IMAGE($T202,1),""))</f>
       </c>
       <c r="B202" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H202="","",$I202)</f>
       </c>
       <c r="C202" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H202="","",IF($Y202="","Cód: "&amp;$H202,"Medidas: "&amp;$Y202&amp;"  ·  Cód: "&amp;$H202))</f>
       </c>
       <c r="D202" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;197,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H202="","",IF($D$3="Mayor",$V202,$U202))</f>
       </c>
     </row>
     <row r="203" ht="90.00" customHeight="1">
       <c r="A203" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H203="","",IFERROR(IMAGE($T203,1),""))</f>
       </c>
       <c r="B203" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H203="","",$I203)</f>
       </c>
       <c r="C203" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H203="","",IF($Y203="","Cód: "&amp;$H203,"Medidas: "&amp;$Y203&amp;"  ·  Cód: "&amp;$H203))</f>
       </c>
       <c r="D203" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;198,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H203="","",IF($D$3="Mayor",$V203,$U203))</f>
       </c>
     </row>
     <row r="204" ht="90.00" customHeight="1">
       <c r="A204" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H204="","",IFERROR(IMAGE($T204,1),""))</f>
       </c>
       <c r="B204" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H204="","",$I204)</f>
       </c>
       <c r="C204" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H204="","",IF($Y204="","Cód: "&amp;$H204,"Medidas: "&amp;$Y204&amp;"  ·  Cód: "&amp;$H204))</f>
       </c>
       <c r="D204" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;199,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H204="","",IF($D$3="Mayor",$V204,$U204))</f>
       </c>
     </row>
     <row r="205" ht="90.00" customHeight="1">
       <c r="A205" s="39">
-        <f>IFERROR(IF(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","",IMAGE(INDEX('Catálogo'!$M:$M,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),1)),"")</f>
+        <f>IF($H205="","",IFERROR(IMAGE($T205,1),""))</f>
       </c>
       <c r="B205" s="40">
-        <f>IFERROR(INDEX('Catálogo'!$B:$B,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"")</f>
+        <f>IF($H205="","",$I205)</f>
       </c>
       <c r="C205" s="41">
-        <f>IFERROR(IF(INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))="","Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),"Medidas: "&amp;INDEX('Catálogo'!$R:$R,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))&amp;"  ·  Cód: "&amp;INDEX('Catálogo'!$A:$A,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H205="","",IF($Y205="","Cód: "&amp;$H205,"Medidas: "&amp;$Y205&amp;"  ·  Cód: "&amp;$H205))</f>
       </c>
       <c r="D205" s="42">
-        <f>IFERROR(IF($D$3="Mayor",INDEX('Catálogo'!$O:$O,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0)),INDEX('Catálogo'!$N:$N,MATCH($B$3&amp;"|"&amp;200,IF($B$3="TODAS",'Catálogo'!$U:$U,'Catálogo'!$Q:$Q),0))),"")</f>
+        <f>IF($H205="","",IF($D$3="Mayor",$V205,$U205))</f>
+      </c>
+    </row>
+    <row r="206" ht="90.00" customHeight="1">
+      <c r="A206" s="39">
+        <f>IF($H206="","",IFERROR(IMAGE($T206,1),""))</f>
+      </c>
+      <c r="B206" s="40">
+        <f>IF($H206="","",$I206)</f>
+      </c>
+      <c r="C206" s="41">
+        <f>IF($H206="","",IF($Y206="","Cód: "&amp;$H206,"Medidas: "&amp;$Y206&amp;"  ·  Cód: "&amp;$H206))</f>
+      </c>
+      <c r="D206" s="42">
+        <f>IF($H206="","",IF($D$3="Mayor",$V206,$U206))</f>
+      </c>
+    </row>
+    <row r="207" ht="90.00" customHeight="1">
+      <c r="A207" s="39">
+        <f>IF($H207="","",IFERROR(IMAGE($T207,1),""))</f>
+      </c>
+      <c r="B207" s="40">
+        <f>IF($H207="","",$I207)</f>
+      </c>
+      <c r="C207" s="41">
+        <f>IF($H207="","",IF($Y207="","Cód: "&amp;$H207,"Medidas: "&amp;$Y207&amp;"  ·  Cód: "&amp;$H207))</f>
+      </c>
+      <c r="D207" s="42">
+        <f>IF($H207="","",IF($D$3="Mayor",$V207,$U207))</f>
+      </c>
+    </row>
+    <row r="208" ht="90.00" customHeight="1">
+      <c r="A208" s="39">
+        <f>IF($H208="","",IFERROR(IMAGE($T208,1),""))</f>
+      </c>
+      <c r="B208" s="40">
+        <f>IF($H208="","",$I208)</f>
+      </c>
+      <c r="C208" s="41">
+        <f>IF($H208="","",IF($Y208="","Cód: "&amp;$H208,"Medidas: "&amp;$Y208&amp;"  ·  Cód: "&amp;$H208))</f>
+      </c>
+      <c r="D208" s="42">
+        <f>IF($H208="","",IF($D$3="Mayor",$V208,$U208))</f>
+      </c>
+    </row>
+    <row r="209" ht="90.00" customHeight="1">
+      <c r="A209" s="39">
+        <f>IF($H209="","",IFERROR(IMAGE($T209,1),""))</f>
+      </c>
+      <c r="B209" s="40">
+        <f>IF($H209="","",$I209)</f>
+      </c>
+      <c r="C209" s="41">
+        <f>IF($H209="","",IF($Y209="","Cód: "&amp;$H209,"Medidas: "&amp;$Y209&amp;"  ·  Cód: "&amp;$H209))</f>
+      </c>
+      <c r="D209" s="42">
+        <f>IF($H209="","",IF($D$3="Mayor",$V209,$U209))</f>
+      </c>
+    </row>
+    <row r="210" ht="90.00" customHeight="1">
+      <c r="A210" s="39">
+        <f>IF($H210="","",IFERROR(IMAGE($T210,1),""))</f>
+      </c>
+      <c r="B210" s="40">
+        <f>IF($H210="","",$I210)</f>
+      </c>
+      <c r="C210" s="41">
+        <f>IF($H210="","",IF($Y210="","Cód: "&amp;$H210,"Medidas: "&amp;$Y210&amp;"  ·  Cód: "&amp;$H210))</f>
+      </c>
+      <c r="D210" s="42">
+        <f>IF($H210="","",IF($D$3="Mayor",$V210,$U210))</f>
+      </c>
+    </row>
+    <row r="211" ht="90.00" customHeight="1">
+      <c r="A211" s="39">
+        <f>IF($H211="","",IFERROR(IMAGE($T211,1),""))</f>
+      </c>
+      <c r="B211" s="40">
+        <f>IF($H211="","",$I211)</f>
+      </c>
+      <c r="C211" s="41">
+        <f>IF($H211="","",IF($Y211="","Cód: "&amp;$H211,"Medidas: "&amp;$Y211&amp;"  ·  Cód: "&amp;$H211))</f>
+      </c>
+      <c r="D211" s="42">
+        <f>IF($H211="","",IF($D$3="Mayor",$V211,$U211))</f>
+      </c>
+    </row>
+    <row r="212" ht="90.00" customHeight="1">
+      <c r="A212" s="39">
+        <f>IF($H212="","",IFERROR(IMAGE($T212,1),""))</f>
+      </c>
+      <c r="B212" s="40">
+        <f>IF($H212="","",$I212)</f>
+      </c>
+      <c r="C212" s="41">
+        <f>IF($H212="","",IF($Y212="","Cód: "&amp;$H212,"Medidas: "&amp;$Y212&amp;"  ·  Cód: "&amp;$H212))</f>
+      </c>
+      <c r="D212" s="42">
+        <f>IF($H212="","",IF($D$3="Mayor",$V212,$U212))</f>
+      </c>
+    </row>
+    <row r="213" ht="90.00" customHeight="1">
+      <c r="A213" s="39">
+        <f>IF($H213="","",IFERROR(IMAGE($T213,1),""))</f>
+      </c>
+      <c r="B213" s="40">
+        <f>IF($H213="","",$I213)</f>
+      </c>
+      <c r="C213" s="41">
+        <f>IF($H213="","",IF($Y213="","Cód: "&amp;$H213,"Medidas: "&amp;$Y213&amp;"  ·  Cód: "&amp;$H213))</f>
+      </c>
+      <c r="D213" s="42">
+        <f>IF($H213="","",IF($D$3="Mayor",$V213,$U213))</f>
+      </c>
+    </row>
+    <row r="214" ht="90.00" customHeight="1">
+      <c r="A214" s="39">
+        <f>IF($H214="","",IFERROR(IMAGE($T214,1),""))</f>
+      </c>
+      <c r="B214" s="40">
+        <f>IF($H214="","",$I214)</f>
+      </c>
+      <c r="C214" s="41">
+        <f>IF($H214="","",IF($Y214="","Cód: "&amp;$H214,"Medidas: "&amp;$Y214&amp;"  ·  Cód: "&amp;$H214))</f>
+      </c>
+      <c r="D214" s="42">
+        <f>IF($H214="","",IF($D$3="Mayor",$V214,$U214))</f>
+      </c>
+    </row>
+    <row r="215" ht="90.00" customHeight="1">
+      <c r="A215" s="39">
+        <f>IF($H215="","",IFERROR(IMAGE($T215,1),""))</f>
+      </c>
+      <c r="B215" s="40">
+        <f>IF($H215="","",$I215)</f>
+      </c>
+      <c r="C215" s="41">
+        <f>IF($H215="","",IF($Y215="","Cód: "&amp;$H215,"Medidas: "&amp;$Y215&amp;"  ·  Cód: "&amp;$H215))</f>
+      </c>
+      <c r="D215" s="42">
+        <f>IF($H215="","",IF($D$3="Mayor",$V215,$U215))</f>
+      </c>
+    </row>
+    <row r="216" ht="90.00" customHeight="1">
+      <c r="A216" s="39">
+        <f>IF($H216="","",IFERROR(IMAGE($T216,1),""))</f>
+      </c>
+      <c r="B216" s="40">
+        <f>IF($H216="","",$I216)</f>
+      </c>
+      <c r="C216" s="41">
+        <f>IF($H216="","",IF($Y216="","Cód: "&amp;$H216,"Medidas: "&amp;$Y216&amp;"  ·  Cód: "&amp;$H216))</f>
+      </c>
+      <c r="D216" s="42">
+        <f>IF($H216="","",IF($D$3="Mayor",$V216,$U216))</f>
+      </c>
+    </row>
+    <row r="217" ht="90.00" customHeight="1">
+      <c r="A217" s="39">
+        <f>IF($H217="","",IFERROR(IMAGE($T217,1),""))</f>
+      </c>
+      <c r="B217" s="40">
+        <f>IF($H217="","",$I217)</f>
+      </c>
+      <c r="C217" s="41">
+        <f>IF($H217="","",IF($Y217="","Cód: "&amp;$H217,"Medidas: "&amp;$Y217&amp;"  ·  Cód: "&amp;$H217))</f>
+      </c>
+      <c r="D217" s="42">
+        <f>IF($H217="","",IF($D$3="Mayor",$V217,$U217))</f>
+      </c>
+    </row>
+    <row r="218" ht="90.00" customHeight="1">
+      <c r="A218" s="39">
+        <f>IF($H218="","",IFERROR(IMAGE($T218,1),""))</f>
+      </c>
+      <c r="B218" s="40">
+        <f>IF($H218="","",$I218)</f>
+      </c>
+      <c r="C218" s="41">
+        <f>IF($H218="","",IF($Y218="","Cód: "&amp;$H218,"Medidas: "&amp;$Y218&amp;"  ·  Cód: "&amp;$H218))</f>
+      </c>
+      <c r="D218" s="42">
+        <f>IF($H218="","",IF($D$3="Mayor",$V218,$U218))</f>
+      </c>
+    </row>
+    <row r="219" ht="90.00" customHeight="1">
+      <c r="A219" s="39">
+        <f>IF($H219="","",IFERROR(IMAGE($T219,1),""))</f>
+      </c>
+      <c r="B219" s="40">
+        <f>IF($H219="","",$I219)</f>
+      </c>
+      <c r="C219" s="41">
+        <f>IF($H219="","",IF($Y219="","Cód: "&amp;$H219,"Medidas: "&amp;$Y219&amp;"  ·  Cód: "&amp;$H219))</f>
+      </c>
+      <c r="D219" s="42">
+        <f>IF($H219="","",IF($D$3="Mayor",$V219,$U219))</f>
+      </c>
+    </row>
+    <row r="220" ht="90.00" customHeight="1">
+      <c r="A220" s="39">
+        <f>IF($H220="","",IFERROR(IMAGE($T220,1),""))</f>
+      </c>
+      <c r="B220" s="40">
+        <f>IF($H220="","",$I220)</f>
+      </c>
+      <c r="C220" s="41">
+        <f>IF($H220="","",IF($Y220="","Cód: "&amp;$H220,"Medidas: "&amp;$Y220&amp;"  ·  Cód: "&amp;$H220))</f>
+      </c>
+      <c r="D220" s="42">
+        <f>IF($H220="","",IF($D$3="Mayor",$V220,$U220))</f>
+      </c>
+    </row>
+    <row r="221" ht="90.00" customHeight="1">
+      <c r="A221" s="39">
+        <f>IF($H221="","",IFERROR(IMAGE($T221,1),""))</f>
+      </c>
+      <c r="B221" s="40">
+        <f>IF($H221="","",$I221)</f>
+      </c>
+      <c r="C221" s="41">
+        <f>IF($H221="","",IF($Y221="","Cód: "&amp;$H221,"Medidas: "&amp;$Y221&amp;"  ·  Cód: "&amp;$H221))</f>
+      </c>
+      <c r="D221" s="42">
+        <f>IF($H221="","",IF($D$3="Mayor",$V221,$U221))</f>
+      </c>
+    </row>
+    <row r="222" ht="90.00" customHeight="1">
+      <c r="A222" s="39">
+        <f>IF($H222="","",IFERROR(IMAGE($T222,1),""))</f>
+      </c>
+      <c r="B222" s="40">
+        <f>IF($H222="","",$I222)</f>
+      </c>
+      <c r="C222" s="41">
+        <f>IF($H222="","",IF($Y222="","Cód: "&amp;$H222,"Medidas: "&amp;$Y222&amp;"  ·  Cód: "&amp;$H222))</f>
+      </c>
+      <c r="D222" s="42">
+        <f>IF($H222="","",IF($D$3="Mayor",$V222,$U222))</f>
+      </c>
+    </row>
+    <row r="223" ht="90.00" customHeight="1">
+      <c r="A223" s="39">
+        <f>IF($H223="","",IFERROR(IMAGE($T223,1),""))</f>
+      </c>
+      <c r="B223" s="40">
+        <f>IF($H223="","",$I223)</f>
+      </c>
+      <c r="C223" s="41">
+        <f>IF($H223="","",IF($Y223="","Cód: "&amp;$H223,"Medidas: "&amp;$Y223&amp;"  ·  Cód: "&amp;$H223))</f>
+      </c>
+      <c r="D223" s="42">
+        <f>IF($H223="","",IF($D$3="Mayor",$V223,$U223))</f>
+      </c>
+    </row>
+    <row r="224" ht="90.00" customHeight="1">
+      <c r="A224" s="39">
+        <f>IF($H224="","",IFERROR(IMAGE($T224,1),""))</f>
+      </c>
+      <c r="B224" s="40">
+        <f>IF($H224="","",$I224)</f>
+      </c>
+      <c r="C224" s="41">
+        <f>IF($H224="","",IF($Y224="","Cód: "&amp;$H224,"Medidas: "&amp;$Y224&amp;"  ·  Cód: "&amp;$H224))</f>
+      </c>
+      <c r="D224" s="42">
+        <f>IF($H224="","",IF($D$3="Mayor",$V224,$U224))</f>
+      </c>
+    </row>
+    <row r="225" ht="90.00" customHeight="1">
+      <c r="A225" s="39">
+        <f>IF($H225="","",IFERROR(IMAGE($T225,1),""))</f>
+      </c>
+      <c r="B225" s="40">
+        <f>IF($H225="","",$I225)</f>
+      </c>
+      <c r="C225" s="41">
+        <f>IF($H225="","",IF($Y225="","Cód: "&amp;$H225,"Medidas: "&amp;$Y225&amp;"  ·  Cód: "&amp;$H225))</f>
+      </c>
+      <c r="D225" s="42">
+        <f>IF($H225="","",IF($D$3="Mayor",$V225,$U225))</f>
+      </c>
+    </row>
+    <row r="226" ht="90.00" customHeight="1">
+      <c r="A226" s="39">
+        <f>IF($H226="","",IFERROR(IMAGE($T226,1),""))</f>
+      </c>
+      <c r="B226" s="40">
+        <f>IF($H226="","",$I226)</f>
+      </c>
+      <c r="C226" s="41">
+        <f>IF($H226="","",IF($Y226="","Cód: "&amp;$H226,"Medidas: "&amp;$Y226&amp;"  ·  Cód: "&amp;$H226))</f>
+      </c>
+      <c r="D226" s="42">
+        <f>IF($H226="","",IF($D$3="Mayor",$V226,$U226))</f>
+      </c>
+    </row>
+    <row r="227" ht="90.00" customHeight="1">
+      <c r="A227" s="39">
+        <f>IF($H227="","",IFERROR(IMAGE($T227,1),""))</f>
+      </c>
+      <c r="B227" s="40">
+        <f>IF($H227="","",$I227)</f>
+      </c>
+      <c r="C227" s="41">
+        <f>IF($H227="","",IF($Y227="","Cód: "&amp;$H227,"Medidas: "&amp;$Y227&amp;"  ·  Cód: "&amp;$H227))</f>
+      </c>
+      <c r="D227" s="42">
+        <f>IF($H227="","",IF($D$3="Mayor",$V227,$U227))</f>
+      </c>
+    </row>
+    <row r="228" ht="90.00" customHeight="1">
+      <c r="A228" s="39">
+        <f>IF($H228="","",IFERROR(IMAGE($T228,1),""))</f>
+      </c>
+      <c r="B228" s="40">
+        <f>IF($H228="","",$I228)</f>
+      </c>
+      <c r="C228" s="41">
+        <f>IF($H228="","",IF($Y228="","Cód: "&amp;$H228,"Medidas: "&amp;$Y228&amp;"  ·  Cód: "&amp;$H228))</f>
+      </c>
+      <c r="D228" s="42">
+        <f>IF($H228="","",IF($D$3="Mayor",$V228,$U228))</f>
+      </c>
+    </row>
+    <row r="229" ht="90.00" customHeight="1">
+      <c r="A229" s="39">
+        <f>IF($H229="","",IFERROR(IMAGE($T229,1),""))</f>
+      </c>
+      <c r="B229" s="40">
+        <f>IF($H229="","",$I229)</f>
+      </c>
+      <c r="C229" s="41">
+        <f>IF($H229="","",IF($Y229="","Cód: "&amp;$H229,"Medidas: "&amp;$Y229&amp;"  ·  Cód: "&amp;$H229))</f>
+      </c>
+      <c r="D229" s="42">
+        <f>IF($H229="","",IF($D$3="Mayor",$V229,$U229))</f>
+      </c>
+    </row>
+    <row r="230" ht="90.00" customHeight="1">
+      <c r="A230" s="39">
+        <f>IF($H230="","",IFERROR(IMAGE($T230,1),""))</f>
+      </c>
+      <c r="B230" s="40">
+        <f>IF($H230="","",$I230)</f>
+      </c>
+      <c r="C230" s="41">
+        <f>IF($H230="","",IF($Y230="","Cód: "&amp;$H230,"Medidas: "&amp;$Y230&amp;"  ·  Cód: "&amp;$H230))</f>
+      </c>
+      <c r="D230" s="42">
+        <f>IF($H230="","",IF($D$3="Mayor",$V230,$U230))</f>
+      </c>
+    </row>
+    <row r="231" ht="90.00" customHeight="1">
+      <c r="A231" s="39">
+        <f>IF($H231="","",IFERROR(IMAGE($T231,1),""))</f>
+      </c>
+      <c r="B231" s="40">
+        <f>IF($H231="","",$I231)</f>
+      </c>
+      <c r="C231" s="41">
+        <f>IF($H231="","",IF($Y231="","Cód: "&amp;$H231,"Medidas: "&amp;$Y231&amp;"  ·  Cód: "&amp;$H231))</f>
+      </c>
+      <c r="D231" s="42">
+        <f>IF($H231="","",IF($D$3="Mayor",$V231,$U231))</f>
+      </c>
+    </row>
+    <row r="232" ht="90.00" customHeight="1">
+      <c r="A232" s="39">
+        <f>IF($H232="","",IFERROR(IMAGE($T232,1),""))</f>
+      </c>
+      <c r="B232" s="40">
+        <f>IF($H232="","",$I232)</f>
+      </c>
+      <c r="C232" s="41">
+        <f>IF($H232="","",IF($Y232="","Cód: "&amp;$H232,"Medidas: "&amp;$Y232&amp;"  ·  Cód: "&amp;$H232))</f>
+      </c>
+      <c r="D232" s="42">
+        <f>IF($H232="","",IF($D$3="Mayor",$V232,$U232))</f>
+      </c>
+    </row>
+    <row r="233" ht="90.00" customHeight="1">
+      <c r="A233" s="39">
+        <f>IF($H233="","",IFERROR(IMAGE($T233,1),""))</f>
+      </c>
+      <c r="B233" s="40">
+        <f>IF($H233="","",$I233)</f>
+      </c>
+      <c r="C233" s="41">
+        <f>IF($H233="","",IF($Y233="","Cód: "&amp;$H233,"Medidas: "&amp;$Y233&amp;"  ·  Cód: "&amp;$H233))</f>
+      </c>
+      <c r="D233" s="42">
+        <f>IF($H233="","",IF($D$3="Mayor",$V233,$U233))</f>
+      </c>
+    </row>
+    <row r="234" ht="90.00" customHeight="1">
+      <c r="A234" s="39">
+        <f>IF($H234="","",IFERROR(IMAGE($T234,1),""))</f>
+      </c>
+      <c r="B234" s="40">
+        <f>IF($H234="","",$I234)</f>
+      </c>
+      <c r="C234" s="41">
+        <f>IF($H234="","",IF($Y234="","Cód: "&amp;$H234,"Medidas: "&amp;$Y234&amp;"  ·  Cód: "&amp;$H234))</f>
+      </c>
+      <c r="D234" s="42">
+        <f>IF($H234="","",IF($D$3="Mayor",$V234,$U234))</f>
+      </c>
+    </row>
+    <row r="235" ht="90.00" customHeight="1">
+      <c r="A235" s="39">
+        <f>IF($H235="","",IFERROR(IMAGE($T235,1),""))</f>
+      </c>
+      <c r="B235" s="40">
+        <f>IF($H235="","",$I235)</f>
+      </c>
+      <c r="C235" s="41">
+        <f>IF($H235="","",IF($Y235="","Cód: "&amp;$H235,"Medidas: "&amp;$Y235&amp;"  ·  Cód: "&amp;$H235))</f>
+      </c>
+      <c r="D235" s="42">
+        <f>IF($H235="","",IF($D$3="Mayor",$V235,$U235))</f>
+      </c>
+    </row>
+    <row r="236" ht="90.00" customHeight="1">
+      <c r="A236" s="39">
+        <f>IF($H236="","",IFERROR(IMAGE($T236,1),""))</f>
+      </c>
+      <c r="B236" s="40">
+        <f>IF($H236="","",$I236)</f>
+      </c>
+      <c r="C236" s="41">
+        <f>IF($H236="","",IF($Y236="","Cód: "&amp;$H236,"Medidas: "&amp;$Y236&amp;"  ·  Cód: "&amp;$H236))</f>
+      </c>
+      <c r="D236" s="42">
+        <f>IF($H236="","",IF($D$3="Mayor",$V236,$U236))</f>
+      </c>
+    </row>
+    <row r="237" ht="90.00" customHeight="1">
+      <c r="A237" s="39">
+        <f>IF($H237="","",IFERROR(IMAGE($T237,1),""))</f>
+      </c>
+      <c r="B237" s="40">
+        <f>IF($H237="","",$I237)</f>
+      </c>
+      <c r="C237" s="41">
+        <f>IF($H237="","",IF($Y237="","Cód: "&amp;$H237,"Medidas: "&amp;$Y237&amp;"  ·  Cód: "&amp;$H237))</f>
+      </c>
+      <c r="D237" s="42">
+        <f>IF($H237="","",IF($D$3="Mayor",$V237,$U237))</f>
+      </c>
+    </row>
+    <row r="238" ht="90.00" customHeight="1">
+      <c r="A238" s="39">
+        <f>IF($H238="","",IFERROR(IMAGE($T238,1),""))</f>
+      </c>
+      <c r="B238" s="40">
+        <f>IF($H238="","",$I238)</f>
+      </c>
+      <c r="C238" s="41">
+        <f>IF($H238="","",IF($Y238="","Cód: "&amp;$H238,"Medidas: "&amp;$Y238&amp;"  ·  Cód: "&amp;$H238))</f>
+      </c>
+      <c r="D238" s="42">
+        <f>IF($H238="","",IF($D$3="Mayor",$V238,$U238))</f>
+      </c>
+    </row>
+    <row r="239" ht="90.00" customHeight="1">
+      <c r="A239" s="39">
+        <f>IF($H239="","",IFERROR(IMAGE($T239,1),""))</f>
+      </c>
+      <c r="B239" s="40">
+        <f>IF($H239="","",$I239)</f>
+      </c>
+      <c r="C239" s="41">
+        <f>IF($H239="","",IF($Y239="","Cód: "&amp;$H239,"Medidas: "&amp;$Y239&amp;"  ·  Cód: "&amp;$H239))</f>
+      </c>
+      <c r="D239" s="42">
+        <f>IF($H239="","",IF($D$3="Mayor",$V239,$U239))</f>
+      </c>
+    </row>
+    <row r="240" ht="90.00" customHeight="1">
+      <c r="A240" s="39">
+        <f>IF($H240="","",IFERROR(IMAGE($T240,1),""))</f>
+      </c>
+      <c r="B240" s="40">
+        <f>IF($H240="","",$I240)</f>
+      </c>
+      <c r="C240" s="41">
+        <f>IF($H240="","",IF($Y240="","Cód: "&amp;$H240,"Medidas: "&amp;$Y240&amp;"  ·  Cód: "&amp;$H240))</f>
+      </c>
+      <c r="D240" s="42">
+        <f>IF($H240="","",IF($D$3="Mayor",$V240,$U240))</f>
+      </c>
+    </row>
+    <row r="241" ht="90.00" customHeight="1">
+      <c r="A241" s="39">
+        <f>IF($H241="","",IFERROR(IMAGE($T241,1),""))</f>
+      </c>
+      <c r="B241" s="40">
+        <f>IF($H241="","",$I241)</f>
+      </c>
+      <c r="C241" s="41">
+        <f>IF($H241="","",IF($Y241="","Cód: "&amp;$H241,"Medidas: "&amp;$Y241&amp;"  ·  Cód: "&amp;$H241))</f>
+      </c>
+      <c r="D241" s="42">
+        <f>IF($H241="","",IF($D$3="Mayor",$V241,$U241))</f>
+      </c>
+    </row>
+    <row r="242" ht="90.00" customHeight="1">
+      <c r="A242" s="39">
+        <f>IF($H242="","",IFERROR(IMAGE($T242,1),""))</f>
+      </c>
+      <c r="B242" s="40">
+        <f>IF($H242="","",$I242)</f>
+      </c>
+      <c r="C242" s="41">
+        <f>IF($H242="","",IF($Y242="","Cód: "&amp;$H242,"Medidas: "&amp;$Y242&amp;"  ·  Cód: "&amp;$H242))</f>
+      </c>
+      <c r="D242" s="42">
+        <f>IF($H242="","",IF($D$3="Mayor",$V242,$U242))</f>
+      </c>
+    </row>
+    <row r="243" ht="90.00" customHeight="1">
+      <c r="A243" s="39">
+        <f>IF($H243="","",IFERROR(IMAGE($T243,1),""))</f>
+      </c>
+      <c r="B243" s="40">
+        <f>IF($H243="","",$I243)</f>
+      </c>
+      <c r="C243" s="41">
+        <f>IF($H243="","",IF($Y243="","Cód: "&amp;$H243,"Medidas: "&amp;$Y243&amp;"  ·  Cód: "&amp;$H243))</f>
+      </c>
+      <c r="D243" s="42">
+        <f>IF($H243="","",IF($D$3="Mayor",$V243,$U243))</f>
+      </c>
+    </row>
+    <row r="244" ht="90.00" customHeight="1">
+      <c r="A244" s="39">
+        <f>IF($H244="","",IFERROR(IMAGE($T244,1),""))</f>
+      </c>
+      <c r="B244" s="40">
+        <f>IF($H244="","",$I244)</f>
+      </c>
+      <c r="C244" s="41">
+        <f>IF($H244="","",IF($Y244="","Cód: "&amp;$H244,"Medidas: "&amp;$Y244&amp;"  ·  Cód: "&amp;$H244))</f>
+      </c>
+      <c r="D244" s="42">
+        <f>IF($H244="","",IF($D$3="Mayor",$V244,$U244))</f>
+      </c>
+    </row>
+    <row r="245" ht="90.00" customHeight="1">
+      <c r="A245" s="39">
+        <f>IF($H245="","",IFERROR(IMAGE($T245,1),""))</f>
+      </c>
+      <c r="B245" s="40">
+        <f>IF($H245="","",$I245)</f>
+      </c>
+      <c r="C245" s="41">
+        <f>IF($H245="","",IF($Y245="","Cód: "&amp;$H245,"Medidas: "&amp;$Y245&amp;"  ·  Cód: "&amp;$H245))</f>
+      </c>
+      <c r="D245" s="42">
+        <f>IF($H245="","",IF($D$3="Mayor",$V245,$U245))</f>
+      </c>
+    </row>
+    <row r="246" ht="90.00" customHeight="1">
+      <c r="A246" s="39">
+        <f>IF($H246="","",IFERROR(IMAGE($T246,1),""))</f>
+      </c>
+      <c r="B246" s="40">
+        <f>IF($H246="","",$I246)</f>
+      </c>
+      <c r="C246" s="41">
+        <f>IF($H246="","",IF($Y246="","Cód: "&amp;$H246,"Medidas: "&amp;$Y246&amp;"  ·  Cód: "&amp;$H246))</f>
+      </c>
+      <c r="D246" s="42">
+        <f>IF($H246="","",IF($D$3="Mayor",$V246,$U246))</f>
+      </c>
+    </row>
+    <row r="247" ht="90.00" customHeight="1">
+      <c r="A247" s="39">
+        <f>IF($H247="","",IFERROR(IMAGE($T247,1),""))</f>
+      </c>
+      <c r="B247" s="40">
+        <f>IF($H247="","",$I247)</f>
+      </c>
+      <c r="C247" s="41">
+        <f>IF($H247="","",IF($Y247="","Cód: "&amp;$H247,"Medidas: "&amp;$Y247&amp;"  ·  Cód: "&amp;$H247))</f>
+      </c>
+      <c r="D247" s="42">
+        <f>IF($H247="","",IF($D$3="Mayor",$V247,$U247))</f>
+      </c>
+    </row>
+    <row r="248" ht="90.00" customHeight="1">
+      <c r="A248" s="39">
+        <f>IF($H248="","",IFERROR(IMAGE($T248,1),""))</f>
+      </c>
+      <c r="B248" s="40">
+        <f>IF($H248="","",$I248)</f>
+      </c>
+      <c r="C248" s="41">
+        <f>IF($H248="","",IF($Y248="","Cód: "&amp;$H248,"Medidas: "&amp;$Y248&amp;"  ·  Cód: "&amp;$H248))</f>
+      </c>
+      <c r="D248" s="42">
+        <f>IF($H248="","",IF($D$3="Mayor",$V248,$U248))</f>
+      </c>
+    </row>
+    <row r="249" ht="90.00" customHeight="1">
+      <c r="A249" s="39">
+        <f>IF($H249="","",IFERROR(IMAGE($T249,1),""))</f>
+      </c>
+      <c r="B249" s="40">
+        <f>IF($H249="","",$I249)</f>
+      </c>
+      <c r="C249" s="41">
+        <f>IF($H249="","",IF($Y249="","Cód: "&amp;$H249,"Medidas: "&amp;$Y249&amp;"  ·  Cód: "&amp;$H249))</f>
+      </c>
+      <c r="D249" s="42">
+        <f>IF($H249="","",IF($D$3="Mayor",$V249,$U249))</f>
+      </c>
+    </row>
+    <row r="250" ht="90.00" customHeight="1">
+      <c r="A250" s="39">
+        <f>IF($H250="","",IFERROR(IMAGE($T250,1),""))</f>
+      </c>
+      <c r="B250" s="40">
+        <f>IF($H250="","",$I250)</f>
+      </c>
+      <c r="C250" s="41">
+        <f>IF($H250="","",IF($Y250="","Cód: "&amp;$H250,"Medidas: "&amp;$Y250&amp;"  ·  Cód: "&amp;$H250))</f>
+      </c>
+      <c r="D250" s="42">
+        <f>IF($H250="","",IF($D$3="Mayor",$V250,$U250))</f>
+      </c>
+    </row>
+    <row r="251" ht="90.00" customHeight="1">
+      <c r="A251" s="39">
+        <f>IF($H251="","",IFERROR(IMAGE($T251,1),""))</f>
+      </c>
+      <c r="B251" s="40">
+        <f>IF($H251="","",$I251)</f>
+      </c>
+      <c r="C251" s="41">
+        <f>IF($H251="","",IF($Y251="","Cód: "&amp;$H251,"Medidas: "&amp;$Y251&amp;"  ·  Cód: "&amp;$H251))</f>
+      </c>
+      <c r="D251" s="42">
+        <f>IF($H251="","",IF($D$3="Mayor",$V251,$U251))</f>
+      </c>
+    </row>
+    <row r="252" ht="90.00" customHeight="1">
+      <c r="A252" s="39">
+        <f>IF($H252="","",IFERROR(IMAGE($T252,1),""))</f>
+      </c>
+      <c r="B252" s="40">
+        <f>IF($H252="","",$I252)</f>
+      </c>
+      <c r="C252" s="41">
+        <f>IF($H252="","",IF($Y252="","Cód: "&amp;$H252,"Medidas: "&amp;$Y252&amp;"  ·  Cód: "&amp;$H252))</f>
+      </c>
+      <c r="D252" s="42">
+        <f>IF($H252="","",IF($D$3="Mayor",$V252,$U252))</f>
+      </c>
+    </row>
+    <row r="253" ht="90.00" customHeight="1">
+      <c r="A253" s="39">
+        <f>IF($H253="","",IFERROR(IMAGE($T253,1),""))</f>
+      </c>
+      <c r="B253" s="40">
+        <f>IF($H253="","",$I253)</f>
+      </c>
+      <c r="C253" s="41">
+        <f>IF($H253="","",IF($Y253="","Cód: "&amp;$H253,"Medidas: "&amp;$Y253&amp;"  ·  Cód: "&amp;$H253))</f>
+      </c>
+      <c r="D253" s="42">
+        <f>IF($H253="","",IF($D$3="Mayor",$V253,$U253))</f>
+      </c>
+    </row>
+    <row r="254" ht="90.00" customHeight="1">
+      <c r="A254" s="39">
+        <f>IF($H254="","",IFERROR(IMAGE($T254,1),""))</f>
+      </c>
+      <c r="B254" s="40">
+        <f>IF($H254="","",$I254)</f>
+      </c>
+      <c r="C254" s="41">
+        <f>IF($H254="","",IF($Y254="","Cód: "&amp;$H254,"Medidas: "&amp;$Y254&amp;"  ·  Cód: "&amp;$H254))</f>
+      </c>
+      <c r="D254" s="42">
+        <f>IF($H254="","",IF($D$3="Mayor",$V254,$U254))</f>
+      </c>
+    </row>
+    <row r="255" ht="90.00" customHeight="1">
+      <c r="A255" s="39">
+        <f>IF($H255="","",IFERROR(IMAGE($T255,1),""))</f>
+      </c>
+      <c r="B255" s="40">
+        <f>IF($H255="","",$I255)</f>
+      </c>
+      <c r="C255" s="41">
+        <f>IF($H255="","",IF($Y255="","Cód: "&amp;$H255,"Medidas: "&amp;$Y255&amp;"  ·  Cód: "&amp;$H255))</f>
+      </c>
+      <c r="D255" s="42">
+        <f>IF($H255="","",IF($D$3="Mayor",$V255,$U255))</f>
       </c>
     </row>
   </sheetData>

</xml_diff>